<commit_message>
Update MLB weather 2026-07-14 12:13 AM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_2026_07_14.xlsx
+++ b/mlb_weather_professional_2026_07_14.xlsx
@@ -518,7 +518,7 @@
     <t>A</t>
   </si>
   <si>
-    <t>2026-07-14 12:08:30 AM PDT</t>
+    <t>2026-07-14 12:13:19 AM PDT</t>
   </si>
   <si>
     <t>LOW</t>
@@ -539,7 +539,7 @@
     <t>Mostly clear</t>
   </si>
   <si>
-    <t>2026-07-14 07:08:30 UTC</t>
+    <t>2026-07-14 07:13:19 UTC</t>
   </si>
   <si>
     <t>2026-07-14T00:18:35+00:00</t>
@@ -1840,7 +1840,7 @@
         <v>165</v>
       </c>
       <c r="W2">
-        <v>409.9</v>
+        <v>414.7</v>
       </c>
       <c r="X2">
         <v>5</v>
@@ -1867,7 +1867,7 @@
         <v>166</v>
       </c>
       <c r="AF2">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="AG2" t="s">
         <v>167</v>
@@ -2546,10 +2546,10 @@
         <v>173</v>
       </c>
       <c r="J2">
-        <v>409.9</v>
+        <v>414.7</v>
       </c>
       <c r="K2">
-        <v>16.9</v>
+        <v>16.8</v>
       </c>
       <c r="L2">
         <v>5</v>
@@ -2687,7 +2687,7 @@
         <v>166</v>
       </c>
       <c r="BE2">
-        <v>3.8</v>
+        <v>3.7</v>
       </c>
       <c r="BF2" t="s">
         <v>166</v>
@@ -2734,10 +2734,10 @@
         <v>173</v>
       </c>
       <c r="J3">
-        <v>409.9</v>
+        <v>414.7</v>
       </c>
       <c r="K3">
-        <v>17.9</v>
+        <v>17.8</v>
       </c>
       <c r="L3">
         <v>5</v>
@@ -2922,10 +2922,10 @@
         <v>173</v>
       </c>
       <c r="J4">
-        <v>409.9</v>
+        <v>414.7</v>
       </c>
       <c r="K4">
-        <v>18.9</v>
+        <v>18.8</v>
       </c>
       <c r="L4">
         <v>5</v>
@@ -3110,10 +3110,10 @@
         <v>173</v>
       </c>
       <c r="J5">
-        <v>409.9</v>
+        <v>414.7</v>
       </c>
       <c r="K5">
-        <v>19.9</v>
+        <v>19.8</v>
       </c>
       <c r="L5">
         <v>5</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 12:26 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_2026_07_14.xlsx
+++ b/mlb_weather_professional_2026_07_14.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="232">
   <si>
     <t>Date</t>
   </si>
@@ -509,7 +509,7 @@
     <t>🔥 Excellent</t>
   </si>
   <si>
-    <t>adjusted carry 87.0; +20 ft carry; +8.9% HR env.</t>
+    <t>adjusted carry 85.5; +20 ft carry; +8.5% HR env.</t>
   </si>
   <si>
     <t>100th</t>
@@ -518,7 +518,7 @@
     <t>A</t>
   </si>
   <si>
-    <t>2026-07-14 12:13:19 AM PDT</t>
+    <t>2026-07-14 12:26:55 PM PDT</t>
   </si>
   <si>
     <t>LOW</t>
@@ -536,13 +536,13 @@
     <t>OPEN_AIR</t>
   </si>
   <si>
-    <t>Mostly clear</t>
-  </si>
-  <si>
-    <t>2026-07-14 07:13:19 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14T00:18:35+00:00</t>
+    <t>Clear</t>
+  </si>
+  <si>
+    <t>2026-07-14 19:26:55 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14T18:41:01+00:00</t>
   </si>
   <si>
     <t>SW</t>
@@ -711,9 +711,6 @@
   </si>
   <si>
     <t>11:00 PM EDT</t>
-  </si>
-  <si>
-    <t>Clear</t>
   </si>
   <si>
     <t>LIGHT</t>
@@ -1804,10 +1801,10 @@
         <v>162</v>
       </c>
       <c r="K2">
-        <v>88.5</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="L2">
-        <v>87</v>
+        <v>85.5</v>
       </c>
       <c r="M2" t="s">
         <v>163</v>
@@ -1819,19 +1816,19 @@
         <v>20</v>
       </c>
       <c r="P2">
-        <v>8.9</v>
+        <v>8.5</v>
       </c>
       <c r="Q2" s="1">
-        <v>88.5</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="R2">
-        <v>87</v>
+        <v>85.5</v>
       </c>
       <c r="S2">
-        <v>96.09999999999999</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="T2">
-        <v>4.8</v>
+        <v>5.8</v>
       </c>
       <c r="U2" s="2">
         <v>1.092</v>
@@ -1840,34 +1837,34 @@
         <v>165</v>
       </c>
       <c r="W2">
-        <v>414.7</v>
+        <v>45.9</v>
       </c>
       <c r="X2">
         <v>5</v>
       </c>
       <c r="Y2" s="1">
-        <v>85.8</v>
+        <v>85.7</v>
       </c>
       <c r="Z2" s="1">
-        <v>88.3</v>
+        <v>88.2</v>
       </c>
       <c r="AA2">
-        <v>9.199999999999999</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="AB2">
-        <v>1745</v>
+        <v>1867</v>
       </c>
       <c r="AC2" t="s">
         <v>166</v>
       </c>
       <c r="AD2">
-        <v>7.7</v>
+        <v>10.4</v>
       </c>
       <c r="AE2" t="s">
         <v>166</v>
       </c>
       <c r="AF2">
-        <v>3.7</v>
+        <v>9.6</v>
       </c>
       <c r="AG2" t="s">
         <v>167</v>
@@ -1915,319 +1912,319 @@
         <v>1.6</v>
       </c>
       <c r="AV2">
-        <v>84.90000000000001</v>
+        <v>86.7</v>
       </c>
       <c r="AW2">
-        <v>66.5</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="AX2">
-        <v>55.2</v>
+        <v>55.4</v>
       </c>
       <c r="AY2">
         <v>1012.2</v>
       </c>
       <c r="AZ2">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="BA2">
-        <v>21.1</v>
+        <v>19.1</v>
       </c>
       <c r="BB2">
-        <v>8.9</v>
+        <v>8.5</v>
       </c>
       <c r="BC2">
-        <v>6.1</v>
+        <v>5.8</v>
       </c>
       <c r="BD2">
-        <v>1.1559</v>
+        <v>1.1515</v>
       </c>
       <c r="BE2">
         <v>59.8</v>
       </c>
       <c r="BF2">
-        <v>58.8</v>
+        <v>59.1</v>
       </c>
       <c r="BG2">
-        <v>52.8</v>
+        <v>51.2</v>
       </c>
       <c r="BH2">
-        <v>-7.1</v>
+        <v>-8.4</v>
       </c>
       <c r="BI2">
-        <v>-0.4</v>
+        <v>0</v>
       </c>
       <c r="BJ2">
-        <v>87.59999999999999</v>
+        <v>89.8</v>
       </c>
       <c r="BK2">
-        <v>67.09999999999999</v>
+        <v>68.7</v>
       </c>
       <c r="BL2">
-        <v>51.8</v>
+        <v>51.4</v>
       </c>
       <c r="BM2">
-        <v>1012.4</v>
+        <v>1012.2</v>
       </c>
       <c r="BN2">
-        <v>39.9</v>
+        <v>0</v>
       </c>
       <c r="BO2">
         <v>0</v>
       </c>
       <c r="BP2">
-        <v>9.300000000000001</v>
+        <v>9.1</v>
       </c>
       <c r="BQ2">
-        <v>20.6</v>
+        <v>18.7</v>
       </c>
       <c r="BR2" t="s">
         <v>174</v>
       </c>
       <c r="BS2">
-        <v>9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="BT2">
-        <v>8.699999999999999</v>
+        <v>8.5</v>
       </c>
       <c r="BU2">
-        <v>6</v>
+        <v>5.8</v>
       </c>
       <c r="BV2">
-        <v>1.1502</v>
+        <v>1.1448</v>
       </c>
       <c r="BW2">
-        <v>1917</v>
+        <v>2070</v>
       </c>
       <c r="BX2">
-        <v>89.5</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="BY2">
-        <v>1.095</v>
+        <v>1.097</v>
       </c>
       <c r="BZ2">
-        <v>86.8</v>
+        <v>87.7</v>
       </c>
       <c r="CA2">
-        <v>89.2</v>
+        <v>90.2</v>
       </c>
       <c r="CB2">
-        <v>87.8</v>
+        <v>87</v>
       </c>
       <c r="CC2">
-        <v>95.8</v>
+        <v>91.7</v>
       </c>
       <c r="CD2">
-        <v>4.8</v>
+        <v>6.8</v>
       </c>
       <c r="CE2">
-        <v>7.7</v>
+        <v>10.4</v>
       </c>
       <c r="CF2" t="s">
         <v>166</v>
       </c>
       <c r="CG2">
-        <v>84.5</v>
+        <v>86.3</v>
       </c>
       <c r="CH2">
-        <v>66.2</v>
+        <v>67.5</v>
       </c>
       <c r="CI2">
-        <v>55.2</v>
+        <v>55.3</v>
       </c>
       <c r="CJ2">
-        <v>1012.2</v>
+        <v>1012.1</v>
       </c>
       <c r="CK2">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="CL2">
         <v>0</v>
       </c>
       <c r="CM2">
-        <v>9.6</v>
+        <v>8.9</v>
       </c>
       <c r="CN2">
-        <v>21.1</v>
+        <v>19.1</v>
       </c>
       <c r="CO2" t="s">
         <v>174</v>
       </c>
       <c r="CP2">
-        <v>9.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="CQ2">
-        <v>9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="CR2">
-        <v>6.2</v>
+        <v>5.7</v>
       </c>
       <c r="CS2">
-        <v>1.1567</v>
+        <v>1.1526</v>
       </c>
       <c r="CT2">
-        <v>1721</v>
+        <v>1838</v>
       </c>
       <c r="CU2">
-        <v>88.90000000000001</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="CV2">
-        <v>1.093</v>
+        <v>1.091</v>
       </c>
       <c r="CW2">
-        <v>86.09999999999999</v>
+        <v>85.3</v>
       </c>
       <c r="CX2">
-        <v>88.59999999999999</v>
+        <v>87.7</v>
       </c>
       <c r="CY2">
-        <v>87.59999999999999</v>
+        <v>85.2</v>
       </c>
       <c r="CZ2">
-        <v>96.7</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="DA2">
-        <v>3.9</v>
+        <v>5</v>
       </c>
       <c r="DB2">
-        <v>4.3</v>
+        <v>7.4</v>
       </c>
       <c r="DC2" t="s">
         <v>166</v>
       </c>
       <c r="DD2">
-        <v>82.40000000000001</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="DE2">
-        <v>66</v>
+        <v>67.5</v>
       </c>
       <c r="DF2">
-        <v>58.5</v>
+        <v>59.7</v>
       </c>
       <c r="DG2">
-        <v>1012.1</v>
+        <v>1012.3</v>
       </c>
       <c r="DH2">
-        <v>44.4</v>
+        <v>0.3</v>
       </c>
       <c r="DI2">
         <v>0</v>
       </c>
       <c r="DJ2">
-        <v>9.800000000000001</v>
+        <v>9.1</v>
       </c>
       <c r="DK2">
-        <v>20.9</v>
+        <v>17.8</v>
       </c>
       <c r="DL2" t="s">
         <v>174</v>
       </c>
       <c r="DM2">
-        <v>9.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="DN2">
-        <v>9.199999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="DO2">
-        <v>6.3</v>
+        <v>5.9</v>
       </c>
       <c r="DP2">
-        <v>1.1614</v>
+        <v>1.1576</v>
       </c>
       <c r="DQ2">
-        <v>1581</v>
+        <v>1679</v>
       </c>
       <c r="DR2">
-        <v>87.59999999999999</v>
+        <v>86.8</v>
       </c>
       <c r="DS2">
-        <v>1.09</v>
+        <v>1.088</v>
       </c>
       <c r="DT2">
-        <v>84.7</v>
+        <v>84.2</v>
       </c>
       <c r="DU2">
-        <v>87.40000000000001</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="DV2">
-        <v>86.09999999999999</v>
+        <v>84.3</v>
       </c>
       <c r="DW2">
-        <v>96.09999999999999</v>
+        <v>93</v>
       </c>
       <c r="DX2">
-        <v>5.3</v>
+        <v>4.3</v>
       </c>
       <c r="DY2">
-        <v>2.2</v>
+        <v>6.8</v>
       </c>
       <c r="DZ2" t="s">
         <v>166</v>
       </c>
       <c r="EA2">
-        <v>80.5</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="EB2">
-        <v>65.5</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="EC2">
-        <v>61.9</v>
+        <v>63.3</v>
       </c>
       <c r="ED2">
-        <v>1012</v>
+        <v>1012.2</v>
       </c>
       <c r="EE2">
-        <v>50.6</v>
+        <v>1</v>
       </c>
       <c r="EF2">
         <v>0</v>
       </c>
       <c r="EG2">
-        <v>9.6</v>
+        <v>9</v>
       </c>
       <c r="EH2">
-        <v>18.6</v>
+        <v>16.8</v>
       </c>
       <c r="EI2" t="s">
         <v>174</v>
       </c>
       <c r="EJ2">
-        <v>9.300000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="EK2">
-        <v>9</v>
+        <v>8.5</v>
       </c>
       <c r="EL2">
-        <v>6.2</v>
+        <v>5.8</v>
       </c>
       <c r="EM2">
-        <v>1.1655</v>
+        <v>1.1631</v>
       </c>
       <c r="EN2">
-        <v>1457</v>
+        <v>1517</v>
       </c>
       <c r="EO2">
-        <v>85.40000000000001</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="EP2">
-        <v>1.085</v>
+        <v>1.084</v>
       </c>
       <c r="EQ2">
-        <v>82.7</v>
+        <v>82.3</v>
       </c>
       <c r="ER2">
-        <v>85.2</v>
+        <v>84.7</v>
       </c>
       <c r="ES2">
-        <v>83.8</v>
+        <v>82.3</v>
       </c>
       <c r="ET2">
-        <v>95.40000000000001</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="EU2">
-        <v>6.1</v>
+        <v>7.2</v>
       </c>
       <c r="EV2">
-        <v>1.3</v>
+        <v>5</v>
       </c>
       <c r="EW2" t="s">
         <v>166</v>
@@ -2292,7 +2289,7 @@
     <col min="20" max="20" width="27.7109375" customWidth="1"/>
     <col min="21" max="21" width="17.7109375" customWidth="1"/>
     <col min="22" max="22" width="25.7109375" customWidth="1"/>
-    <col min="23" max="23" width="14.7109375" customWidth="1"/>
+    <col min="23" max="23" width="12.7109375" customWidth="1"/>
     <col min="24" max="24" width="10.7109375" customWidth="1"/>
     <col min="25" max="25" width="14.7109375" customWidth="1"/>
     <col min="26" max="26" width="13.7109375" customWidth="1"/>
@@ -2546,31 +2543,31 @@
         <v>173</v>
       </c>
       <c r="J2">
-        <v>414.7</v>
+        <v>45.9</v>
       </c>
       <c r="K2">
-        <v>16.8</v>
+        <v>4.6</v>
       </c>
       <c r="L2">
         <v>5</v>
       </c>
       <c r="M2">
-        <v>0.78</v>
+        <v>1.31</v>
       </c>
       <c r="N2">
-        <v>0.57</v>
+        <v>0.53</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>4.8</v>
+        <v>6.8</v>
       </c>
       <c r="Q2">
-        <v>95.8</v>
+        <v>91.7</v>
       </c>
       <c r="R2">
-        <v>87.8</v>
+        <v>87</v>
       </c>
       <c r="S2">
         <v>0.98</v>
@@ -2588,25 +2585,25 @@
         <v>171</v>
       </c>
       <c r="X2">
-        <v>87.59999999999999</v>
+        <v>89.8</v>
       </c>
       <c r="Y2">
-        <v>90.3</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="Z2">
-        <v>67.09999999999999</v>
+        <v>68.7</v>
       </c>
       <c r="AA2">
-        <v>51.8</v>
+        <v>51.4</v>
       </c>
       <c r="AB2">
-        <v>1012.4</v>
+        <v>1012.2</v>
       </c>
       <c r="AC2">
-        <v>1014.6</v>
+        <v>1014.5</v>
       </c>
       <c r="AD2">
-        <v>39.9</v>
+        <v>0</v>
       </c>
       <c r="AE2">
         <v>0</v>
@@ -2615,16 +2612,16 @@
         <v>0</v>
       </c>
       <c r="AG2">
-        <v>70.90000000000001</v>
+        <v>74</v>
       </c>
       <c r="AH2">
-        <v>773</v>
+        <v>1042</v>
       </c>
       <c r="AI2">
-        <v>9.300000000000001</v>
+        <v>9.1</v>
       </c>
       <c r="AJ2">
-        <v>20.6</v>
+        <v>18.7</v>
       </c>
       <c r="AK2" t="s">
         <v>174</v>
@@ -2633,25 +2630,25 @@
         <v>225</v>
       </c>
       <c r="AM2">
-        <v>9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="AN2">
-        <v>8.699999999999999</v>
+        <v>8.5</v>
       </c>
       <c r="AO2">
-        <v>6</v>
+        <v>5.8</v>
       </c>
       <c r="AP2">
-        <v>-2.4</v>
+        <v>-2.3</v>
       </c>
       <c r="AQ2">
-        <v>1.1502</v>
+        <v>1.1448</v>
       </c>
       <c r="AR2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="AS2">
-        <v>1917</v>
+        <v>2070</v>
       </c>
       <c r="AT2" t="s">
         <v>167</v>
@@ -2660,49 +2657,49 @@
         <v>168</v>
       </c>
       <c r="AV2">
-        <v>89.5</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="AW2">
-        <v>1.095</v>
+        <v>1.097</v>
       </c>
       <c r="AX2">
-        <v>86.8</v>
+        <v>87.7</v>
       </c>
       <c r="AY2">
-        <v>89.2</v>
+        <v>90.2</v>
       </c>
       <c r="AZ2">
-        <v>60.2</v>
+        <v>60.5</v>
       </c>
       <c r="BA2">
-        <v>59.4</v>
+        <v>59.9</v>
       </c>
       <c r="BB2">
-        <v>49.3</v>
+        <v>46.9</v>
       </c>
       <c r="BC2">
-        <v>7.7</v>
+        <v>10.4</v>
       </c>
       <c r="BD2" t="s">
         <v>166</v>
       </c>
       <c r="BE2">
-        <v>3.7</v>
+        <v>9.6</v>
       </c>
       <c r="BF2" t="s">
         <v>166</v>
       </c>
       <c r="BG2">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="BH2">
-        <v>86.8</v>
+        <v>87.8</v>
       </c>
       <c r="BI2">
         <v>10</v>
       </c>
       <c r="BJ2">
-        <v>9</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="3" spans="1:62">
@@ -2734,31 +2731,31 @@
         <v>173</v>
       </c>
       <c r="J3">
-        <v>414.7</v>
+        <v>45.9</v>
       </c>
       <c r="K3">
-        <v>17.8</v>
+        <v>5.6</v>
       </c>
       <c r="L3">
         <v>5</v>
       </c>
       <c r="M3">
-        <v>0.12</v>
+        <v>0.41</v>
       </c>
       <c r="N3">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>3.9</v>
+        <v>5</v>
       </c>
       <c r="Q3">
-        <v>96.7</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="R3">
-        <v>87.59999999999999</v>
+        <v>85.2</v>
       </c>
       <c r="S3">
         <v>0.98</v>
@@ -2773,28 +2770,28 @@
         <v>1.6</v>
       </c>
       <c r="W3" t="s">
-        <v>230</v>
+        <v>171</v>
       </c>
       <c r="X3">
-        <v>84.5</v>
+        <v>86.3</v>
       </c>
       <c r="Y3">
-        <v>85.5</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="Z3">
-        <v>66.2</v>
+        <v>67.5</v>
       </c>
       <c r="AA3">
-        <v>55.2</v>
+        <v>55.3</v>
       </c>
       <c r="AB3">
-        <v>1012.2</v>
+        <v>1012.1</v>
       </c>
       <c r="AC3">
-        <v>1014.5</v>
+        <v>1014.4</v>
       </c>
       <c r="AD3">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AE3">
         <v>0</v>
@@ -2803,16 +2800,16 @@
         <v>0</v>
       </c>
       <c r="AG3">
-        <v>66.90000000000001</v>
+        <v>67.7</v>
       </c>
       <c r="AH3">
-        <v>429</v>
+        <v>743</v>
       </c>
       <c r="AI3">
-        <v>9.6</v>
+        <v>8.9</v>
       </c>
       <c r="AJ3">
-        <v>21.1</v>
+        <v>19.1</v>
       </c>
       <c r="AK3" t="s">
         <v>174</v>
@@ -2821,25 +2818,25 @@
         <v>225</v>
       </c>
       <c r="AM3">
-        <v>9.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="AN3">
-        <v>9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="AO3">
-        <v>6.2</v>
+        <v>5.7</v>
       </c>
       <c r="AP3">
-        <v>-2.5</v>
+        <v>-2.3</v>
       </c>
       <c r="AQ3">
-        <v>1.1567</v>
+        <v>1.1526</v>
       </c>
       <c r="AR3" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="AS3">
-        <v>1721</v>
+        <v>1838</v>
       </c>
       <c r="AT3" t="s">
         <v>167</v>
@@ -2848,49 +2845,49 @@
         <v>168</v>
       </c>
       <c r="AV3">
-        <v>88.90000000000001</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="AW3">
-        <v>1.093</v>
+        <v>1.091</v>
       </c>
       <c r="AX3">
-        <v>86.09999999999999</v>
+        <v>85.3</v>
       </c>
       <c r="AY3">
-        <v>88.59999999999999</v>
+        <v>87.7</v>
       </c>
       <c r="AZ3">
-        <v>59.8</v>
+        <v>59.6</v>
       </c>
       <c r="BA3">
-        <v>58.7</v>
+        <v>58.9</v>
       </c>
       <c r="BB3">
-        <v>53</v>
+        <v>51.6</v>
       </c>
       <c r="BC3">
-        <v>4.3</v>
+        <v>7.4</v>
       </c>
       <c r="BD3" t="s">
         <v>166</v>
       </c>
       <c r="BE3">
-        <v>2.8</v>
+        <v>8.9</v>
       </c>
       <c r="BF3" t="s">
         <v>166</v>
       </c>
       <c r="BG3">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="BH3">
-        <v>83.7</v>
+        <v>84.5</v>
       </c>
       <c r="BI3">
         <v>10</v>
       </c>
       <c r="BJ3">
-        <v>9.6</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:62">
@@ -2922,31 +2919,31 @@
         <v>173</v>
       </c>
       <c r="J4">
-        <v>414.7</v>
+        <v>45.9</v>
       </c>
       <c r="K4">
-        <v>18.8</v>
+        <v>6.6</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>0.45</v>
+        <v>0.3</v>
       </c>
       <c r="N4">
-        <v>1.14</v>
+        <v>1.04</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>5.3</v>
+        <v>4.3</v>
       </c>
       <c r="Q4">
-        <v>96.09999999999999</v>
+        <v>93</v>
       </c>
       <c r="R4">
-        <v>86.09999999999999</v>
+        <v>84.3</v>
       </c>
       <c r="S4">
         <v>0.98</v>
@@ -2964,25 +2961,25 @@
         <v>171</v>
       </c>
       <c r="X4">
-        <v>82.40000000000001</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="Y4">
-        <v>82.2</v>
+        <v>85.2</v>
       </c>
       <c r="Z4">
-        <v>66</v>
+        <v>67.5</v>
       </c>
       <c r="AA4">
-        <v>58.5</v>
+        <v>59.7</v>
       </c>
       <c r="AB4">
-        <v>1012.1</v>
+        <v>1012.3</v>
       </c>
       <c r="AC4">
-        <v>1014.4</v>
+        <v>1014.5</v>
       </c>
       <c r="AD4">
-        <v>44.4</v>
+        <v>0.3</v>
       </c>
       <c r="AE4">
         <v>0</v>
@@ -2991,16 +2988,16 @@
         <v>0</v>
       </c>
       <c r="AG4">
-        <v>61.8</v>
+        <v>55.5</v>
       </c>
       <c r="AH4">
-        <v>224</v>
+        <v>684</v>
       </c>
       <c r="AI4">
-        <v>9.800000000000001</v>
+        <v>9.1</v>
       </c>
       <c r="AJ4">
-        <v>20.9</v>
+        <v>17.8</v>
       </c>
       <c r="AK4" t="s">
         <v>174</v>
@@ -3009,25 +3006,25 @@
         <v>225</v>
       </c>
       <c r="AM4">
-        <v>9.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="AN4">
-        <v>9.199999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="AO4">
-        <v>6.3</v>
+        <v>5.9</v>
       </c>
       <c r="AP4">
-        <v>-2.5</v>
+        <v>-2.4</v>
       </c>
       <c r="AQ4">
-        <v>1.1614</v>
+        <v>1.1576</v>
       </c>
       <c r="AR4" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="AS4">
-        <v>1581</v>
+        <v>1679</v>
       </c>
       <c r="AT4" t="s">
         <v>167</v>
@@ -3036,49 +3033,49 @@
         <v>168</v>
       </c>
       <c r="AV4">
-        <v>87.59999999999999</v>
+        <v>86.8</v>
       </c>
       <c r="AW4">
-        <v>1.09</v>
+        <v>1.088</v>
       </c>
       <c r="AX4">
-        <v>84.7</v>
+        <v>84.2</v>
       </c>
       <c r="AY4">
-        <v>87.40000000000001</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="AZ4">
-        <v>59.5</v>
+        <v>59.3</v>
       </c>
       <c r="BA4">
-        <v>58.3</v>
+        <v>58.5</v>
       </c>
       <c r="BB4">
-        <v>55.9</v>
+        <v>55.2</v>
       </c>
       <c r="BC4">
-        <v>2.2</v>
+        <v>6.8</v>
       </c>
       <c r="BD4" t="s">
         <v>166</v>
       </c>
       <c r="BE4">
-        <v>2.8</v>
+        <v>9.1</v>
       </c>
       <c r="BF4" t="s">
         <v>166</v>
       </c>
       <c r="BG4">
+        <v>85</v>
+      </c>
+      <c r="BH4">
         <v>82</v>
-      </c>
-      <c r="BH4">
-        <v>81.40000000000001</v>
       </c>
       <c r="BI4">
         <v>10</v>
       </c>
       <c r="BJ4">
-        <v>10</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="5" spans="1:62">
@@ -3110,31 +3107,31 @@
         <v>173</v>
       </c>
       <c r="J5">
-        <v>414.7</v>
+        <v>45.9</v>
       </c>
       <c r="K5">
-        <v>19.8</v>
+        <v>7.6</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>0.83</v>
+        <v>0.93</v>
       </c>
       <c r="N5">
-        <v>0.9399999999999999</v>
+        <v>1.16</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>6.1</v>
+        <v>7.2</v>
       </c>
       <c r="Q5">
-        <v>95.40000000000001</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="R5">
-        <v>83.8</v>
+        <v>82.3</v>
       </c>
       <c r="S5">
         <v>0.98</v>
@@ -3152,25 +3149,25 @@
         <v>171</v>
       </c>
       <c r="X5">
-        <v>80.5</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="Y5">
-        <v>79.8</v>
+        <v>82.5</v>
       </c>
       <c r="Z5">
-        <v>65.5</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="AA5">
-        <v>61.9</v>
+        <v>63.3</v>
       </c>
       <c r="AB5">
-        <v>1012</v>
+        <v>1012.2</v>
       </c>
       <c r="AC5">
-        <v>1014.3</v>
+        <v>1014.5</v>
       </c>
       <c r="AD5">
-        <v>50.6</v>
+        <v>1</v>
       </c>
       <c r="AE5">
         <v>0</v>
@@ -3179,16 +3176,16 @@
         <v>0</v>
       </c>
       <c r="AG5">
-        <v>60.1</v>
+        <v>49.1</v>
       </c>
       <c r="AH5">
-        <v>134</v>
+        <v>504</v>
       </c>
       <c r="AI5">
-        <v>9.6</v>
+        <v>9</v>
       </c>
       <c r="AJ5">
-        <v>18.6</v>
+        <v>16.8</v>
       </c>
       <c r="AK5" t="s">
         <v>174</v>
@@ -3197,25 +3194,25 @@
         <v>225</v>
       </c>
       <c r="AM5">
-        <v>9.300000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="AN5">
-        <v>9</v>
+        <v>8.5</v>
       </c>
       <c r="AO5">
-        <v>6.2</v>
+        <v>5.8</v>
       </c>
       <c r="AP5">
-        <v>-2.5</v>
+        <v>-2.3</v>
       </c>
       <c r="AQ5">
-        <v>1.1655</v>
+        <v>1.1631</v>
       </c>
       <c r="AR5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="AS5">
-        <v>1457</v>
+        <v>1517</v>
       </c>
       <c r="AT5" t="s">
         <v>167</v>
@@ -3224,49 +3221,49 @@
         <v>168</v>
       </c>
       <c r="AV5">
-        <v>85.40000000000001</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="AW5">
-        <v>1.085</v>
+        <v>1.084</v>
       </c>
       <c r="AX5">
-        <v>82.7</v>
+        <v>82.3</v>
       </c>
       <c r="AY5">
-        <v>85.2</v>
+        <v>84.7</v>
       </c>
       <c r="AZ5">
+        <v>58.7</v>
+      </c>
+      <c r="BA5">
+        <v>57.9</v>
+      </c>
+      <c r="BB5">
         <v>59</v>
       </c>
-      <c r="BA5">
-        <v>57.7</v>
-      </c>
-      <c r="BB5">
-        <v>60.2</v>
-      </c>
       <c r="BC5">
-        <v>1.3</v>
+        <v>5</v>
       </c>
       <c r="BD5" t="s">
         <v>166</v>
       </c>
       <c r="BE5">
-        <v>3.3</v>
+        <v>7.9</v>
       </c>
       <c r="BF5" t="s">
         <v>166</v>
       </c>
       <c r="BG5">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="BH5">
-        <v>79.59999999999999</v>
+        <v>79.8</v>
       </c>
       <c r="BI5">
         <v>10</v>
       </c>
       <c r="BJ5">
-        <v>9.6</v>
+        <v>8.5</v>
       </c>
     </row>
   </sheetData>
@@ -3371,10 +3368,10 @@
         <v>160</v>
       </c>
       <c r="E2">
-        <v>88.5</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="F2">
-        <v>87</v>
+        <v>85.5</v>
       </c>
       <c r="G2" t="s">
         <v>163</v>
@@ -3386,22 +3383,22 @@
         <v>20</v>
       </c>
       <c r="J2" s="5">
-        <v>8.9</v>
+        <v>8.5</v>
       </c>
       <c r="K2" t="s">
         <v>161</v>
       </c>
       <c r="L2">
-        <v>96.09999999999999</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="M2">
-        <v>9.199999999999999</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="N2">
-        <v>84.90000000000001</v>
+        <v>86.7</v>
       </c>
       <c r="O2">
-        <v>1745</v>
+        <v>1867</v>
       </c>
       <c r="P2" t="s">
         <v>167</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 12:34 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_2026_07_14.xlsx
+++ b/mlb_weather_professional_2026_07_14.xlsx
@@ -12,8 +12,8 @@
     <sheet name="HR Weather" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Game Summary'!$A$1:$EX$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hourly Detail'!$A$1:$BJ$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Game Summary'!$A$1:$FK$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hourly Detail'!$A$1:$BU$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'HR Weather'!$A$1:$R$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="264">
   <si>
     <t>Date</t>
   </si>
@@ -86,6 +86,39 @@
     <t>Game Carry Multiplier</t>
   </si>
   <si>
+    <t>Forecast Trend</t>
+  </si>
+  <si>
+    <t>Carry Score Change Since Last Run</t>
+  </si>
+  <si>
+    <t>Temp Change Since Last Run F</t>
+  </si>
+  <si>
+    <t>Wind Toward CF Change Since Last Run MPH</t>
+  </si>
+  <si>
+    <t>Precip Change Since Last Run Pct</t>
+  </si>
+  <si>
+    <t>Game Probability Wind Blowing Out %</t>
+  </si>
+  <si>
+    <t>Game Probability Wind Blowing In %</t>
+  </si>
+  <si>
+    <t>Game Wind Direction Spread Degrees</t>
+  </si>
+  <si>
+    <t>Game Wind Toward CF Spread MPH</t>
+  </si>
+  <si>
+    <t>Current Temp Bias F</t>
+  </si>
+  <si>
+    <t>Current Wind Bias MPH</t>
+  </si>
+  <si>
     <t>Forecast Run PT</t>
   </si>
   <si>
@@ -482,6 +515,12 @@
     <t>+3 Hours Delay Risk</t>
   </si>
   <si>
+    <t>Previous Forecast Run UTC</t>
+  </si>
+  <si>
+    <t>Wind Out Probability Change Since Last Run Pct</t>
+  </si>
+  <si>
     <t>Carry Percentile Value</t>
   </si>
   <si>
@@ -509,7 +548,7 @@
     <t>🔥 Excellent</t>
   </si>
   <si>
-    <t>adjusted carry 85.5; +20 ft carry; +8.5% HR env.</t>
+    <t>adjusted carry 84.3; +19 ft carry; +8.2% HR env.</t>
   </si>
   <si>
     <t>100th</t>
@@ -518,7 +557,10 @@
     <t>A</t>
   </si>
   <si>
-    <t>2026-07-14 12:26:55 PM PDT</t>
+    <t>STEADY</t>
+  </si>
+  <si>
+    <t>2026-07-14 12:34:18 PM PDT</t>
   </si>
   <si>
     <t>LOW</t>
@@ -539,15 +581,18 @@
     <t>Clear</t>
   </si>
   <si>
+    <t>2026-07-14 19:34:18 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14T18:41:01+00:00</t>
+  </si>
+  <si>
+    <t>SW</t>
+  </si>
+  <si>
     <t>2026-07-14 19:26:55 UTC</t>
   </si>
   <si>
-    <t>2026-07-14T18:41:01+00:00</t>
-  </si>
-  <si>
-    <t>SW</t>
-  </si>
-  <si>
     <t>Period</t>
   </si>
   <si>
@@ -566,6 +611,39 @@
     <t>Precip Model Spread Pct</t>
   </si>
   <si>
+    <t>Wind Direction Spread Degrees</t>
+  </si>
+  <si>
+    <t>Wind Toward CF Spread MPH</t>
+  </si>
+  <si>
+    <t>Probability Wind Blowing Out %</t>
+  </si>
+  <si>
+    <t>Probability Wind Blowing In %</t>
+  </si>
+  <si>
+    <t>Exact-Time Interpolation</t>
+  </si>
+  <si>
+    <t>Interpolation Lower Time</t>
+  </si>
+  <si>
+    <t>Interpolation Upper Time</t>
+  </si>
+  <si>
+    <t>Interpolation Fraction</t>
+  </si>
+  <si>
+    <t>Observation Bias Weight</t>
+  </si>
+  <si>
+    <t>Temperature Bias Applied F</t>
+  </si>
+  <si>
+    <t>Wind Bias Applied MPH</t>
+  </si>
+  <si>
     <t>Ensemble Disagreement Score</t>
   </si>
   <si>
@@ -711,6 +789,24 @@
   </si>
   <si>
     <t>11:00 PM EDT</t>
+  </si>
+  <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>2026-07-14T19:00</t>
+  </si>
+  <si>
+    <t>2026-07-14T20:00</t>
+  </si>
+  <si>
+    <t>2026-07-14T21:00</t>
+  </si>
+  <si>
+    <t>2026-07-14T22:00</t>
+  </si>
+  <si>
+    <t>2026-07-14T23:00</t>
   </si>
   <si>
     <t>LIGHT</t>
@@ -1172,7 +1268,7 @@
   <sheetPr>
     <tabColor rgb="FF70AD47"/>
   </sheetPr>
-  <dimension ref="A1:EX2"/>
+  <dimension ref="A1:FK2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -1195,117 +1291,126 @@
     <col min="19" max="19" width="27.7109375" customWidth="1"/>
     <col min="20" max="20" width="34.7109375" customWidth="1"/>
     <col min="21" max="21" width="20.7109375" style="2" customWidth="1"/>
-    <col min="22" max="22" width="28.7109375" customWidth="1"/>
-    <col min="23" max="23" width="22.7109375" customWidth="1"/>
-    <col min="24" max="24" width="18.7109375" customWidth="1"/>
-    <col min="25" max="26" width="18.7109375" style="1" customWidth="1"/>
-    <col min="27" max="27" width="29.7109375" customWidth="1"/>
-    <col min="28" max="28" width="30.7109375" customWidth="1"/>
-    <col min="29" max="29" width="16.7109375" customWidth="1"/>
-    <col min="30" max="31" width="22.7109375" customWidth="1"/>
-    <col min="32" max="32" width="28.7109375" customWidth="1"/>
-    <col min="33" max="33" width="23.7109375" customWidth="1"/>
-    <col min="34" max="34" width="19.7109375" customWidth="1"/>
-    <col min="35" max="35" width="20.7109375" customWidth="1"/>
-    <col min="36" max="36" width="13.7109375" customWidth="1"/>
-    <col min="37" max="38" width="11.7109375" customWidth="1"/>
-    <col min="39" max="40" width="20.7109375" customWidth="1"/>
-    <col min="41" max="41" width="11.7109375" customWidth="1"/>
-    <col min="42" max="42" width="20.7109375" customWidth="1"/>
-    <col min="43" max="43" width="25.7109375" customWidth="1"/>
-    <col min="44" max="44" width="27.7109375" customWidth="1"/>
-    <col min="45" max="45" width="20.7109375" customWidth="1"/>
-    <col min="46" max="46" width="27.7109375" customWidth="1"/>
-    <col min="47" max="48" width="17.7109375" customWidth="1"/>
-    <col min="49" max="49" width="22.7109375" customWidth="1"/>
-    <col min="50" max="50" width="15.7109375" customWidth="1"/>
-    <col min="51" max="51" width="23.7109375" customWidth="1"/>
-    <col min="52" max="53" width="19.7109375" customWidth="1"/>
-    <col min="54" max="55" width="29.7109375" customWidth="1"/>
-    <col min="56" max="56" width="28.7109375" customWidth="1"/>
-    <col min="57" max="57" width="16.7109375" customWidth="1"/>
-    <col min="58" max="58" width="28.7109375" customWidth="1"/>
-    <col min="59" max="59" width="29.7109375" customWidth="1"/>
-    <col min="60" max="60" width="27.7109375" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="62" width="20.7109375" customWidth="1"/>
-    <col min="63" max="63" width="25.7109375" customWidth="1"/>
-    <col min="64" max="64" width="18.7109375" customWidth="1"/>
-    <col min="65" max="65" width="34.7109375" customWidth="1"/>
-    <col min="66" max="66" width="27.7109375" customWidth="1"/>
-    <col min="67" max="68" width="22.7109375" customWidth="1"/>
-    <col min="69" max="69" width="27.7109375" customWidth="1"/>
-    <col min="70" max="70" width="23.7109375" customWidth="1"/>
-    <col min="71" max="73" width="32.7109375" customWidth="1"/>
-    <col min="74" max="74" width="31.7109375" customWidth="1"/>
-    <col min="75" max="75" width="33.7109375" customWidth="1"/>
-    <col min="76" max="76" width="28.7109375" customWidth="1"/>
-    <col min="77" max="77" width="30.7109375" customWidth="1"/>
-    <col min="78" max="79" width="29.7109375" customWidth="1"/>
-    <col min="80" max="82" width="34.7109375" customWidth="1"/>
-    <col min="83" max="83" width="30.7109375" customWidth="1"/>
-    <col min="84" max="84" width="24.7109375" customWidth="1"/>
-    <col min="85" max="85" width="16.7109375" customWidth="1"/>
-    <col min="86" max="86" width="21.7109375" customWidth="1"/>
-    <col min="87" max="87" width="14.7109375" customWidth="1"/>
+    <col min="22" max="22" width="16.7109375" customWidth="1"/>
+    <col min="23" max="23" width="34.7109375" customWidth="1"/>
+    <col min="24" max="24" width="30.7109375" customWidth="1"/>
+    <col min="25" max="29" width="34.7109375" customWidth="1"/>
+    <col min="30" max="30" width="32.7109375" customWidth="1"/>
+    <col min="31" max="31" width="21.7109375" customWidth="1"/>
+    <col min="32" max="32" width="23.7109375" customWidth="1"/>
+    <col min="33" max="33" width="28.7109375" customWidth="1"/>
+    <col min="34" max="34" width="22.7109375" customWidth="1"/>
+    <col min="35" max="35" width="18.7109375" customWidth="1"/>
+    <col min="36" max="37" width="18.7109375" style="1" customWidth="1"/>
+    <col min="38" max="38" width="29.7109375" customWidth="1"/>
+    <col min="39" max="39" width="30.7109375" customWidth="1"/>
+    <col min="40" max="40" width="16.7109375" customWidth="1"/>
+    <col min="41" max="42" width="22.7109375" customWidth="1"/>
+    <col min="43" max="43" width="28.7109375" customWidth="1"/>
+    <col min="44" max="44" width="23.7109375" customWidth="1"/>
+    <col min="45" max="45" width="19.7109375" customWidth="1"/>
+    <col min="46" max="46" width="20.7109375" customWidth="1"/>
+    <col min="47" max="47" width="13.7109375" customWidth="1"/>
+    <col min="48" max="49" width="11.7109375" customWidth="1"/>
+    <col min="50" max="51" width="20.7109375" customWidth="1"/>
+    <col min="52" max="52" width="11.7109375" customWidth="1"/>
+    <col min="53" max="53" width="20.7109375" customWidth="1"/>
+    <col min="54" max="54" width="25.7109375" customWidth="1"/>
+    <col min="55" max="55" width="27.7109375" customWidth="1"/>
+    <col min="56" max="56" width="20.7109375" customWidth="1"/>
+    <col min="57" max="57" width="27.7109375" customWidth="1"/>
+    <col min="58" max="59" width="17.7109375" customWidth="1"/>
+    <col min="60" max="60" width="22.7109375" customWidth="1"/>
+    <col min="61" max="61" width="15.7109375" customWidth="1"/>
+    <col min="62" max="62" width="23.7109375" customWidth="1"/>
+    <col min="63" max="64" width="19.7109375" customWidth="1"/>
+    <col min="65" max="66" width="29.7109375" customWidth="1"/>
+    <col min="67" max="67" width="28.7109375" customWidth="1"/>
+    <col min="68" max="68" width="16.7109375" customWidth="1"/>
+    <col min="69" max="69" width="28.7109375" customWidth="1"/>
+    <col min="70" max="70" width="29.7109375" customWidth="1"/>
+    <col min="71" max="71" width="27.7109375" customWidth="1"/>
+    <col min="72" max="72" width="21.7109375" customWidth="1"/>
+    <col min="73" max="73" width="20.7109375" customWidth="1"/>
+    <col min="74" max="74" width="25.7109375" customWidth="1"/>
+    <col min="75" max="75" width="18.7109375" customWidth="1"/>
+    <col min="76" max="76" width="34.7109375" customWidth="1"/>
+    <col min="77" max="77" width="27.7109375" customWidth="1"/>
+    <col min="78" max="79" width="22.7109375" customWidth="1"/>
+    <col min="80" max="80" width="27.7109375" customWidth="1"/>
+    <col min="81" max="81" width="23.7109375" customWidth="1"/>
+    <col min="82" max="84" width="32.7109375" customWidth="1"/>
+    <col min="85" max="85" width="31.7109375" customWidth="1"/>
+    <col min="86" max="86" width="33.7109375" customWidth="1"/>
+    <col min="87" max="87" width="28.7109375" customWidth="1"/>
     <col min="88" max="88" width="30.7109375" customWidth="1"/>
-    <col min="89" max="89" width="23.7109375" customWidth="1"/>
-    <col min="90" max="91" width="18.7109375" customWidth="1"/>
-    <col min="92" max="92" width="23.7109375" customWidth="1"/>
-    <col min="93" max="93" width="19.7109375" customWidth="1"/>
-    <col min="94" max="96" width="28.7109375" customWidth="1"/>
-    <col min="97" max="97" width="27.7109375" customWidth="1"/>
-    <col min="98" max="98" width="29.7109375" customWidth="1"/>
-    <col min="99" max="99" width="24.7109375" customWidth="1"/>
-    <col min="100" max="100" width="26.7109375" customWidth="1"/>
-    <col min="101" max="102" width="25.7109375" customWidth="1"/>
-    <col min="103" max="103" width="34.7109375" customWidth="1"/>
-    <col min="104" max="104" width="30.7109375" customWidth="1"/>
-    <col min="105" max="105" width="34.7109375" customWidth="1"/>
-    <col min="106" max="106" width="26.7109375" customWidth="1"/>
-    <col min="107" max="107" width="20.7109375" customWidth="1"/>
-    <col min="108" max="108" width="17.7109375" customWidth="1"/>
-    <col min="109" max="109" width="22.7109375" customWidth="1"/>
-    <col min="110" max="110" width="15.7109375" customWidth="1"/>
-    <col min="111" max="111" width="31.7109375" customWidth="1"/>
-    <col min="112" max="112" width="24.7109375" customWidth="1"/>
-    <col min="113" max="114" width="19.7109375" customWidth="1"/>
-    <col min="115" max="115" width="24.7109375" customWidth="1"/>
-    <col min="116" max="116" width="20.7109375" customWidth="1"/>
-    <col min="117" max="119" width="29.7109375" customWidth="1"/>
-    <col min="120" max="120" width="28.7109375" customWidth="1"/>
-    <col min="121" max="121" width="30.7109375" customWidth="1"/>
-    <col min="122" max="122" width="25.7109375" customWidth="1"/>
-    <col min="123" max="123" width="27.7109375" customWidth="1"/>
-    <col min="124" max="125" width="26.7109375" customWidth="1"/>
-    <col min="126" max="126" width="34.7109375" customWidth="1"/>
-    <col min="127" max="127" width="31.7109375" customWidth="1"/>
-    <col min="128" max="128" width="34.7109375" customWidth="1"/>
-    <col min="129" max="129" width="27.7109375" customWidth="1"/>
-    <col min="130" max="130" width="21.7109375" customWidth="1"/>
-    <col min="131" max="131" width="17.7109375" customWidth="1"/>
-    <col min="132" max="132" width="22.7109375" customWidth="1"/>
-    <col min="133" max="133" width="15.7109375" customWidth="1"/>
-    <col min="134" max="134" width="31.7109375" customWidth="1"/>
-    <col min="135" max="135" width="24.7109375" customWidth="1"/>
-    <col min="136" max="137" width="19.7109375" customWidth="1"/>
-    <col min="138" max="138" width="24.7109375" customWidth="1"/>
-    <col min="139" max="139" width="20.7109375" customWidth="1"/>
-    <col min="140" max="142" width="29.7109375" customWidth="1"/>
-    <col min="143" max="143" width="28.7109375" customWidth="1"/>
-    <col min="144" max="144" width="30.7109375" customWidth="1"/>
-    <col min="145" max="145" width="25.7109375" customWidth="1"/>
-    <col min="146" max="146" width="27.7109375" customWidth="1"/>
-    <col min="147" max="148" width="26.7109375" customWidth="1"/>
-    <col min="149" max="149" width="34.7109375" customWidth="1"/>
-    <col min="150" max="150" width="31.7109375" customWidth="1"/>
-    <col min="151" max="151" width="34.7109375" customWidth="1"/>
-    <col min="152" max="152" width="27.7109375" customWidth="1"/>
-    <col min="153" max="153" width="21.7109375" customWidth="1"/>
-    <col min="154" max="154" width="24.7109375" customWidth="1"/>
+    <col min="89" max="90" width="29.7109375" customWidth="1"/>
+    <col min="91" max="93" width="34.7109375" customWidth="1"/>
+    <col min="94" max="94" width="30.7109375" customWidth="1"/>
+    <col min="95" max="95" width="24.7109375" customWidth="1"/>
+    <col min="96" max="96" width="16.7109375" customWidth="1"/>
+    <col min="97" max="97" width="21.7109375" customWidth="1"/>
+    <col min="98" max="98" width="14.7109375" customWidth="1"/>
+    <col min="99" max="99" width="30.7109375" customWidth="1"/>
+    <col min="100" max="100" width="23.7109375" customWidth="1"/>
+    <col min="101" max="102" width="18.7109375" customWidth="1"/>
+    <col min="103" max="103" width="23.7109375" customWidth="1"/>
+    <col min="104" max="104" width="19.7109375" customWidth="1"/>
+    <col min="105" max="107" width="28.7109375" customWidth="1"/>
+    <col min="108" max="108" width="27.7109375" customWidth="1"/>
+    <col min="109" max="109" width="29.7109375" customWidth="1"/>
+    <col min="110" max="110" width="24.7109375" customWidth="1"/>
+    <col min="111" max="111" width="26.7109375" customWidth="1"/>
+    <col min="112" max="113" width="25.7109375" customWidth="1"/>
+    <col min="114" max="114" width="34.7109375" customWidth="1"/>
+    <col min="115" max="115" width="30.7109375" customWidth="1"/>
+    <col min="116" max="116" width="34.7109375" customWidth="1"/>
+    <col min="117" max="117" width="26.7109375" customWidth="1"/>
+    <col min="118" max="118" width="20.7109375" customWidth="1"/>
+    <col min="119" max="119" width="17.7109375" customWidth="1"/>
+    <col min="120" max="120" width="22.7109375" customWidth="1"/>
+    <col min="121" max="121" width="15.7109375" customWidth="1"/>
+    <col min="122" max="122" width="31.7109375" customWidth="1"/>
+    <col min="123" max="123" width="24.7109375" customWidth="1"/>
+    <col min="124" max="125" width="19.7109375" customWidth="1"/>
+    <col min="126" max="126" width="24.7109375" customWidth="1"/>
+    <col min="127" max="127" width="20.7109375" customWidth="1"/>
+    <col min="128" max="130" width="29.7109375" customWidth="1"/>
+    <col min="131" max="131" width="28.7109375" customWidth="1"/>
+    <col min="132" max="132" width="30.7109375" customWidth="1"/>
+    <col min="133" max="133" width="25.7109375" customWidth="1"/>
+    <col min="134" max="134" width="27.7109375" customWidth="1"/>
+    <col min="135" max="136" width="26.7109375" customWidth="1"/>
+    <col min="137" max="137" width="34.7109375" customWidth="1"/>
+    <col min="138" max="138" width="31.7109375" customWidth="1"/>
+    <col min="139" max="139" width="34.7109375" customWidth="1"/>
+    <col min="140" max="140" width="27.7109375" customWidth="1"/>
+    <col min="141" max="141" width="21.7109375" customWidth="1"/>
+    <col min="142" max="142" width="17.7109375" customWidth="1"/>
+    <col min="143" max="143" width="22.7109375" customWidth="1"/>
+    <col min="144" max="144" width="15.7109375" customWidth="1"/>
+    <col min="145" max="145" width="31.7109375" customWidth="1"/>
+    <col min="146" max="146" width="24.7109375" customWidth="1"/>
+    <col min="147" max="148" width="19.7109375" customWidth="1"/>
+    <col min="149" max="149" width="24.7109375" customWidth="1"/>
+    <col min="150" max="150" width="20.7109375" customWidth="1"/>
+    <col min="151" max="153" width="29.7109375" customWidth="1"/>
+    <col min="154" max="154" width="28.7109375" customWidth="1"/>
+    <col min="155" max="155" width="30.7109375" customWidth="1"/>
+    <col min="156" max="156" width="25.7109375" customWidth="1"/>
+    <col min="157" max="157" width="27.7109375" customWidth="1"/>
+    <col min="158" max="159" width="26.7109375" customWidth="1"/>
+    <col min="160" max="160" width="34.7109375" customWidth="1"/>
+    <col min="161" max="161" width="31.7109375" customWidth="1"/>
+    <col min="162" max="162" width="34.7109375" customWidth="1"/>
+    <col min="163" max="163" width="27.7109375" customWidth="1"/>
+    <col min="164" max="164" width="21.7109375" customWidth="1"/>
+    <col min="165" max="165" width="27.7109375" customWidth="1"/>
+    <col min="166" max="166" width="34.7109375" customWidth="1"/>
+    <col min="167" max="167" width="24.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:154" ht="34" customHeight="1">
+    <row r="1" spans="1:167" ht="34" customHeight="1">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1768,473 +1873,551 @@
       <c r="EX1" s="3" t="s">
         <v>153</v>
       </c>
+      <c r="EY1" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="EZ1" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="FA1" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="FB1" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="FC1" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="FD1" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="FE1" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="FF1" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="FG1" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="FH1" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="FI1" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="FJ1" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="FK1" s="3" t="s">
+        <v>166</v>
+      </c>
     </row>
-    <row r="2" spans="1:154">
+    <row r="2" spans="1:167">
       <c r="A2" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="B2" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="C2" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="D2" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="E2" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
       <c r="F2" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="G2" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="H2" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="I2" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="J2" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="K2">
-        <v>88.40000000000001</v>
+        <v>87.8</v>
       </c>
       <c r="L2">
-        <v>85.5</v>
+        <v>84.3</v>
       </c>
       <c r="M2" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
       <c r="N2" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
       <c r="O2">
+        <v>19</v>
+      </c>
+      <c r="P2">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>87.8</v>
+      </c>
+      <c r="R2">
+        <v>84.3</v>
+      </c>
+      <c r="S2">
+        <v>90.8</v>
+      </c>
+      <c r="T2">
+        <v>6.7</v>
+      </c>
+      <c r="U2" s="2">
+        <v>1.091</v>
+      </c>
+      <c r="V2" t="s">
+        <v>178</v>
+      </c>
+      <c r="W2">
+        <v>-1.2</v>
+      </c>
+      <c r="X2">
+        <v>86.3</v>
+      </c>
+      <c r="Y2">
+        <v>-0.1</v>
+      </c>
+      <c r="Z2">
+        <v>0</v>
+      </c>
+      <c r="AA2">
+        <v>100</v>
+      </c>
+      <c r="AB2">
+        <v>0</v>
+      </c>
+      <c r="AC2">
+        <v>2.3</v>
+      </c>
+      <c r="AD2">
+        <v>0.9</v>
+      </c>
+      <c r="AE2">
+        <v>0.15</v>
+      </c>
+      <c r="AF2">
+        <v>0.12</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>179</v>
+      </c>
+      <c r="AH2">
+        <v>53.3</v>
+      </c>
+      <c r="AI2">
+        <v>5</v>
+      </c>
+      <c r="AJ2" s="1">
+        <v>85.2</v>
+      </c>
+      <c r="AK2" s="1">
+        <v>87.59999999999999</v>
+      </c>
+      <c r="AL2">
+        <v>8.6</v>
+      </c>
+      <c r="AM2">
+        <v>1833</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>180</v>
+      </c>
+      <c r="AO2">
+        <v>10.4</v>
+      </c>
+      <c r="AP2" t="s">
+        <v>180</v>
+      </c>
+      <c r="AQ2">
+        <v>12.1</v>
+      </c>
+      <c r="AR2" t="s">
+        <v>181</v>
+      </c>
+      <c r="AS2" t="s">
+        <v>182</v>
+      </c>
+      <c r="AT2" t="s">
+        <v>173</v>
+      </c>
+      <c r="AU2" t="s">
+        <v>183</v>
+      </c>
+      <c r="AV2">
+        <v>39.9061</v>
+      </c>
+      <c r="AW2">
+        <v>-75.1665</v>
+      </c>
+      <c r="AX2">
         <v>20</v>
       </c>
-      <c r="P2">
+      <c r="AY2">
+        <v>60</v>
+      </c>
+      <c r="AZ2" t="s">
+        <v>184</v>
+      </c>
+      <c r="BA2" t="s">
+        <v>185</v>
+      </c>
+      <c r="BB2" t="s">
+        <v>186</v>
+      </c>
+      <c r="BC2" t="s">
+        <v>187</v>
+      </c>
+      <c r="BD2">
+        <v>0.98</v>
+      </c>
+      <c r="BE2">
+        <v>0.7</v>
+      </c>
+      <c r="BF2">
+        <v>1.6</v>
+      </c>
+      <c r="BG2">
+        <v>86.3</v>
+      </c>
+      <c r="BH2">
+        <v>67.40000000000001</v>
+      </c>
+      <c r="BI2">
+        <v>55.4</v>
+      </c>
+      <c r="BJ2">
+        <v>1012.2</v>
+      </c>
+      <c r="BK2">
+        <v>8.9</v>
+      </c>
+      <c r="BL2">
+        <v>19.4</v>
+      </c>
+      <c r="BM2">
+        <v>8.4</v>
+      </c>
+      <c r="BN2">
+        <v>5.7</v>
+      </c>
+      <c r="BO2">
+        <v>1.1528</v>
+      </c>
+      <c r="BP2">
+        <v>59.6</v>
+      </c>
+      <c r="BQ2">
+        <v>58.9</v>
+      </c>
+      <c r="BR2">
+        <v>52.5</v>
+      </c>
+      <c r="BS2">
+        <v>-8.699999999999999</v>
+      </c>
+      <c r="BT2">
+        <v>0</v>
+      </c>
+      <c r="BU2">
+        <v>89.5</v>
+      </c>
+      <c r="BV2">
+        <v>68.3</v>
+      </c>
+      <c r="BW2">
+        <v>51.4</v>
+      </c>
+      <c r="BX2">
+        <v>1012.2</v>
+      </c>
+      <c r="BY2">
+        <v>0</v>
+      </c>
+      <c r="BZ2">
+        <v>0</v>
+      </c>
+      <c r="CA2">
+        <v>9</v>
+      </c>
+      <c r="CB2">
+        <v>19.4</v>
+      </c>
+      <c r="CC2" t="s">
+        <v>188</v>
+      </c>
+      <c r="CD2">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="CE2">
         <v>8.5</v>
       </c>
-      <c r="Q2" s="1">
-        <v>88.40000000000001</v>
-      </c>
-      <c r="R2">
-        <v>85.5</v>
-      </c>
-      <c r="S2">
-        <v>92.40000000000001</v>
-      </c>
-      <c r="T2">
+      <c r="CF2">
         <v>5.8</v>
       </c>
-      <c r="U2" s="2">
-        <v>1.092</v>
-      </c>
-      <c r="V2" t="s">
-        <v>165</v>
-      </c>
-      <c r="W2">
-        <v>45.9</v>
-      </c>
-      <c r="X2">
+      <c r="CG2">
+        <v>1.1457</v>
+      </c>
+      <c r="CH2">
+        <v>2045</v>
+      </c>
+      <c r="CI2">
+        <v>90.09999999999999</v>
+      </c>
+      <c r="CJ2">
+        <v>1.096</v>
+      </c>
+      <c r="CK2">
+        <v>87.5</v>
+      </c>
+      <c r="CL2">
+        <v>89.90000000000001</v>
+      </c>
+      <c r="CM2">
+        <v>86.7</v>
+      </c>
+      <c r="CN2">
+        <v>91.5</v>
+      </c>
+      <c r="CO2">
+        <v>5.3</v>
+      </c>
+      <c r="CP2">
+        <v>10.4</v>
+      </c>
+      <c r="CQ2" t="s">
+        <v>180</v>
+      </c>
+      <c r="CR2">
+        <v>85.7</v>
+      </c>
+      <c r="CS2">
+        <v>66.90000000000001</v>
+      </c>
+      <c r="CT2">
+        <v>55.3</v>
+      </c>
+      <c r="CU2">
+        <v>1012.1</v>
+      </c>
+      <c r="CV2">
+        <v>0</v>
+      </c>
+      <c r="CW2">
+        <v>0</v>
+      </c>
+      <c r="CX2">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="CY2">
+        <v>17.5</v>
+      </c>
+      <c r="CZ2" t="s">
+        <v>188</v>
+      </c>
+      <c r="DA2">
+        <v>8.5</v>
+      </c>
+      <c r="DB2">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="DC2">
+        <v>5.7</v>
+      </c>
+      <c r="DD2">
+        <v>1.1539</v>
+      </c>
+      <c r="DE2">
+        <v>1802</v>
+      </c>
+      <c r="DF2">
+        <v>87.2</v>
+      </c>
+      <c r="DG2">
+        <v>1.089</v>
+      </c>
+      <c r="DH2">
+        <v>84.59999999999999</v>
+      </c>
+      <c r="DI2">
+        <v>87</v>
+      </c>
+      <c r="DJ2">
+        <v>84</v>
+      </c>
+      <c r="DK2">
+        <v>91.40000000000001</v>
+      </c>
+      <c r="DL2">
+        <v>5.7</v>
+      </c>
+      <c r="DM2">
+        <v>7.4</v>
+      </c>
+      <c r="DN2" t="s">
+        <v>180</v>
+      </c>
+      <c r="DO2">
+        <v>83.3</v>
+      </c>
+      <c r="DP2">
+        <v>66.8</v>
+      </c>
+      <c r="DQ2">
+        <v>59.7</v>
+      </c>
+      <c r="DR2">
+        <v>1012.3</v>
+      </c>
+      <c r="DS2">
+        <v>0.3</v>
+      </c>
+      <c r="DT2">
+        <v>0</v>
+      </c>
+      <c r="DU2">
+        <v>8.9</v>
+      </c>
+      <c r="DV2">
+        <v>17.5</v>
+      </c>
+      <c r="DW2" t="s">
+        <v>188</v>
+      </c>
+      <c r="DX2">
+        <v>8.6</v>
+      </c>
+      <c r="DY2">
+        <v>8.4</v>
+      </c>
+      <c r="DZ2">
+        <v>5.7</v>
+      </c>
+      <c r="EA2">
+        <v>1.1593</v>
+      </c>
+      <c r="EB2">
+        <v>1637</v>
+      </c>
+      <c r="EC2">
+        <v>85.90000000000001</v>
+      </c>
+      <c r="ED2">
+        <v>1.086</v>
+      </c>
+      <c r="EE2">
+        <v>83.3</v>
+      </c>
+      <c r="EF2">
+        <v>85.7</v>
+      </c>
+      <c r="EG2">
+        <v>82.2</v>
+      </c>
+      <c r="EH2">
+        <v>89.5</v>
+      </c>
+      <c r="EI2">
+        <v>8.5</v>
+      </c>
+      <c r="EJ2">
+        <v>6.8</v>
+      </c>
+      <c r="EK2" t="s">
+        <v>180</v>
+      </c>
+      <c r="EL2">
+        <v>80.8</v>
+      </c>
+      <c r="EM2">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="EN2">
+        <v>63.3</v>
+      </c>
+      <c r="EO2">
+        <v>1012.2</v>
+      </c>
+      <c r="EP2">
+        <v>1</v>
+      </c>
+      <c r="EQ2">
+        <v>0</v>
+      </c>
+      <c r="ER2">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="ES2">
+        <v>16.8</v>
+      </c>
+      <c r="ET2" t="s">
+        <v>188</v>
+      </c>
+      <c r="EU2">
+        <v>8.5</v>
+      </c>
+      <c r="EV2">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="EW2">
+        <v>5.7</v>
+      </c>
+      <c r="EX2">
+        <v>1.1648</v>
+      </c>
+      <c r="EY2">
+        <v>1472</v>
+      </c>
+      <c r="EZ2">
+        <v>84</v>
+      </c>
+      <c r="FA2">
+        <v>1.082</v>
+      </c>
+      <c r="FB2">
+        <v>81.5</v>
+      </c>
+      <c r="FC2">
+        <v>83.8</v>
+      </c>
+      <c r="FD2">
+        <v>80.2</v>
+      </c>
+      <c r="FE2">
+        <v>88.59999999999999</v>
+      </c>
+      <c r="FF2">
+        <v>11.7</v>
+      </c>
+      <c r="FG2">
         <v>5</v>
       </c>
-      <c r="Y2" s="1">
-        <v>85.7</v>
-      </c>
-      <c r="Z2" s="1">
-        <v>88.2</v>
-      </c>
-      <c r="AA2">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="AB2">
-        <v>1867</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>166</v>
-      </c>
-      <c r="AD2">
-        <v>10.4</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>166</v>
-      </c>
-      <c r="AF2">
-        <v>9.6</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>167</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>168</v>
-      </c>
-      <c r="AI2" t="s">
-        <v>160</v>
-      </c>
-      <c r="AJ2" t="s">
-        <v>169</v>
-      </c>
-      <c r="AK2">
-        <v>39.9061</v>
-      </c>
-      <c r="AL2">
-        <v>-75.1665</v>
-      </c>
-      <c r="AM2">
-        <v>20</v>
-      </c>
-      <c r="AN2">
-        <v>60</v>
-      </c>
-      <c r="AO2" t="s">
-        <v>170</v>
-      </c>
-      <c r="AP2" t="s">
-        <v>171</v>
-      </c>
-      <c r="AQ2" t="s">
-        <v>172</v>
-      </c>
-      <c r="AR2" t="s">
-        <v>173</v>
-      </c>
-      <c r="AS2">
-        <v>0.98</v>
-      </c>
-      <c r="AT2">
-        <v>0.7</v>
-      </c>
-      <c r="AU2">
-        <v>1.6</v>
-      </c>
-      <c r="AV2">
-        <v>86.7</v>
-      </c>
-      <c r="AW2">
-        <v>67.90000000000001</v>
-      </c>
-      <c r="AX2">
-        <v>55.4</v>
-      </c>
-      <c r="AY2">
-        <v>1012.2</v>
-      </c>
-      <c r="AZ2">
-        <v>9</v>
-      </c>
-      <c r="BA2">
-        <v>19.1</v>
-      </c>
-      <c r="BB2">
-        <v>8.5</v>
-      </c>
-      <c r="BC2">
-        <v>5.8</v>
-      </c>
-      <c r="BD2">
-        <v>1.1515</v>
-      </c>
-      <c r="BE2">
-        <v>59.8</v>
-      </c>
-      <c r="BF2">
-        <v>59.1</v>
-      </c>
-      <c r="BG2">
-        <v>51.2</v>
-      </c>
-      <c r="BH2">
-        <v>-8.4</v>
-      </c>
-      <c r="BI2">
-        <v>0</v>
-      </c>
-      <c r="BJ2">
-        <v>89.8</v>
-      </c>
-      <c r="BK2">
-        <v>68.7</v>
-      </c>
-      <c r="BL2">
-        <v>51.4</v>
-      </c>
-      <c r="BM2">
-        <v>1012.2</v>
-      </c>
-      <c r="BN2">
-        <v>0</v>
-      </c>
-      <c r="BO2">
-        <v>0</v>
-      </c>
-      <c r="BP2">
-        <v>9.1</v>
-      </c>
-      <c r="BQ2">
-        <v>18.7</v>
-      </c>
-      <c r="BR2" t="s">
-        <v>174</v>
-      </c>
-      <c r="BS2">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="BT2">
-        <v>8.5</v>
-      </c>
-      <c r="BU2">
-        <v>5.8</v>
-      </c>
-      <c r="BV2">
-        <v>1.1448</v>
-      </c>
-      <c r="BW2">
-        <v>2070</v>
-      </c>
-      <c r="BX2">
-        <v>90.40000000000001</v>
-      </c>
-      <c r="BY2">
-        <v>1.097</v>
-      </c>
-      <c r="BZ2">
-        <v>87.7</v>
-      </c>
-      <c r="CA2">
-        <v>90.2</v>
-      </c>
-      <c r="CB2">
-        <v>87</v>
-      </c>
-      <c r="CC2">
-        <v>91.7</v>
-      </c>
-      <c r="CD2">
-        <v>6.8</v>
-      </c>
-      <c r="CE2">
-        <v>10.4</v>
-      </c>
-      <c r="CF2" t="s">
-        <v>166</v>
-      </c>
-      <c r="CG2">
-        <v>86.3</v>
-      </c>
-      <c r="CH2">
-        <v>67.5</v>
-      </c>
-      <c r="CI2">
-        <v>55.3</v>
-      </c>
-      <c r="CJ2">
-        <v>1012.1</v>
-      </c>
-      <c r="CK2">
-        <v>0</v>
-      </c>
-      <c r="CL2">
-        <v>0</v>
-      </c>
-      <c r="CM2">
-        <v>8.9</v>
-      </c>
-      <c r="CN2">
-        <v>19.1</v>
-      </c>
-      <c r="CO2" t="s">
-        <v>174</v>
-      </c>
-      <c r="CP2">
-        <v>8.6</v>
-      </c>
-      <c r="CQ2">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="CR2">
-        <v>5.7</v>
-      </c>
-      <c r="CS2">
-        <v>1.1526</v>
-      </c>
-      <c r="CT2">
-        <v>1838</v>
-      </c>
-      <c r="CU2">
-        <v>87.90000000000001</v>
-      </c>
-      <c r="CV2">
-        <v>1.091</v>
-      </c>
-      <c r="CW2">
-        <v>85.3</v>
-      </c>
-      <c r="CX2">
-        <v>87.7</v>
-      </c>
-      <c r="CY2">
-        <v>85.2</v>
-      </c>
-      <c r="CZ2">
-        <v>92.90000000000001</v>
-      </c>
-      <c r="DA2">
-        <v>5</v>
-      </c>
-      <c r="DB2">
-        <v>7.4</v>
-      </c>
-      <c r="DC2" t="s">
-        <v>166</v>
-      </c>
-      <c r="DD2">
-        <v>83.90000000000001</v>
-      </c>
-      <c r="DE2">
-        <v>67.5</v>
-      </c>
-      <c r="DF2">
-        <v>59.7</v>
-      </c>
-      <c r="DG2">
-        <v>1012.3</v>
-      </c>
-      <c r="DH2">
-        <v>0.3</v>
-      </c>
-      <c r="DI2">
-        <v>0</v>
-      </c>
-      <c r="DJ2">
-        <v>9.1</v>
-      </c>
-      <c r="DK2">
-        <v>17.8</v>
-      </c>
-      <c r="DL2" t="s">
-        <v>174</v>
-      </c>
-      <c r="DM2">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="DN2">
-        <v>8.6</v>
-      </c>
-      <c r="DO2">
-        <v>5.9</v>
-      </c>
-      <c r="DP2">
-        <v>1.1576</v>
-      </c>
-      <c r="DQ2">
-        <v>1679</v>
-      </c>
-      <c r="DR2">
-        <v>86.8</v>
-      </c>
-      <c r="DS2">
-        <v>1.088</v>
-      </c>
-      <c r="DT2">
-        <v>84.2</v>
-      </c>
-      <c r="DU2">
-        <v>86.59999999999999</v>
-      </c>
-      <c r="DV2">
-        <v>84.3</v>
-      </c>
-      <c r="DW2">
-        <v>93</v>
-      </c>
-      <c r="DX2">
-        <v>4.3</v>
-      </c>
-      <c r="DY2">
-        <v>6.8</v>
-      </c>
-      <c r="DZ2" t="s">
-        <v>166</v>
-      </c>
-      <c r="EA2">
-        <v>81.40000000000001</v>
-      </c>
-      <c r="EB2">
-        <v>67.09999999999999</v>
-      </c>
-      <c r="EC2">
-        <v>63.3</v>
-      </c>
-      <c r="ED2">
-        <v>1012.2</v>
-      </c>
-      <c r="EE2">
-        <v>1</v>
-      </c>
-      <c r="EF2">
-        <v>0</v>
-      </c>
-      <c r="EG2">
-        <v>9</v>
-      </c>
-      <c r="EH2">
-        <v>16.8</v>
-      </c>
-      <c r="EI2" t="s">
-        <v>174</v>
-      </c>
-      <c r="EJ2">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="EK2">
-        <v>8.5</v>
-      </c>
-      <c r="EL2">
-        <v>5.8</v>
-      </c>
-      <c r="EM2">
-        <v>1.1631</v>
-      </c>
-      <c r="EN2">
-        <v>1517</v>
-      </c>
-      <c r="EO2">
-        <v>84.90000000000001</v>
-      </c>
-      <c r="EP2">
-        <v>1.084</v>
-      </c>
-      <c r="EQ2">
-        <v>82.3</v>
-      </c>
-      <c r="ER2">
-        <v>84.7</v>
-      </c>
-      <c r="ES2">
-        <v>82.3</v>
-      </c>
-      <c r="ET2">
-        <v>92.40000000000001</v>
-      </c>
-      <c r="EU2">
-        <v>7.2</v>
-      </c>
-      <c r="EV2">
-        <v>5</v>
-      </c>
-      <c r="EW2" t="s">
-        <v>166</v>
-      </c>
-      <c r="EX2">
+      <c r="FH2" t="s">
+        <v>180</v>
+      </c>
+      <c r="FI2" t="s">
+        <v>189</v>
+      </c>
+      <c r="FJ2">
+        <v>100</v>
+      </c>
+      <c r="FK2">
         <v>100</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:EX2"/>
+  <autoFilter ref="A1:FK2"/>
   <conditionalFormatting sqref="C2">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>OR(ISNUMBER(SEARCH("Elite",$I2)),ISNUMBER(SEARCH("Excellent",$I2)),ISNUMBER(SEARCH("Very Good",$I2)),ISNUMBER(SEARCH("Good",$I2)))</formula>
@@ -2266,7 +2449,7 @@
   <sheetPr>
     <tabColor rgb="FF5B9BD5"/>
   </sheetPr>
-  <dimension ref="A1:BJ5"/>
+  <dimension ref="A1:BU5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
@@ -2283,50 +2466,58 @@
     <col min="14" max="14" width="23.7109375" customWidth="1"/>
     <col min="15" max="15" width="25.7109375" customWidth="1"/>
     <col min="16" max="16" width="28.7109375" customWidth="1"/>
-    <col min="17" max="17" width="22.7109375" customWidth="1"/>
-    <col min="18" max="18" width="28.7109375" customWidth="1"/>
-    <col min="19" max="19" width="20.7109375" customWidth="1"/>
-    <col min="20" max="20" width="27.7109375" customWidth="1"/>
-    <col min="21" max="21" width="17.7109375" customWidth="1"/>
-    <col min="22" max="22" width="25.7109375" customWidth="1"/>
-    <col min="23" max="23" width="12.7109375" customWidth="1"/>
-    <col min="24" max="24" width="10.7109375" customWidth="1"/>
-    <col min="25" max="25" width="14.7109375" customWidth="1"/>
-    <col min="26" max="26" width="13.7109375" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" customWidth="1"/>
+    <col min="17" max="17" width="27.7109375" customWidth="1"/>
+    <col min="18" max="19" width="28.7109375" customWidth="1"/>
+    <col min="20" max="22" width="26.7109375" customWidth="1"/>
+    <col min="23" max="23" width="24.7109375" customWidth="1"/>
+    <col min="24" max="24" width="25.7109375" customWidth="1"/>
+    <col min="25" max="25" width="28.7109375" customWidth="1"/>
+    <col min="26" max="26" width="23.7109375" customWidth="1"/>
+    <col min="27" max="27" width="28.7109375" customWidth="1"/>
     <col min="28" max="28" width="22.7109375" customWidth="1"/>
-    <col min="29" max="29" width="24.7109375" customWidth="1"/>
-    <col min="30" max="30" width="15.7109375" customWidth="1"/>
-    <col min="31" max="31" width="10.7109375" customWidth="1"/>
-    <col min="32" max="32" width="15.7109375" customWidth="1"/>
-    <col min="33" max="33" width="18.7109375" customWidth="1"/>
-    <col min="34" max="34" width="11.7109375" customWidth="1"/>
+    <col min="29" max="29" width="28.7109375" customWidth="1"/>
+    <col min="30" max="30" width="20.7109375" customWidth="1"/>
+    <col min="31" max="31" width="27.7109375" customWidth="1"/>
+    <col min="32" max="32" width="17.7109375" customWidth="1"/>
+    <col min="33" max="33" width="25.7109375" customWidth="1"/>
+    <col min="34" max="34" width="12.7109375" customWidth="1"/>
     <col min="35" max="35" width="10.7109375" customWidth="1"/>
-    <col min="36" max="36" width="15.7109375" customWidth="1"/>
-    <col min="37" max="37" width="11.7109375" customWidth="1"/>
-    <col min="38" max="38" width="19.7109375" customWidth="1"/>
-    <col min="39" max="41" width="20.7109375" customWidth="1"/>
-    <col min="42" max="42" width="15.7109375" customWidth="1"/>
-    <col min="43" max="44" width="19.7109375" customWidth="1"/>
-    <col min="45" max="45" width="21.7109375" customWidth="1"/>
-    <col min="46" max="46" width="13.7109375" customWidth="1"/>
+    <col min="36" max="36" width="14.7109375" customWidth="1"/>
+    <col min="37" max="37" width="13.7109375" customWidth="1"/>
+    <col min="38" max="38" width="10.7109375" customWidth="1"/>
+    <col min="39" max="39" width="22.7109375" customWidth="1"/>
+    <col min="40" max="40" width="24.7109375" customWidth="1"/>
+    <col min="41" max="41" width="15.7109375" customWidth="1"/>
+    <col min="42" max="42" width="10.7109375" customWidth="1"/>
+    <col min="43" max="43" width="15.7109375" customWidth="1"/>
+    <col min="44" max="44" width="18.7109375" customWidth="1"/>
+    <col min="45" max="45" width="11.7109375" customWidth="1"/>
+    <col min="46" max="46" width="10.7109375" customWidth="1"/>
     <col min="47" max="47" width="15.7109375" customWidth="1"/>
-    <col min="48" max="48" width="16.7109375" customWidth="1"/>
-    <col min="49" max="49" width="18.7109375" customWidth="1"/>
-    <col min="50" max="51" width="17.7109375" customWidth="1"/>
-    <col min="52" max="52" width="11.7109375" customWidth="1"/>
-    <col min="53" max="53" width="23.7109375" customWidth="1"/>
-    <col min="54" max="54" width="24.7109375" customWidth="1"/>
-    <col min="55" max="55" width="18.7109375" customWidth="1"/>
-    <col min="56" max="56" width="12.7109375" customWidth="1"/>
-    <col min="57" max="57" width="28.7109375" customWidth="1"/>
-    <col min="58" max="58" width="22.7109375" customWidth="1"/>
-    <col min="59" max="59" width="12.7109375" customWidth="1"/>
-    <col min="60" max="61" width="14.7109375" customWidth="1"/>
-    <col min="62" max="62" width="16.7109375" customWidth="1"/>
+    <col min="48" max="48" width="11.7109375" customWidth="1"/>
+    <col min="49" max="49" width="19.7109375" customWidth="1"/>
+    <col min="50" max="52" width="20.7109375" customWidth="1"/>
+    <col min="53" max="53" width="15.7109375" customWidth="1"/>
+    <col min="54" max="55" width="19.7109375" customWidth="1"/>
+    <col min="56" max="56" width="21.7109375" customWidth="1"/>
+    <col min="57" max="57" width="13.7109375" customWidth="1"/>
+    <col min="58" max="58" width="15.7109375" customWidth="1"/>
+    <col min="59" max="59" width="16.7109375" customWidth="1"/>
+    <col min="60" max="60" width="18.7109375" customWidth="1"/>
+    <col min="61" max="62" width="17.7109375" customWidth="1"/>
+    <col min="63" max="63" width="11.7109375" customWidth="1"/>
+    <col min="64" max="64" width="23.7109375" customWidth="1"/>
+    <col min="65" max="65" width="24.7109375" customWidth="1"/>
+    <col min="66" max="66" width="18.7109375" customWidth="1"/>
+    <col min="67" max="67" width="12.7109375" customWidth="1"/>
+    <col min="68" max="68" width="28.7109375" customWidth="1"/>
+    <col min="69" max="69" width="22.7109375" customWidth="1"/>
+    <col min="70" max="70" width="12.7109375" customWidth="1"/>
+    <col min="71" max="72" width="14.7109375" customWidth="1"/>
+    <col min="73" max="73" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:62" ht="34" customHeight="1">
+    <row r="1" spans="1:73" ht="34" customHeight="1">
       <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
@@ -2340,934 +2531,1099 @@
         <v>6</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>176</v>
+        <v>191</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="W1" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="X1" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="Y1" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="Z1" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="AA1" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="AB1" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="AC1" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="AD1" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="AE1" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF1" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="AG1" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="AH1" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="AI1" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="AJ1" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="AK1" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="AL1" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="AM1" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="AN1" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="AO1" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="AP1" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="AQ1" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="AR1" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="AS1" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="AT1" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="AU1" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="AV1" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="AW1" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="AX1" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="AY1" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="AZ1" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="BA1" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="BB1" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="BC1" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="BD1" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="BE1" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="BF1" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="BG1" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="BH1" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="BI1" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="BJ1" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="BK1" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="BL1" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="BM1" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="BN1" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="BO1" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="BP1" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="N1" s="3" t="s">
+      <c r="BQ1" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="BR1" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="BS1" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="BT1" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="BU1" s="3" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="2" spans="1:73">
+      <c r="A2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C2" t="s">
+        <v>170</v>
+      </c>
+      <c r="D2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E2" t="s">
+        <v>249</v>
+      </c>
+      <c r="F2" t="s">
+        <v>172</v>
+      </c>
+      <c r="G2" t="s">
+        <v>186</v>
+      </c>
+      <c r="H2" t="s">
         <v>179</v>
       </c>
-      <c r="O1" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="R1" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="U1" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="V1" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="W1" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="X1" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="Y1" s="3" t="s">
+      <c r="I2" t="s">
         <v>187</v>
       </c>
-      <c r="Z1" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="AA1" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="AB1" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="AC1" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="AD1" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="AE1" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="AF1" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="AG1" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="AH1" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="AI1" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="AJ1" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="AK1" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="AL1" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="AM1" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="AN1" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="AO1" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="AP1" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="AQ1" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="AR1" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="AS1" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="AT1" s="3" t="s">
-        <v>208</v>
-      </c>
-      <c r="AU1" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="AV1" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="AW1" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="AX1" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="AY1" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="AZ1" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="BA1" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="BB1" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="BC1" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="BD1" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="BE1" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="BF1" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="BG1" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="BH1" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="BI1" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="BJ1" s="3" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="2" spans="1:62">
-      <c r="A2" t="s">
-        <v>155</v>
-      </c>
-      <c r="B2" t="s">
-        <v>156</v>
-      </c>
-      <c r="C2" t="s">
-        <v>157</v>
-      </c>
-      <c r="D2" t="s">
-        <v>160</v>
-      </c>
-      <c r="E2" t="s">
-        <v>223</v>
-      </c>
-      <c r="F2" t="s">
-        <v>159</v>
-      </c>
-      <c r="G2" t="s">
-        <v>172</v>
-      </c>
-      <c r="H2" t="s">
-        <v>165</v>
-      </c>
-      <c r="I2" t="s">
-        <v>173</v>
-      </c>
       <c r="J2">
-        <v>45.9</v>
+        <v>53.3</v>
       </c>
       <c r="K2">
-        <v>4.6</v>
+        <v>4.4</v>
       </c>
       <c r="L2">
         <v>5</v>
       </c>
       <c r="M2">
-        <v>1.31</v>
+        <v>0.9</v>
       </c>
       <c r="N2">
-        <v>0.53</v>
+        <v>0.57</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>6.8</v>
+        <v>1.2</v>
       </c>
       <c r="Q2">
-        <v>91.7</v>
+        <v>0.5</v>
       </c>
       <c r="R2">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="S2">
+        <v>0</v>
+      </c>
+      <c r="T2" t="s">
+        <v>256</v>
+      </c>
+      <c r="U2" t="s">
+        <v>257</v>
+      </c>
+      <c r="V2" t="s">
+        <v>258</v>
+      </c>
+      <c r="W2">
+        <v>1</v>
+      </c>
+      <c r="X2">
+        <v>0.478</v>
+      </c>
+      <c r="Y2">
+        <v>0.15</v>
+      </c>
+      <c r="Z2">
+        <v>0.12</v>
+      </c>
+      <c r="AA2">
+        <v>5.3</v>
+      </c>
+      <c r="AB2">
+        <v>91.5</v>
+      </c>
+      <c r="AC2">
+        <v>86.7</v>
+      </c>
+      <c r="AD2">
         <v>0.98</v>
       </c>
-      <c r="T2">
+      <c r="AE2">
         <v>0.7</v>
       </c>
-      <c r="U2">
+      <c r="AF2">
         <v>1.6</v>
       </c>
-      <c r="V2">
+      <c r="AG2">
         <v>1.6</v>
       </c>
-      <c r="W2" t="s">
-        <v>171</v>
-      </c>
-      <c r="X2">
-        <v>89.8</v>
-      </c>
-      <c r="Y2">
-        <v>92.59999999999999</v>
-      </c>
-      <c r="Z2">
-        <v>68.7</v>
-      </c>
-      <c r="AA2">
+      <c r="AH2" t="s">
+        <v>185</v>
+      </c>
+      <c r="AI2">
+        <v>89.5</v>
+      </c>
+      <c r="AJ2">
+        <v>91</v>
+      </c>
+      <c r="AK2">
+        <v>68.3</v>
+      </c>
+      <c r="AL2">
         <v>51.4</v>
       </c>
-      <c r="AB2">
+      <c r="AM2">
         <v>1012.2</v>
       </c>
-      <c r="AC2">
+      <c r="AN2">
         <v>1014.5</v>
       </c>
-      <c r="AD2">
+      <c r="AO2">
         <v>0</v>
       </c>
-      <c r="AE2">
+      <c r="AP2">
         <v>0</v>
       </c>
-      <c r="AF2">
+      <c r="AQ2">
         <v>0</v>
       </c>
-      <c r="AG2">
-        <v>74</v>
-      </c>
-      <c r="AH2">
+      <c r="AR2">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="AS2">
         <v>1042</v>
       </c>
-      <c r="AI2">
-        <v>9.1</v>
-      </c>
-      <c r="AJ2">
-        <v>18.7</v>
-      </c>
-      <c r="AK2" t="s">
-        <v>174</v>
-      </c>
-      <c r="AL2">
+      <c r="AT2">
+        <v>9</v>
+      </c>
+      <c r="AU2">
+        <v>19.4</v>
+      </c>
+      <c r="AV2" t="s">
+        <v>188</v>
+      </c>
+      <c r="AW2">
         <v>225</v>
       </c>
-      <c r="AM2">
+      <c r="AX2">
         <v>8.699999999999999</v>
       </c>
-      <c r="AN2">
+      <c r="AY2">
         <v>8.5</v>
       </c>
-      <c r="AO2">
+      <c r="AZ2">
         <v>5.8</v>
       </c>
-      <c r="AP2">
+      <c r="BA2">
         <v>-2.3</v>
       </c>
-      <c r="AQ2">
-        <v>1.1448</v>
-      </c>
-      <c r="AR2" t="s">
-        <v>230</v>
-      </c>
-      <c r="AS2">
-        <v>2070</v>
-      </c>
-      <c r="AT2" t="s">
-        <v>167</v>
-      </c>
-      <c r="AU2" t="s">
+      <c r="BB2">
+        <v>1.1457</v>
+      </c>
+      <c r="BC2" t="s">
+        <v>262</v>
+      </c>
+      <c r="BD2">
+        <v>2045</v>
+      </c>
+      <c r="BE2" t="s">
+        <v>181</v>
+      </c>
+      <c r="BF2" t="s">
+        <v>182</v>
+      </c>
+      <c r="BG2">
+        <v>90.09999999999999</v>
+      </c>
+      <c r="BH2">
+        <v>1.096</v>
+      </c>
+      <c r="BI2">
+        <v>87.5</v>
+      </c>
+      <c r="BJ2">
+        <v>89.90000000000001</v>
+      </c>
+      <c r="BK2">
+        <v>60.3</v>
+      </c>
+      <c r="BL2">
+        <v>59.8</v>
+      </c>
+      <c r="BM2">
+        <v>47.2</v>
+      </c>
+      <c r="BN2">
+        <v>10.4</v>
+      </c>
+      <c r="BO2" t="s">
+        <v>180</v>
+      </c>
+      <c r="BP2">
+        <v>11.1</v>
+      </c>
+      <c r="BQ2" t="s">
+        <v>180</v>
+      </c>
+      <c r="BR2">
+        <v>91</v>
+      </c>
+      <c r="BS2">
+        <v>87.09999999999999</v>
+      </c>
+      <c r="BT2">
+        <v>10</v>
+      </c>
+      <c r="BU2">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:73">
+      <c r="A3" t="s">
         <v>168</v>
       </c>
-      <c r="AV2">
-        <v>90.40000000000001</v>
-      </c>
-      <c r="AW2">
-        <v>1.097</v>
-      </c>
-      <c r="AX2">
-        <v>87.7</v>
-      </c>
-      <c r="AY2">
-        <v>90.2</v>
-      </c>
-      <c r="AZ2">
-        <v>60.5</v>
-      </c>
-      <c r="BA2">
-        <v>59.9</v>
-      </c>
-      <c r="BB2">
-        <v>46.9</v>
-      </c>
-      <c r="BC2">
-        <v>10.4</v>
-      </c>
-      <c r="BD2" t="s">
-        <v>166</v>
-      </c>
-      <c r="BE2">
-        <v>9.6</v>
-      </c>
-      <c r="BF2" t="s">
-        <v>166</v>
-      </c>
-      <c r="BG2">
-        <v>91</v>
-      </c>
-      <c r="BH2">
-        <v>87.8</v>
-      </c>
-      <c r="BI2">
-        <v>10</v>
-      </c>
-      <c r="BJ2">
-        <v>8.6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:62">
-      <c r="A3" t="s">
-        <v>155</v>
-      </c>
       <c r="B3" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="C3" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="D3" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="E3" t="s">
-        <v>224</v>
+        <v>250</v>
       </c>
       <c r="F3" t="s">
-        <v>227</v>
+        <v>253</v>
       </c>
       <c r="G3" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="H3" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="I3" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="J3">
-        <v>45.9</v>
+        <v>53.3</v>
       </c>
       <c r="K3">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
       <c r="L3">
         <v>5</v>
       </c>
       <c r="M3">
-        <v>0.41</v>
+        <v>0.59</v>
       </c>
       <c r="N3">
-        <v>1.1</v>
+        <v>1.11</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>5</v>
+        <v>2.1</v>
       </c>
       <c r="Q3">
-        <v>92.90000000000001</v>
+        <v>1.1</v>
       </c>
       <c r="R3">
-        <v>85.2</v>
+        <v>100</v>
       </c>
       <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3" t="s">
+        <v>256</v>
+      </c>
+      <c r="U3" t="s">
+        <v>258</v>
+      </c>
+      <c r="V3" t="s">
+        <v>259</v>
+      </c>
+      <c r="W3">
+        <v>1</v>
+      </c>
+      <c r="X3">
+        <v>0.4047</v>
+      </c>
+      <c r="Y3">
+        <v>0.13</v>
+      </c>
+      <c r="Z3">
+        <v>0.1</v>
+      </c>
+      <c r="AA3">
+        <v>5.7</v>
+      </c>
+      <c r="AB3">
+        <v>91.40000000000001</v>
+      </c>
+      <c r="AC3">
+        <v>84</v>
+      </c>
+      <c r="AD3">
         <v>0.98</v>
       </c>
-      <c r="T3">
+      <c r="AE3">
         <v>0.7</v>
       </c>
-      <c r="U3">
+      <c r="AF3">
         <v>1.6</v>
       </c>
-      <c r="V3">
+      <c r="AG3">
         <v>1.6</v>
       </c>
-      <c r="W3" t="s">
-        <v>171</v>
-      </c>
-      <c r="X3">
-        <v>86.3</v>
-      </c>
-      <c r="Y3">
-        <v>87.90000000000001</v>
-      </c>
-      <c r="Z3">
-        <v>67.5</v>
-      </c>
-      <c r="AA3">
+      <c r="AH3" t="s">
+        <v>185</v>
+      </c>
+      <c r="AI3">
+        <v>85.7</v>
+      </c>
+      <c r="AJ3">
+        <v>85.5</v>
+      </c>
+      <c r="AK3">
+        <v>66.90000000000001</v>
+      </c>
+      <c r="AL3">
         <v>55.3</v>
       </c>
-      <c r="AB3">
+      <c r="AM3">
         <v>1012.1</v>
       </c>
-      <c r="AC3">
+      <c r="AN3">
         <v>1014.4</v>
       </c>
-      <c r="AD3">
+      <c r="AO3">
         <v>0</v>
       </c>
-      <c r="AE3">
+      <c r="AP3">
         <v>0</v>
       </c>
-      <c r="AF3">
+      <c r="AQ3">
         <v>0</v>
       </c>
-      <c r="AG3">
-        <v>67.7</v>
-      </c>
-      <c r="AH3">
+      <c r="AR3">
+        <v>60.8</v>
+      </c>
+      <c r="AS3">
         <v>743</v>
       </c>
-      <c r="AI3">
-        <v>8.9</v>
-      </c>
-      <c r="AJ3">
-        <v>19.1</v>
-      </c>
-      <c r="AK3" t="s">
-        <v>174</v>
-      </c>
-      <c r="AL3">
+      <c r="AT3">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="AU3">
+        <v>17.5</v>
+      </c>
+      <c r="AV3" t="s">
+        <v>188</v>
+      </c>
+      <c r="AW3">
         <v>225</v>
       </c>
-      <c r="AM3">
-        <v>8.6</v>
-      </c>
-      <c r="AN3">
+      <c r="AX3">
+        <v>8.5</v>
+      </c>
+      <c r="AY3">
         <v>8.300000000000001</v>
       </c>
-      <c r="AO3">
+      <c r="AZ3">
         <v>5.7</v>
       </c>
-      <c r="AP3">
+      <c r="BA3">
         <v>-2.3</v>
       </c>
-      <c r="AQ3">
-        <v>1.1526</v>
-      </c>
-      <c r="AR3" t="s">
-        <v>230</v>
-      </c>
-      <c r="AS3">
-        <v>1838</v>
-      </c>
-      <c r="AT3" t="s">
-        <v>167</v>
-      </c>
-      <c r="AU3" t="s">
+      <c r="BB3">
+        <v>1.1539</v>
+      </c>
+      <c r="BC3" t="s">
+        <v>262</v>
+      </c>
+      <c r="BD3">
+        <v>1802</v>
+      </c>
+      <c r="BE3" t="s">
+        <v>181</v>
+      </c>
+      <c r="BF3" t="s">
+        <v>182</v>
+      </c>
+      <c r="BG3">
+        <v>87.2</v>
+      </c>
+      <c r="BH3">
+        <v>1.089</v>
+      </c>
+      <c r="BI3">
+        <v>84.59999999999999</v>
+      </c>
+      <c r="BJ3">
+        <v>87</v>
+      </c>
+      <c r="BK3">
+        <v>59.5</v>
+      </c>
+      <c r="BL3">
+        <v>58.7</v>
+      </c>
+      <c r="BM3">
+        <v>54</v>
+      </c>
+      <c r="BN3">
+        <v>7.4</v>
+      </c>
+      <c r="BO3" t="s">
+        <v>180</v>
+      </c>
+      <c r="BP3">
+        <v>10.9</v>
+      </c>
+      <c r="BQ3" t="s">
+        <v>180</v>
+      </c>
+      <c r="BR3">
+        <v>87</v>
+      </c>
+      <c r="BS3">
+        <v>83.59999999999999</v>
+      </c>
+      <c r="BT3">
+        <v>10</v>
+      </c>
+      <c r="BU3">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:73">
+      <c r="A4" t="s">
         <v>168</v>
       </c>
-      <c r="AV3">
-        <v>87.90000000000001</v>
-      </c>
-      <c r="AW3">
-        <v>1.091</v>
-      </c>
-      <c r="AX3">
-        <v>85.3</v>
-      </c>
-      <c r="AY3">
-        <v>87.7</v>
-      </c>
-      <c r="AZ3">
-        <v>59.6</v>
-      </c>
-      <c r="BA3">
-        <v>58.9</v>
-      </c>
-      <c r="BB3">
-        <v>51.6</v>
-      </c>
-      <c r="BC3">
-        <v>7.4</v>
-      </c>
-      <c r="BD3" t="s">
-        <v>166</v>
-      </c>
-      <c r="BE3">
-        <v>8.9</v>
-      </c>
-      <c r="BF3" t="s">
-        <v>166</v>
-      </c>
-      <c r="BG3">
-        <v>87</v>
-      </c>
-      <c r="BH3">
-        <v>84.5</v>
-      </c>
-      <c r="BI3">
-        <v>10</v>
-      </c>
-      <c r="BJ3">
-        <v>8.300000000000001</v>
-      </c>
-    </row>
-    <row r="4" spans="1:62">
-      <c r="A4" t="s">
-        <v>155</v>
-      </c>
       <c r="B4" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="C4" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="D4" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="E4" t="s">
-        <v>225</v>
+        <v>251</v>
       </c>
       <c r="F4" t="s">
-        <v>228</v>
+        <v>254</v>
       </c>
       <c r="G4" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="H4" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="I4" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="J4">
-        <v>45.9</v>
+        <v>53.3</v>
       </c>
       <c r="K4">
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>0.3</v>
+        <v>1.27</v>
       </c>
       <c r="N4">
-        <v>1.04</v>
+        <v>1.14</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>4.3</v>
+        <v>3.5</v>
       </c>
       <c r="Q4">
-        <v>93</v>
+        <v>1.2</v>
       </c>
       <c r="R4">
-        <v>84.3</v>
+        <v>100</v>
       </c>
       <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4" t="s">
+        <v>256</v>
+      </c>
+      <c r="U4" t="s">
+        <v>259</v>
+      </c>
+      <c r="V4" t="s">
+        <v>260</v>
+      </c>
+      <c r="W4">
+        <v>1</v>
+      </c>
+      <c r="X4">
+        <v>0.3425</v>
+      </c>
+      <c r="Y4">
+        <v>0.11</v>
+      </c>
+      <c r="Z4">
+        <v>0.08</v>
+      </c>
+      <c r="AA4">
+        <v>8.5</v>
+      </c>
+      <c r="AB4">
+        <v>89.5</v>
+      </c>
+      <c r="AC4">
+        <v>82.2</v>
+      </c>
+      <c r="AD4">
         <v>0.98</v>
       </c>
-      <c r="T4">
+      <c r="AE4">
         <v>0.7</v>
       </c>
-      <c r="U4">
+      <c r="AF4">
         <v>1.6</v>
       </c>
-      <c r="V4">
+      <c r="AG4">
         <v>1.6</v>
       </c>
-      <c r="W4" t="s">
-        <v>171</v>
-      </c>
-      <c r="X4">
-        <v>83.90000000000001</v>
-      </c>
-      <c r="Y4">
-        <v>85.2</v>
-      </c>
-      <c r="Z4">
-        <v>67.5</v>
-      </c>
-      <c r="AA4">
+      <c r="AH4" t="s">
+        <v>185</v>
+      </c>
+      <c r="AI4">
+        <v>83.3</v>
+      </c>
+      <c r="AJ4">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="AK4">
+        <v>66.8</v>
+      </c>
+      <c r="AL4">
         <v>59.7</v>
       </c>
-      <c r="AB4">
+      <c r="AM4">
         <v>1012.3</v>
       </c>
-      <c r="AC4">
+      <c r="AN4">
         <v>1014.5</v>
       </c>
-      <c r="AD4">
+      <c r="AO4">
         <v>0.3</v>
       </c>
-      <c r="AE4">
+      <c r="AP4">
         <v>0</v>
       </c>
-      <c r="AF4">
+      <c r="AQ4">
         <v>0</v>
       </c>
-      <c r="AG4">
-        <v>55.5</v>
-      </c>
-      <c r="AH4">
+      <c r="AR4">
+        <v>50.6</v>
+      </c>
+      <c r="AS4">
         <v>684</v>
       </c>
-      <c r="AI4">
-        <v>9.1</v>
-      </c>
-      <c r="AJ4">
-        <v>17.8</v>
-      </c>
-      <c r="AK4" t="s">
-        <v>174</v>
-      </c>
-      <c r="AL4">
+      <c r="AT4">
+        <v>8.9</v>
+      </c>
+      <c r="AU4">
+        <v>17.5</v>
+      </c>
+      <c r="AV4" t="s">
+        <v>188</v>
+      </c>
+      <c r="AW4">
         <v>225</v>
       </c>
-      <c r="AM4">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="AN4">
+      <c r="AX4">
         <v>8.6</v>
       </c>
-      <c r="AO4">
-        <v>5.9</v>
-      </c>
-      <c r="AP4">
-        <v>-2.4</v>
-      </c>
-      <c r="AQ4">
-        <v>1.1576</v>
-      </c>
-      <c r="AR4" t="s">
-        <v>230</v>
-      </c>
-      <c r="AS4">
-        <v>1679</v>
-      </c>
-      <c r="AT4" t="s">
-        <v>167</v>
-      </c>
-      <c r="AU4" t="s">
+      <c r="AY4">
+        <v>8.4</v>
+      </c>
+      <c r="AZ4">
+        <v>5.7</v>
+      </c>
+      <c r="BA4">
+        <v>-2.3</v>
+      </c>
+      <c r="BB4">
+        <v>1.1593</v>
+      </c>
+      <c r="BC4" t="s">
+        <v>262</v>
+      </c>
+      <c r="BD4">
+        <v>1637</v>
+      </c>
+      <c r="BE4" t="s">
+        <v>181</v>
+      </c>
+      <c r="BF4" t="s">
+        <v>182</v>
+      </c>
+      <c r="BG4">
+        <v>85.90000000000001</v>
+      </c>
+      <c r="BH4">
+        <v>1.086</v>
+      </c>
+      <c r="BI4">
+        <v>83.3</v>
+      </c>
+      <c r="BJ4">
+        <v>85.7</v>
+      </c>
+      <c r="BK4">
+        <v>59</v>
+      </c>
+      <c r="BL4">
+        <v>58.2</v>
+      </c>
+      <c r="BM4">
+        <v>56.8</v>
+      </c>
+      <c r="BN4">
+        <v>6.8</v>
+      </c>
+      <c r="BO4" t="s">
+        <v>180</v>
+      </c>
+      <c r="BP4">
+        <v>12.1</v>
+      </c>
+      <c r="BQ4" t="s">
+        <v>180</v>
+      </c>
+      <c r="BR4">
+        <v>85</v>
+      </c>
+      <c r="BS4">
+        <v>80.90000000000001</v>
+      </c>
+      <c r="BT4">
+        <v>10</v>
+      </c>
+      <c r="BU4">
+        <v>8.4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:73">
+      <c r="A5" t="s">
         <v>168</v>
       </c>
-      <c r="AV4">
-        <v>86.8</v>
-      </c>
-      <c r="AW4">
-        <v>1.088</v>
-      </c>
-      <c r="AX4">
-        <v>84.2</v>
-      </c>
-      <c r="AY4">
-        <v>86.59999999999999</v>
-      </c>
-      <c r="AZ4">
-        <v>59.3</v>
-      </c>
-      <c r="BA4">
-        <v>58.5</v>
-      </c>
-      <c r="BB4">
-        <v>55.2</v>
-      </c>
-      <c r="BC4">
-        <v>6.8</v>
-      </c>
-      <c r="BD4" t="s">
-        <v>166</v>
-      </c>
-      <c r="BE4">
-        <v>9.1</v>
-      </c>
-      <c r="BF4" t="s">
-        <v>166</v>
-      </c>
-      <c r="BG4">
-        <v>85</v>
-      </c>
-      <c r="BH4">
-        <v>82</v>
-      </c>
-      <c r="BI4">
-        <v>10</v>
-      </c>
-      <c r="BJ4">
-        <v>8.699999999999999</v>
-      </c>
-    </row>
-    <row r="5" spans="1:62">
-      <c r="A5" t="s">
-        <v>155</v>
-      </c>
       <c r="B5" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="C5" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="D5" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="E5" t="s">
-        <v>226</v>
+        <v>252</v>
       </c>
       <c r="F5" t="s">
-        <v>229</v>
+        <v>255</v>
       </c>
       <c r="G5" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="H5" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="I5" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="J5">
-        <v>45.9</v>
+        <v>53.3</v>
       </c>
       <c r="K5">
-        <v>7.6</v>
+        <v>7.4</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>0.93</v>
+        <v>1.96</v>
       </c>
       <c r="N5">
-        <v>1.16</v>
+        <v>1.3</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>7.2</v>
+        <v>5</v>
       </c>
       <c r="Q5">
-        <v>92.40000000000001</v>
+        <v>1.4</v>
       </c>
       <c r="R5">
-        <v>82.3</v>
+        <v>100</v>
       </c>
       <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5" t="s">
+        <v>256</v>
+      </c>
+      <c r="U5" t="s">
+        <v>260</v>
+      </c>
+      <c r="V5" t="s">
+        <v>261</v>
+      </c>
+      <c r="W5">
+        <v>1</v>
+      </c>
+      <c r="X5">
+        <v>0.29</v>
+      </c>
+      <c r="Y5">
+        <v>0.09</v>
+      </c>
+      <c r="Z5">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="AA5">
+        <v>11.7</v>
+      </c>
+      <c r="AB5">
+        <v>88.59999999999999</v>
+      </c>
+      <c r="AC5">
+        <v>80.2</v>
+      </c>
+      <c r="AD5">
         <v>0.98</v>
       </c>
-      <c r="T5">
+      <c r="AE5">
         <v>0.7</v>
       </c>
-      <c r="U5">
+      <c r="AF5">
         <v>1.6</v>
       </c>
-      <c r="V5">
+      <c r="AG5">
         <v>1.6</v>
       </c>
-      <c r="W5" t="s">
-        <v>171</v>
-      </c>
-      <c r="X5">
-        <v>81.40000000000001</v>
-      </c>
-      <c r="Y5">
-        <v>82.5</v>
-      </c>
-      <c r="Z5">
-        <v>67.09999999999999</v>
-      </c>
-      <c r="AA5">
+      <c r="AH5" t="s">
+        <v>185</v>
+      </c>
+      <c r="AI5">
+        <v>80.8</v>
+      </c>
+      <c r="AJ5">
+        <v>79.7</v>
+      </c>
+      <c r="AK5">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="AL5">
         <v>63.3</v>
       </c>
-      <c r="AB5">
+      <c r="AM5">
         <v>1012.2</v>
       </c>
-      <c r="AC5">
+      <c r="AN5">
         <v>1014.5</v>
       </c>
-      <c r="AD5">
+      <c r="AO5">
         <v>1</v>
       </c>
-      <c r="AE5">
+      <c r="AP5">
         <v>0</v>
       </c>
-      <c r="AF5">
+      <c r="AQ5">
         <v>0</v>
       </c>
-      <c r="AG5">
-        <v>49.1</v>
-      </c>
-      <c r="AH5">
+      <c r="AR5">
+        <v>43.6</v>
+      </c>
+      <c r="AS5">
         <v>504</v>
       </c>
-      <c r="AI5">
-        <v>9</v>
-      </c>
-      <c r="AJ5">
+      <c r="AT5">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="AU5">
         <v>16.8</v>
       </c>
-      <c r="AK5" t="s">
-        <v>174</v>
-      </c>
-      <c r="AL5">
+      <c r="AV5" t="s">
+        <v>188</v>
+      </c>
+      <c r="AW5">
         <v>225</v>
       </c>
-      <c r="AM5">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="AN5">
+      <c r="AX5">
         <v>8.5</v>
       </c>
-      <c r="AO5">
-        <v>5.8</v>
-      </c>
-      <c r="AP5">
+      <c r="AY5">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="AZ5">
+        <v>5.7</v>
+      </c>
+      <c r="BA5">
         <v>-2.3</v>
       </c>
-      <c r="AQ5">
-        <v>1.1631</v>
-      </c>
-      <c r="AR5" t="s">
-        <v>231</v>
-      </c>
-      <c r="AS5">
-        <v>1517</v>
-      </c>
-      <c r="AT5" t="s">
-        <v>167</v>
-      </c>
-      <c r="AU5" t="s">
-        <v>168</v>
-      </c>
-      <c r="AV5">
-        <v>84.90000000000001</v>
-      </c>
-      <c r="AW5">
-        <v>1.084</v>
-      </c>
-      <c r="AX5">
-        <v>82.3</v>
-      </c>
-      <c r="AY5">
-        <v>84.7</v>
-      </c>
-      <c r="AZ5">
-        <v>58.7</v>
-      </c>
-      <c r="BA5">
-        <v>57.9</v>
-      </c>
       <c r="BB5">
-        <v>59</v>
-      </c>
-      <c r="BC5">
+        <v>1.1648</v>
+      </c>
+      <c r="BC5" t="s">
+        <v>263</v>
+      </c>
+      <c r="BD5">
+        <v>1472</v>
+      </c>
+      <c r="BE5" t="s">
+        <v>181</v>
+      </c>
+      <c r="BF5" t="s">
+        <v>182</v>
+      </c>
+      <c r="BG5">
+        <v>84</v>
+      </c>
+      <c r="BH5">
+        <v>1.082</v>
+      </c>
+      <c r="BI5">
+        <v>81.5</v>
+      </c>
+      <c r="BJ5">
+        <v>83.8</v>
+      </c>
+      <c r="BK5">
+        <v>58.4</v>
+      </c>
+      <c r="BL5">
+        <v>57.5</v>
+      </c>
+      <c r="BM5">
+        <v>60.4</v>
+      </c>
+      <c r="BN5">
         <v>5</v>
       </c>
-      <c r="BD5" t="s">
-        <v>166</v>
-      </c>
-      <c r="BE5">
-        <v>7.9</v>
-      </c>
-      <c r="BF5" t="s">
-        <v>166</v>
-      </c>
-      <c r="BG5">
+      <c r="BO5" t="s">
+        <v>180</v>
+      </c>
+      <c r="BP5">
+        <v>11</v>
+      </c>
+      <c r="BQ5" t="s">
+        <v>180</v>
+      </c>
+      <c r="BR5">
         <v>82</v>
       </c>
-      <c r="BH5">
-        <v>79.8</v>
-      </c>
-      <c r="BI5">
+      <c r="BS5">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="BT5">
         <v>10</v>
       </c>
-      <c r="BJ5">
-        <v>8.5</v>
+      <c r="BU5">
+        <v>8.1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BJ5"/>
+  <autoFilter ref="A1:BU5"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3336,75 +3692,75 @@
         <v>18</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:18">
       <c r="A2" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="B2" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="C2" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
       <c r="D2" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="E2">
-        <v>88.40000000000001</v>
+        <v>87.8</v>
       </c>
       <c r="F2">
-        <v>85.5</v>
+        <v>84.3</v>
       </c>
       <c r="G2" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
       <c r="H2" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
       <c r="I2" s="4">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J2" s="5">
-        <v>8.5</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="K2" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="L2">
-        <v>92.40000000000001</v>
+        <v>90.8</v>
       </c>
       <c r="M2">
-        <v>8.699999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="N2">
-        <v>86.7</v>
+        <v>86.3</v>
       </c>
       <c r="O2">
-        <v>1867</v>
+        <v>1833</v>
       </c>
       <c r="P2" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="Q2" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="R2">
         <v>5</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 12:54 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_2026_07_14.xlsx
+++ b/mlb_weather_professional_2026_07_14.xlsx
@@ -560,7 +560,7 @@
     <t>STEADY</t>
   </si>
   <si>
-    <t>2026-07-14 12:34:18 PM PDT</t>
+    <t>2026-07-14 12:54:42 PM PDT</t>
   </si>
   <si>
     <t>LOW</t>
@@ -581,16 +581,16 @@
     <t>Clear</t>
   </si>
   <si>
+    <t>2026-07-14 19:54:42 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14T18:41:01+00:00</t>
+  </si>
+  <si>
+    <t>SW</t>
+  </si>
+  <si>
     <t>2026-07-14 19:34:18 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14T18:41:01+00:00</t>
-  </si>
-  <si>
-    <t>SW</t>
-  </si>
-  <si>
-    <t>2026-07-14 19:26:55 UTC</t>
   </si>
   <si>
     <t>Period</t>
@@ -1945,7 +1945,7 @@
         <v>175</v>
       </c>
       <c r="K2">
-        <v>87.8</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="L2">
         <v>84.3</v>
@@ -1963,16 +1963,16 @@
         <v>8.199999999999999</v>
       </c>
       <c r="Q2" s="1">
-        <v>87.8</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="R2">
         <v>84.3</v>
       </c>
       <c r="S2">
-        <v>90.8</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="T2">
-        <v>6.7</v>
+        <v>7.1</v>
       </c>
       <c r="U2" s="2">
         <v>1.091</v>
@@ -1981,13 +1981,13 @@
         <v>178</v>
       </c>
       <c r="W2">
-        <v>-1.2</v>
+        <v>0</v>
       </c>
       <c r="X2">
-        <v>86.3</v>
+        <v>-0.1</v>
       </c>
       <c r="Y2">
-        <v>-0.1</v>
+        <v>0</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -1999,49 +1999,49 @@
         <v>0</v>
       </c>
       <c r="AC2">
-        <v>2.3</v>
+        <v>4.2</v>
       </c>
       <c r="AD2">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="AE2">
-        <v>0.15</v>
+        <v>-0.05</v>
       </c>
       <c r="AF2">
-        <v>0.12</v>
+        <v>0.02</v>
       </c>
       <c r="AG2" t="s">
         <v>179</v>
       </c>
       <c r="AH2">
-        <v>53.3</v>
+        <v>73.7</v>
       </c>
       <c r="AI2">
         <v>5</v>
       </c>
       <c r="AJ2" s="1">
-        <v>85.2</v>
+        <v>85.3</v>
       </c>
       <c r="AK2" s="1">
-        <v>87.59999999999999</v>
+        <v>87.7</v>
       </c>
       <c r="AL2">
         <v>8.6</v>
       </c>
       <c r="AM2">
-        <v>1833</v>
+        <v>1832</v>
       </c>
       <c r="AN2" t="s">
         <v>180</v>
       </c>
       <c r="AO2">
-        <v>10.4</v>
+        <v>11.2</v>
       </c>
       <c r="AP2" t="s">
         <v>180</v>
       </c>
       <c r="AQ2">
-        <v>12.1</v>
+        <v>12</v>
       </c>
       <c r="AR2" t="s">
         <v>181</v>
@@ -2089,13 +2089,13 @@
         <v>1.6</v>
       </c>
       <c r="BG2">
-        <v>86.3</v>
+        <v>86.2</v>
       </c>
       <c r="BH2">
-        <v>67.40000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="BI2">
-        <v>55.4</v>
+        <v>56.1</v>
       </c>
       <c r="BJ2">
         <v>1012.2</v>
@@ -2110,34 +2110,34 @@
         <v>8.4</v>
       </c>
       <c r="BN2">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="BO2">
-        <v>1.1528</v>
+        <v>1.1527</v>
       </c>
       <c r="BP2">
         <v>59.6</v>
       </c>
       <c r="BQ2">
-        <v>58.9</v>
+        <v>59</v>
       </c>
       <c r="BR2">
-        <v>52.5</v>
+        <v>52</v>
       </c>
       <c r="BS2">
         <v>-8.699999999999999</v>
       </c>
       <c r="BT2">
-        <v>0</v>
+        <v>-0.1</v>
       </c>
       <c r="BU2">
-        <v>89.5</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="BV2">
-        <v>68.3</v>
+        <v>68.5</v>
       </c>
       <c r="BW2">
-        <v>51.4</v>
+        <v>51.8</v>
       </c>
       <c r="BX2">
         <v>1012.2</v>
@@ -2170,31 +2170,31 @@
         <v>1.1457</v>
       </c>
       <c r="CH2">
-        <v>2045</v>
+        <v>2042</v>
       </c>
       <c r="CI2">
-        <v>90.09999999999999</v>
+        <v>90.2</v>
       </c>
       <c r="CJ2">
         <v>1.096</v>
       </c>
       <c r="CK2">
-        <v>87.5</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="CL2">
-        <v>89.90000000000001</v>
+        <v>90</v>
       </c>
       <c r="CM2">
         <v>86.7</v>
       </c>
       <c r="CN2">
-        <v>91.5</v>
+        <v>91.3</v>
       </c>
       <c r="CO2">
-        <v>5.3</v>
+        <v>5.8</v>
       </c>
       <c r="CP2">
-        <v>10.4</v>
+        <v>11.2</v>
       </c>
       <c r="CQ2" t="s">
         <v>180</v>
@@ -2203,10 +2203,10 @@
         <v>85.7</v>
       </c>
       <c r="CS2">
-        <v>66.90000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="CT2">
-        <v>55.3</v>
+        <v>56.1</v>
       </c>
       <c r="CU2">
         <v>1012.1</v>
@@ -2221,7 +2221,7 @@
         <v>8.800000000000001</v>
       </c>
       <c r="CY2">
-        <v>17.5</v>
+        <v>17.7</v>
       </c>
       <c r="CZ2" t="s">
         <v>188</v>
@@ -2236,10 +2236,10 @@
         <v>5.7</v>
       </c>
       <c r="DD2">
-        <v>1.1539</v>
+        <v>1.1538</v>
       </c>
       <c r="DE2">
-        <v>1802</v>
+        <v>1801</v>
       </c>
       <c r="DF2">
         <v>87.2</v>
@@ -2257,13 +2257,13 @@
         <v>84</v>
       </c>
       <c r="DK2">
-        <v>91.40000000000001</v>
+        <v>91.3</v>
       </c>
       <c r="DL2">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="DM2">
-        <v>7.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="DN2" t="s">
         <v>180</v>
@@ -2272,25 +2272,25 @@
         <v>83.3</v>
       </c>
       <c r="DP2">
-        <v>66.8</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="DQ2">
-        <v>59.7</v>
+        <v>60.7</v>
       </c>
       <c r="DR2">
-        <v>1012.3</v>
+        <v>1012.2</v>
       </c>
       <c r="DS2">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="DT2">
         <v>0</v>
       </c>
       <c r="DU2">
-        <v>8.9</v>
+        <v>9</v>
       </c>
       <c r="DV2">
-        <v>17.5</v>
+        <v>17.7</v>
       </c>
       <c r="DW2" t="s">
         <v>188</v>
@@ -2302,55 +2302,55 @@
         <v>8.4</v>
       </c>
       <c r="DZ2">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="EA2">
-        <v>1.1593</v>
+        <v>1.1591</v>
       </c>
       <c r="EB2">
         <v>1637</v>
       </c>
       <c r="EC2">
+        <v>86.09999999999999</v>
+      </c>
+      <c r="ED2">
+        <v>1.087</v>
+      </c>
+      <c r="EE2">
+        <v>83.5</v>
+      </c>
+      <c r="EF2">
         <v>85.90000000000001</v>
-      </c>
-      <c r="ED2">
-        <v>1.086</v>
-      </c>
-      <c r="EE2">
-        <v>83.3</v>
-      </c>
-      <c r="EF2">
-        <v>85.7</v>
       </c>
       <c r="EG2">
         <v>82.2</v>
       </c>
       <c r="EH2">
-        <v>89.5</v>
+        <v>89.3</v>
       </c>
       <c r="EI2">
-        <v>8.5</v>
+        <v>9</v>
       </c>
       <c r="EJ2">
-        <v>6.8</v>
+        <v>7.8</v>
       </c>
       <c r="EK2" t="s">
         <v>180</v>
       </c>
       <c r="EL2">
-        <v>80.8</v>
+        <v>80.7</v>
       </c>
       <c r="EM2">
-        <v>66.40000000000001</v>
+        <v>67</v>
       </c>
       <c r="EN2">
-        <v>63.3</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="EO2">
-        <v>1012.2</v>
+        <v>1012.1</v>
       </c>
       <c r="EP2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="EQ2">
         <v>0</v>
@@ -2359,7 +2359,7 @@
         <v>8.800000000000001</v>
       </c>
       <c r="ES2">
-        <v>16.8</v>
+        <v>17</v>
       </c>
       <c r="ET2" t="s">
         <v>188</v>
@@ -2374,34 +2374,34 @@
         <v>5.7</v>
       </c>
       <c r="EX2">
-        <v>1.1648</v>
+        <v>1.1645</v>
       </c>
       <c r="EY2">
-        <v>1472</v>
+        <v>1474</v>
       </c>
       <c r="EZ2">
-        <v>84</v>
+        <v>84.2</v>
       </c>
       <c r="FA2">
         <v>1.082</v>
       </c>
       <c r="FB2">
-        <v>81.5</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="FC2">
-        <v>83.8</v>
+        <v>84</v>
       </c>
       <c r="FD2">
         <v>80.2</v>
       </c>
       <c r="FE2">
-        <v>88.59999999999999</v>
+        <v>88.5</v>
       </c>
       <c r="FF2">
-        <v>11.7</v>
+        <v>12.1</v>
       </c>
       <c r="FG2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="FH2" t="s">
         <v>180</v>
@@ -2410,7 +2410,7 @@
         <v>189</v>
       </c>
       <c r="FJ2">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="FK2">
         <v>100</v>
@@ -2767,28 +2767,28 @@
         <v>187</v>
       </c>
       <c r="J2">
-        <v>53.3</v>
+        <v>73.7</v>
       </c>
       <c r="K2">
-        <v>4.4</v>
+        <v>4.1</v>
       </c>
       <c r="L2">
         <v>5</v>
       </c>
       <c r="M2">
-        <v>0.9</v>
+        <v>0.96</v>
       </c>
       <c r="N2">
-        <v>0.57</v>
+        <v>0.66</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>1.2</v>
+        <v>2.2</v>
       </c>
       <c r="Q2">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="R2">
         <v>100</v>
@@ -2809,19 +2809,19 @@
         <v>1</v>
       </c>
       <c r="X2">
-        <v>0.478</v>
+        <v>0.5059</v>
       </c>
       <c r="Y2">
-        <v>0.15</v>
+        <v>-0.05</v>
       </c>
       <c r="Z2">
-        <v>0.12</v>
+        <v>0.02</v>
       </c>
       <c r="AA2">
-        <v>5.3</v>
+        <v>5.8</v>
       </c>
       <c r="AB2">
-        <v>91.5</v>
+        <v>91.3</v>
       </c>
       <c r="AC2">
         <v>86.7</v>
@@ -2842,16 +2842,16 @@
         <v>185</v>
       </c>
       <c r="AI2">
-        <v>89.5</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="AJ2">
         <v>91</v>
       </c>
       <c r="AK2">
-        <v>68.3</v>
+        <v>68.5</v>
       </c>
       <c r="AL2">
-        <v>51.4</v>
+        <v>51.8</v>
       </c>
       <c r="AM2">
         <v>1012.2</v>
@@ -2872,7 +2872,7 @@
         <v>71.40000000000001</v>
       </c>
       <c r="AS2">
-        <v>1042</v>
+        <v>1120</v>
       </c>
       <c r="AT2">
         <v>9</v>
@@ -2905,7 +2905,7 @@
         <v>262</v>
       </c>
       <c r="BD2">
-        <v>2045</v>
+        <v>2042</v>
       </c>
       <c r="BE2" t="s">
         <v>181</v>
@@ -2914,16 +2914,16 @@
         <v>182</v>
       </c>
       <c r="BG2">
-        <v>90.09999999999999</v>
+        <v>90.2</v>
       </c>
       <c r="BH2">
         <v>1.096</v>
       </c>
       <c r="BI2">
-        <v>87.5</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="BJ2">
-        <v>89.90000000000001</v>
+        <v>90</v>
       </c>
       <c r="BK2">
         <v>60.3</v>
@@ -2932,10 +2932,10 @@
         <v>59.8</v>
       </c>
       <c r="BM2">
-        <v>47.2</v>
+        <v>46.9</v>
       </c>
       <c r="BN2">
-        <v>10.4</v>
+        <v>11.2</v>
       </c>
       <c r="BO2" t="s">
         <v>180</v>
@@ -2956,7 +2956,7 @@
         <v>10</v>
       </c>
       <c r="BU2">
-        <v>8.5</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="3" spans="1:73">
@@ -2988,28 +2988,28 @@
         <v>187</v>
       </c>
       <c r="J3">
-        <v>53.3</v>
+        <v>73.7</v>
       </c>
       <c r="K3">
-        <v>5.4</v>
+        <v>5.1</v>
       </c>
       <c r="L3">
         <v>5</v>
       </c>
       <c r="M3">
-        <v>0.59</v>
+        <v>0.62</v>
       </c>
       <c r="N3">
-        <v>1.11</v>
+        <v>1.12</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>2.1</v>
+        <v>4.2</v>
       </c>
       <c r="Q3">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="R3">
         <v>100</v>
@@ -3030,19 +3030,19 @@
         <v>1</v>
       </c>
       <c r="X3">
-        <v>0.4047</v>
+        <v>0.4282</v>
       </c>
       <c r="Y3">
-        <v>0.13</v>
+        <v>-0.04</v>
       </c>
       <c r="Z3">
-        <v>0.1</v>
+        <v>0.01</v>
       </c>
       <c r="AA3">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="AB3">
-        <v>91.40000000000001</v>
+        <v>91.3</v>
       </c>
       <c r="AC3">
         <v>84</v>
@@ -3069,10 +3069,10 @@
         <v>85.5</v>
       </c>
       <c r="AK3">
-        <v>66.90000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="AL3">
-        <v>55.3</v>
+        <v>56.1</v>
       </c>
       <c r="AM3">
         <v>1012.1</v>
@@ -3093,13 +3093,13 @@
         <v>60.8</v>
       </c>
       <c r="AS3">
-        <v>743</v>
+        <v>825</v>
       </c>
       <c r="AT3">
         <v>8.800000000000001</v>
       </c>
       <c r="AU3">
-        <v>17.5</v>
+        <v>17.7</v>
       </c>
       <c r="AV3" t="s">
         <v>188</v>
@@ -3120,13 +3120,13 @@
         <v>-2.3</v>
       </c>
       <c r="BB3">
-        <v>1.1539</v>
+        <v>1.1538</v>
       </c>
       <c r="BC3" t="s">
         <v>262</v>
       </c>
       <c r="BD3">
-        <v>1802</v>
+        <v>1801</v>
       </c>
       <c r="BE3" t="s">
         <v>181</v>
@@ -3147,22 +3147,22 @@
         <v>87</v>
       </c>
       <c r="BK3">
-        <v>59.5</v>
+        <v>59.4</v>
       </c>
       <c r="BL3">
         <v>58.7</v>
       </c>
       <c r="BM3">
-        <v>54</v>
+        <v>53.6</v>
       </c>
       <c r="BN3">
-        <v>7.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="BO3" t="s">
         <v>180</v>
       </c>
       <c r="BP3">
-        <v>10.9</v>
+        <v>11</v>
       </c>
       <c r="BQ3" t="s">
         <v>180</v>
@@ -3171,7 +3171,7 @@
         <v>87</v>
       </c>
       <c r="BS3">
-        <v>83.59999999999999</v>
+        <v>83.5</v>
       </c>
       <c r="BT3">
         <v>10</v>
@@ -3209,28 +3209,28 @@
         <v>187</v>
       </c>
       <c r="J4">
-        <v>53.3</v>
+        <v>73.7</v>
       </c>
       <c r="K4">
-        <v>6.4</v>
+        <v>6.1</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>1.27</v>
+        <v>1.28</v>
       </c>
       <c r="N4">
-        <v>1.14</v>
+        <v>1.28</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>3.5</v>
+        <v>6.1</v>
       </c>
       <c r="Q4">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="R4">
         <v>100</v>
@@ -3251,19 +3251,19 @@
         <v>1</v>
       </c>
       <c r="X4">
-        <v>0.3425</v>
+        <v>0.3625</v>
       </c>
       <c r="Y4">
-        <v>0.11</v>
+        <v>-0.03</v>
       </c>
       <c r="Z4">
-        <v>0.08</v>
+        <v>0.01</v>
       </c>
       <c r="AA4">
-        <v>8.5</v>
+        <v>9</v>
       </c>
       <c r="AB4">
-        <v>89.5</v>
+        <v>89.3</v>
       </c>
       <c r="AC4">
         <v>82.2</v>
@@ -3290,19 +3290,19 @@
         <v>82.59999999999999</v>
       </c>
       <c r="AK4">
-        <v>66.8</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="AL4">
-        <v>59.7</v>
+        <v>60.7</v>
       </c>
       <c r="AM4">
-        <v>1012.3</v>
+        <v>1012.2</v>
       </c>
       <c r="AN4">
         <v>1014.5</v>
       </c>
       <c r="AO4">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="AP4">
         <v>0</v>
@@ -3314,13 +3314,13 @@
         <v>50.6</v>
       </c>
       <c r="AS4">
-        <v>684</v>
+        <v>779</v>
       </c>
       <c r="AT4">
-        <v>8.9</v>
+        <v>9</v>
       </c>
       <c r="AU4">
-        <v>17.5</v>
+        <v>17.7</v>
       </c>
       <c r="AV4" t="s">
         <v>188</v>
@@ -3335,13 +3335,13 @@
         <v>8.4</v>
       </c>
       <c r="AZ4">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="BA4">
         <v>-2.3</v>
       </c>
       <c r="BB4">
-        <v>1.1593</v>
+        <v>1.1591</v>
       </c>
       <c r="BC4" t="s">
         <v>262</v>
@@ -3356,34 +3356,34 @@
         <v>182</v>
       </c>
       <c r="BG4">
+        <v>86.09999999999999</v>
+      </c>
+      <c r="BH4">
+        <v>1.087</v>
+      </c>
+      <c r="BI4">
+        <v>83.5</v>
+      </c>
+      <c r="BJ4">
         <v>85.90000000000001</v>
       </c>
-      <c r="BH4">
-        <v>1.086</v>
-      </c>
-      <c r="BI4">
-        <v>83.3</v>
-      </c>
-      <c r="BJ4">
-        <v>85.7</v>
-      </c>
       <c r="BK4">
-        <v>59</v>
+        <v>59.1</v>
       </c>
       <c r="BL4">
-        <v>58.2</v>
+        <v>58.3</v>
       </c>
       <c r="BM4">
-        <v>56.8</v>
+        <v>56.1</v>
       </c>
       <c r="BN4">
-        <v>6.8</v>
+        <v>7.8</v>
       </c>
       <c r="BO4" t="s">
         <v>180</v>
       </c>
       <c r="BP4">
-        <v>12.1</v>
+        <v>12</v>
       </c>
       <c r="BQ4" t="s">
         <v>180</v>
@@ -3392,7 +3392,7 @@
         <v>85</v>
       </c>
       <c r="BS4">
-        <v>80.90000000000001</v>
+        <v>80.8</v>
       </c>
       <c r="BT4">
         <v>10</v>
@@ -3430,28 +3430,28 @@
         <v>187</v>
       </c>
       <c r="J5">
-        <v>53.3</v>
+        <v>73.7</v>
       </c>
       <c r="K5">
-        <v>7.4</v>
+        <v>7.1</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>1.96</v>
+        <v>1.99</v>
       </c>
       <c r="N5">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="O5">
         <v>0</v>
       </c>
       <c r="P5">
-        <v>5</v>
+        <v>7.9</v>
       </c>
       <c r="Q5">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="R5">
         <v>100</v>
@@ -3472,19 +3472,19 @@
         <v>1</v>
       </c>
       <c r="X5">
-        <v>0.29</v>
+        <v>0.3069</v>
       </c>
       <c r="Y5">
-        <v>0.09</v>
+        <v>-0.03</v>
       </c>
       <c r="Z5">
-        <v>0.07000000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="AA5">
-        <v>11.7</v>
+        <v>12.1</v>
       </c>
       <c r="AB5">
-        <v>88.59999999999999</v>
+        <v>88.5</v>
       </c>
       <c r="AC5">
         <v>80.2</v>
@@ -3505,25 +3505,25 @@
         <v>185</v>
       </c>
       <c r="AI5">
-        <v>80.8</v>
+        <v>80.7</v>
       </c>
       <c r="AJ5">
         <v>79.7</v>
       </c>
       <c r="AK5">
-        <v>66.40000000000001</v>
+        <v>67</v>
       </c>
       <c r="AL5">
-        <v>63.3</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="AM5">
-        <v>1012.2</v>
+        <v>1012.1</v>
       </c>
       <c r="AN5">
-        <v>1014.5</v>
+        <v>1014.4</v>
       </c>
       <c r="AO5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP5">
         <v>0</v>
@@ -3535,13 +3535,13 @@
         <v>43.6</v>
       </c>
       <c r="AS5">
-        <v>504</v>
+        <v>602</v>
       </c>
       <c r="AT5">
         <v>8.800000000000001</v>
       </c>
       <c r="AU5">
-        <v>16.8</v>
+        <v>17</v>
       </c>
       <c r="AV5" t="s">
         <v>188</v>
@@ -3562,13 +3562,13 @@
         <v>-2.3</v>
       </c>
       <c r="BB5">
-        <v>1.1648</v>
+        <v>1.1645</v>
       </c>
       <c r="BC5" t="s">
         <v>263</v>
       </c>
       <c r="BD5">
-        <v>1472</v>
+        <v>1474</v>
       </c>
       <c r="BE5" t="s">
         <v>181</v>
@@ -3577,28 +3577,28 @@
         <v>182</v>
       </c>
       <c r="BG5">
-        <v>84</v>
+        <v>84.2</v>
       </c>
       <c r="BH5">
         <v>1.082</v>
       </c>
       <c r="BI5">
-        <v>81.5</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="BJ5">
-        <v>83.8</v>
+        <v>84</v>
       </c>
       <c r="BK5">
-        <v>58.4</v>
+        <v>58.5</v>
       </c>
       <c r="BL5">
-        <v>57.5</v>
+        <v>57.6</v>
       </c>
       <c r="BM5">
-        <v>60.4</v>
+        <v>59.8</v>
       </c>
       <c r="BN5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BO5" t="s">
         <v>180</v>
@@ -3619,7 +3619,7 @@
         <v>10</v>
       </c>
       <c r="BU5">
-        <v>8.1</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -3724,7 +3724,7 @@
         <v>173</v>
       </c>
       <c r="E2">
-        <v>87.8</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="F2">
         <v>84.3</v>
@@ -3745,16 +3745,16 @@
         <v>174</v>
       </c>
       <c r="L2">
-        <v>90.8</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="M2">
         <v>8.6</v>
       </c>
       <c r="N2">
-        <v>86.3</v>
+        <v>86.2</v>
       </c>
       <c r="O2">
-        <v>1833</v>
+        <v>1832</v>
       </c>
       <c r="P2" t="s">
         <v>181</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 01:15 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_2026_07_14.xlsx
+++ b/mlb_weather_professional_2026_07_14.xlsx
@@ -12,16 +12,16 @@
     <sheet name="HR Weather" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Game Summary'!$A$1:$FK$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hourly Detail'!$A$1:$BU$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'HR Weather'!$A$1:$R$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Game Summary'!$A$1:$FU$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hourly Detail'!$A$1:$CD$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'HR Weather'!$A$1:$S$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="674" uniqueCount="279">
   <si>
     <t>Date</t>
   </si>
@@ -221,6 +221,24 @@
     <t>Game Avg Wind Toward RF MPH</t>
   </si>
   <si>
+    <t>Game Effective Wind Vector MPH</t>
+  </si>
+  <si>
+    <t>Game Park Swirl Uncertainty MPH</t>
+  </si>
+  <si>
+    <t>LF Shield Multiplier</t>
+  </si>
+  <si>
+    <t>CF Shield Multiplier</t>
+  </si>
+  <si>
+    <t>RF Shield Multiplier</t>
+  </si>
+  <si>
+    <t>Park Swirl Factor</t>
+  </si>
+  <si>
     <t>Game Avg Air Density kg/m3</t>
   </si>
   <si>
@@ -239,6 +257,15 @@
     <t>Pressure Change hPa</t>
   </si>
   <si>
+    <t>Park Learned Calibration Points</t>
+  </si>
+  <si>
+    <t>Park Calibration Settled Games</t>
+  </si>
+  <si>
+    <t>Pre-Calibration HR Score</t>
+  </si>
+  <si>
     <t>First Pitch Temp F</t>
   </si>
   <si>
@@ -524,6 +551,9 @@
     <t>Carry Percentile Value</t>
   </si>
   <si>
+    <t>Estimated FT Change by Wind</t>
+  </si>
+  <si>
     <t>2026-07-14</t>
   </si>
   <si>
@@ -545,22 +575,22 @@
     <t>Citizens Bank Park</t>
   </si>
   <si>
-    <t>🔥 Excellent</t>
-  </si>
-  <si>
-    <t>adjusted carry 84.3; +19 ft carry; +8.2% HR env.</t>
+    <t>🟢 Very Good</t>
+  </si>
+  <si>
+    <t>adjusted carry 79.8; +16 ft carry; +7.2% HR env.</t>
   </si>
   <si>
     <t>100th</t>
   </si>
   <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>STEADY</t>
-  </si>
-  <si>
-    <t>2026-07-14 01:02:26 PM PDT</t>
+    <t>A-</t>
+  </si>
+  <si>
+    <t>WORSENING RAPIDLY</t>
+  </si>
+  <si>
+    <t>2026-07-14 01:15:39 PM PDT</t>
   </si>
   <si>
     <t>LOW</t>
@@ -581,18 +611,18 @@
     <t>Clear</t>
   </si>
   <si>
+    <t>2026-07-14 20:15:39 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14T18:41:01+00:00</t>
+  </si>
+  <si>
+    <t>SW</t>
+  </si>
+  <si>
     <t>2026-07-14 20:02:26 UTC</t>
   </si>
   <si>
-    <t>2026-07-14T18:41:01+00:00</t>
-  </si>
-  <si>
-    <t>SW</t>
-  </si>
-  <si>
-    <t>2026-07-14 19:54:42 UTC</t>
-  </si>
-  <si>
     <t>Period</t>
   </si>
   <si>
@@ -704,6 +734,15 @@
     <t>Wind From Degrees</t>
   </si>
   <si>
+    <t>Raw Wind Toward CF MPH</t>
+  </si>
+  <si>
+    <t>Raw Wind Toward LF MPH</t>
+  </si>
+  <si>
+    <t>Raw Wind Toward RF MPH</t>
+  </si>
+  <si>
     <t>Wind Toward CF MPH</t>
   </si>
   <si>
@@ -714,6 +753,12 @@
   </si>
   <si>
     <t>Crosswind MPH</t>
+  </si>
+  <si>
+    <t>Effective Wind Vector MPH</t>
+  </si>
+  <si>
+    <t>Park Swirl Uncertainty MPH</t>
   </si>
   <si>
     <t>Air Density kg/m3</t>
@@ -1268,7 +1313,7 @@
   <sheetPr>
     <tabColor rgb="FF70AD47"/>
   </sheetPr>
-  <dimension ref="A1:FK2"/>
+  <dimension ref="A1:FU2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -1291,7 +1336,7 @@
     <col min="19" max="19" width="27.7109375" customWidth="1"/>
     <col min="20" max="20" width="34.7109375" customWidth="1"/>
     <col min="21" max="21" width="20.7109375" style="2" customWidth="1"/>
-    <col min="22" max="22" width="16.7109375" customWidth="1"/>
+    <col min="22" max="22" width="19.7109375" customWidth="1"/>
     <col min="23" max="23" width="34.7109375" customWidth="1"/>
     <col min="24" max="24" width="30.7109375" customWidth="1"/>
     <col min="25" max="29" width="34.7109375" customWidth="1"/>
@@ -1325,92 +1370,100 @@
     <col min="62" max="62" width="23.7109375" customWidth="1"/>
     <col min="63" max="64" width="19.7109375" customWidth="1"/>
     <col min="65" max="66" width="29.7109375" customWidth="1"/>
-    <col min="67" max="67" width="28.7109375" customWidth="1"/>
-    <col min="68" max="68" width="16.7109375" customWidth="1"/>
-    <col min="69" max="69" width="28.7109375" customWidth="1"/>
-    <col min="70" max="70" width="29.7109375" customWidth="1"/>
-    <col min="71" max="71" width="27.7109375" customWidth="1"/>
-    <col min="72" max="72" width="21.7109375" customWidth="1"/>
-    <col min="73" max="73" width="20.7109375" customWidth="1"/>
-    <col min="74" max="74" width="25.7109375" customWidth="1"/>
-    <col min="75" max="75" width="18.7109375" customWidth="1"/>
-    <col min="76" max="76" width="34.7109375" customWidth="1"/>
+    <col min="67" max="67" width="32.7109375" customWidth="1"/>
+    <col min="68" max="68" width="33.7109375" customWidth="1"/>
+    <col min="69" max="71" width="22.7109375" customWidth="1"/>
+    <col min="72" max="72" width="19.7109375" customWidth="1"/>
+    <col min="73" max="73" width="28.7109375" customWidth="1"/>
+    <col min="74" max="74" width="16.7109375" customWidth="1"/>
+    <col min="75" max="75" width="28.7109375" customWidth="1"/>
+    <col min="76" max="76" width="29.7109375" customWidth="1"/>
     <col min="77" max="77" width="27.7109375" customWidth="1"/>
-    <col min="78" max="79" width="22.7109375" customWidth="1"/>
-    <col min="80" max="80" width="27.7109375" customWidth="1"/>
-    <col min="81" max="81" width="23.7109375" customWidth="1"/>
-    <col min="82" max="84" width="32.7109375" customWidth="1"/>
-    <col min="85" max="85" width="31.7109375" customWidth="1"/>
-    <col min="86" max="86" width="33.7109375" customWidth="1"/>
-    <col min="87" max="87" width="28.7109375" customWidth="1"/>
-    <col min="88" max="88" width="30.7109375" customWidth="1"/>
-    <col min="89" max="90" width="29.7109375" customWidth="1"/>
-    <col min="91" max="93" width="34.7109375" customWidth="1"/>
-    <col min="94" max="94" width="30.7109375" customWidth="1"/>
-    <col min="95" max="95" width="24.7109375" customWidth="1"/>
-    <col min="96" max="96" width="16.7109375" customWidth="1"/>
-    <col min="97" max="97" width="21.7109375" customWidth="1"/>
-    <col min="98" max="98" width="14.7109375" customWidth="1"/>
-    <col min="99" max="99" width="30.7109375" customWidth="1"/>
-    <col min="100" max="100" width="23.7109375" customWidth="1"/>
-    <col min="101" max="102" width="18.7109375" customWidth="1"/>
-    <col min="103" max="103" width="23.7109375" customWidth="1"/>
-    <col min="104" max="104" width="19.7109375" customWidth="1"/>
-    <col min="105" max="107" width="28.7109375" customWidth="1"/>
-    <col min="108" max="108" width="27.7109375" customWidth="1"/>
-    <col min="109" max="109" width="29.7109375" customWidth="1"/>
-    <col min="110" max="110" width="24.7109375" customWidth="1"/>
-    <col min="111" max="111" width="26.7109375" customWidth="1"/>
-    <col min="112" max="113" width="25.7109375" customWidth="1"/>
-    <col min="114" max="114" width="34.7109375" customWidth="1"/>
-    <col min="115" max="115" width="30.7109375" customWidth="1"/>
-    <col min="116" max="116" width="34.7109375" customWidth="1"/>
-    <col min="117" max="117" width="26.7109375" customWidth="1"/>
-    <col min="118" max="118" width="20.7109375" customWidth="1"/>
-    <col min="119" max="119" width="17.7109375" customWidth="1"/>
-    <col min="120" max="120" width="22.7109375" customWidth="1"/>
-    <col min="121" max="121" width="15.7109375" customWidth="1"/>
-    <col min="122" max="122" width="31.7109375" customWidth="1"/>
-    <col min="123" max="123" width="24.7109375" customWidth="1"/>
-    <col min="124" max="125" width="19.7109375" customWidth="1"/>
-    <col min="126" max="126" width="24.7109375" customWidth="1"/>
+    <col min="78" max="78" width="21.7109375" customWidth="1"/>
+    <col min="79" max="79" width="33.7109375" customWidth="1"/>
+    <col min="80" max="80" width="32.7109375" customWidth="1"/>
+    <col min="81" max="81" width="26.7109375" customWidth="1"/>
+    <col min="82" max="82" width="20.7109375" customWidth="1"/>
+    <col min="83" max="83" width="25.7109375" customWidth="1"/>
+    <col min="84" max="84" width="18.7109375" customWidth="1"/>
+    <col min="85" max="85" width="34.7109375" customWidth="1"/>
+    <col min="86" max="86" width="27.7109375" customWidth="1"/>
+    <col min="87" max="88" width="22.7109375" customWidth="1"/>
+    <col min="89" max="89" width="27.7109375" customWidth="1"/>
+    <col min="90" max="90" width="23.7109375" customWidth="1"/>
+    <col min="91" max="93" width="32.7109375" customWidth="1"/>
+    <col min="94" max="94" width="31.7109375" customWidth="1"/>
+    <col min="95" max="95" width="33.7109375" customWidth="1"/>
+    <col min="96" max="96" width="28.7109375" customWidth="1"/>
+    <col min="97" max="97" width="30.7109375" customWidth="1"/>
+    <col min="98" max="99" width="29.7109375" customWidth="1"/>
+    <col min="100" max="102" width="34.7109375" customWidth="1"/>
+    <col min="103" max="103" width="30.7109375" customWidth="1"/>
+    <col min="104" max="104" width="24.7109375" customWidth="1"/>
+    <col min="105" max="105" width="16.7109375" customWidth="1"/>
+    <col min="106" max="106" width="21.7109375" customWidth="1"/>
+    <col min="107" max="107" width="14.7109375" customWidth="1"/>
+    <col min="108" max="108" width="30.7109375" customWidth="1"/>
+    <col min="109" max="109" width="23.7109375" customWidth="1"/>
+    <col min="110" max="111" width="18.7109375" customWidth="1"/>
+    <col min="112" max="112" width="23.7109375" customWidth="1"/>
+    <col min="113" max="113" width="19.7109375" customWidth="1"/>
+    <col min="114" max="116" width="28.7109375" customWidth="1"/>
+    <col min="117" max="117" width="27.7109375" customWidth="1"/>
+    <col min="118" max="118" width="29.7109375" customWidth="1"/>
+    <col min="119" max="119" width="24.7109375" customWidth="1"/>
+    <col min="120" max="120" width="26.7109375" customWidth="1"/>
+    <col min="121" max="122" width="25.7109375" customWidth="1"/>
+    <col min="123" max="123" width="34.7109375" customWidth="1"/>
+    <col min="124" max="124" width="30.7109375" customWidth="1"/>
+    <col min="125" max="125" width="34.7109375" customWidth="1"/>
+    <col min="126" max="126" width="26.7109375" customWidth="1"/>
     <col min="127" max="127" width="20.7109375" customWidth="1"/>
-    <col min="128" max="130" width="29.7109375" customWidth="1"/>
-    <col min="131" max="131" width="28.7109375" customWidth="1"/>
-    <col min="132" max="132" width="30.7109375" customWidth="1"/>
-    <col min="133" max="133" width="25.7109375" customWidth="1"/>
-    <col min="134" max="134" width="27.7109375" customWidth="1"/>
-    <col min="135" max="136" width="26.7109375" customWidth="1"/>
-    <col min="137" max="137" width="34.7109375" customWidth="1"/>
-    <col min="138" max="138" width="31.7109375" customWidth="1"/>
-    <col min="139" max="139" width="34.7109375" customWidth="1"/>
-    <col min="140" max="140" width="27.7109375" customWidth="1"/>
-    <col min="141" max="141" width="21.7109375" customWidth="1"/>
-    <col min="142" max="142" width="17.7109375" customWidth="1"/>
-    <col min="143" max="143" width="22.7109375" customWidth="1"/>
-    <col min="144" max="144" width="15.7109375" customWidth="1"/>
-    <col min="145" max="145" width="31.7109375" customWidth="1"/>
-    <col min="146" max="146" width="24.7109375" customWidth="1"/>
-    <col min="147" max="148" width="19.7109375" customWidth="1"/>
-    <col min="149" max="149" width="24.7109375" customWidth="1"/>
-    <col min="150" max="150" width="20.7109375" customWidth="1"/>
-    <col min="151" max="153" width="29.7109375" customWidth="1"/>
-    <col min="154" max="154" width="28.7109375" customWidth="1"/>
-    <col min="155" max="155" width="30.7109375" customWidth="1"/>
-    <col min="156" max="156" width="25.7109375" customWidth="1"/>
-    <col min="157" max="157" width="27.7109375" customWidth="1"/>
-    <col min="158" max="159" width="26.7109375" customWidth="1"/>
-    <col min="160" max="160" width="34.7109375" customWidth="1"/>
-    <col min="161" max="161" width="31.7109375" customWidth="1"/>
-    <col min="162" max="162" width="34.7109375" customWidth="1"/>
-    <col min="163" max="163" width="27.7109375" customWidth="1"/>
-    <col min="164" max="164" width="21.7109375" customWidth="1"/>
-    <col min="165" max="165" width="27.7109375" customWidth="1"/>
-    <col min="166" max="166" width="34.7109375" customWidth="1"/>
-    <col min="167" max="167" width="24.7109375" customWidth="1"/>
+    <col min="128" max="128" width="17.7109375" customWidth="1"/>
+    <col min="129" max="129" width="22.7109375" customWidth="1"/>
+    <col min="130" max="130" width="15.7109375" customWidth="1"/>
+    <col min="131" max="131" width="31.7109375" customWidth="1"/>
+    <col min="132" max="132" width="24.7109375" customWidth="1"/>
+    <col min="133" max="134" width="19.7109375" customWidth="1"/>
+    <col min="135" max="135" width="24.7109375" customWidth="1"/>
+    <col min="136" max="136" width="20.7109375" customWidth="1"/>
+    <col min="137" max="139" width="29.7109375" customWidth="1"/>
+    <col min="140" max="140" width="28.7109375" customWidth="1"/>
+    <col min="141" max="141" width="30.7109375" customWidth="1"/>
+    <col min="142" max="142" width="25.7109375" customWidth="1"/>
+    <col min="143" max="143" width="27.7109375" customWidth="1"/>
+    <col min="144" max="145" width="26.7109375" customWidth="1"/>
+    <col min="146" max="146" width="34.7109375" customWidth="1"/>
+    <col min="147" max="147" width="31.7109375" customWidth="1"/>
+    <col min="148" max="148" width="34.7109375" customWidth="1"/>
+    <col min="149" max="149" width="27.7109375" customWidth="1"/>
+    <col min="150" max="150" width="21.7109375" customWidth="1"/>
+    <col min="151" max="151" width="17.7109375" customWidth="1"/>
+    <col min="152" max="152" width="22.7109375" customWidth="1"/>
+    <col min="153" max="153" width="15.7109375" customWidth="1"/>
+    <col min="154" max="154" width="31.7109375" customWidth="1"/>
+    <col min="155" max="155" width="24.7109375" customWidth="1"/>
+    <col min="156" max="157" width="19.7109375" customWidth="1"/>
+    <col min="158" max="158" width="24.7109375" customWidth="1"/>
+    <col min="159" max="159" width="20.7109375" customWidth="1"/>
+    <col min="160" max="162" width="29.7109375" customWidth="1"/>
+    <col min="163" max="163" width="28.7109375" customWidth="1"/>
+    <col min="164" max="164" width="30.7109375" customWidth="1"/>
+    <col min="165" max="165" width="25.7109375" customWidth="1"/>
+    <col min="166" max="166" width="27.7109375" customWidth="1"/>
+    <col min="167" max="168" width="26.7109375" customWidth="1"/>
+    <col min="169" max="169" width="34.7109375" customWidth="1"/>
+    <col min="170" max="170" width="31.7109375" customWidth="1"/>
+    <col min="171" max="171" width="34.7109375" customWidth="1"/>
+    <col min="172" max="172" width="27.7109375" customWidth="1"/>
+    <col min="173" max="173" width="21.7109375" customWidth="1"/>
+    <col min="174" max="174" width="27.7109375" customWidth="1"/>
+    <col min="175" max="175" width="34.7109375" customWidth="1"/>
+    <col min="176" max="176" width="24.7109375" customWidth="1"/>
+    <col min="177" max="177" width="29.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:167" ht="34" customHeight="1">
+    <row r="1" spans="1:177" ht="34" customHeight="1">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1912,82 +1965,112 @@
       <c r="FK1" s="3" t="s">
         <v>166</v>
       </c>
+      <c r="FL1" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="FM1" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="FN1" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="FO1" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="FP1" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="FQ1" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="FR1" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="FS1" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="FT1" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="FU1" s="3" t="s">
+        <v>176</v>
+      </c>
     </row>
-    <row r="2" spans="1:167">
+    <row r="2" spans="1:177">
       <c r="A2" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="B2" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="C2" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="D2" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="E2" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="F2" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="G2" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="H2" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="I2" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="J2" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="K2">
-        <v>87.90000000000001</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="L2">
-        <v>84.3</v>
+        <v>79.8</v>
       </c>
       <c r="M2" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="N2" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="O2">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="P2">
-        <v>8.199999999999999</v>
+        <v>7.2</v>
       </c>
       <c r="Q2" s="1">
-        <v>87.90000000000001</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="R2">
-        <v>84.3</v>
+        <v>79.8</v>
       </c>
       <c r="S2">
         <v>90.7</v>
       </c>
       <c r="T2">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="U2" s="2">
-        <v>1.091</v>
+        <v>1.072</v>
       </c>
       <c r="V2" t="s">
-        <v>178</v>
+        <v>188</v>
       </c>
       <c r="W2">
-        <v>0</v>
+        <v>-4.5</v>
       </c>
       <c r="X2">
         <v>0</v>
       </c>
       <c r="Y2">
-        <v>0</v>
+        <v>-1.4</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -2002,58 +2085,58 @@
         <v>4.2</v>
       </c>
       <c r="AD2">
-        <v>1.1</v>
+        <v>0.4</v>
       </c>
       <c r="AE2">
-        <v>-0</v>
+        <v>0.15</v>
       </c>
       <c r="AF2">
-        <v>-0.03</v>
+        <v>0.1</v>
       </c>
       <c r="AG2" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="AH2">
-        <v>81.40000000000001</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="AI2">
         <v>5</v>
       </c>
       <c r="AJ2" s="1">
-        <v>85.3</v>
+        <v>84.5</v>
       </c>
       <c r="AK2" s="1">
-        <v>87.7</v>
+        <v>79.5</v>
       </c>
       <c r="AL2">
-        <v>8.6</v>
+        <v>7.2</v>
       </c>
       <c r="AM2">
-        <v>1832</v>
+        <v>1826</v>
       </c>
       <c r="AN2" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="AO2">
-        <v>11.2</v>
+        <v>10.9</v>
       </c>
       <c r="AP2" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="AQ2">
         <v>12</v>
       </c>
       <c r="AR2" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
       <c r="AS2" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="AT2" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="AU2" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="AV2">
         <v>39.9061</v>
@@ -2065,19 +2148,19 @@
         <v>20</v>
       </c>
       <c r="AY2">
-        <v>60</v>
+        <v>10.07</v>
       </c>
       <c r="AZ2" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="BA2" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
       <c r="BB2" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="BC2" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
       <c r="BD2">
         <v>0.98</v>
@@ -2092,13 +2175,13 @@
         <v>86.2</v>
       </c>
       <c r="BH2">
-        <v>67.8</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="BI2">
-        <v>56.1</v>
+        <v>57.2</v>
       </c>
       <c r="BJ2">
-        <v>1012.2</v>
+        <v>1012.4</v>
       </c>
       <c r="BK2">
         <v>8.9</v>
@@ -2107,317 +2190,347 @@
         <v>19.4</v>
       </c>
       <c r="BM2">
+        <v>2.7</v>
+      </c>
+      <c r="BN2">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="BO2">
+        <v>6.4</v>
+      </c>
+      <c r="BP2">
+        <v>0.8</v>
+      </c>
+      <c r="BQ2">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="BR2">
+        <v>1.03</v>
+      </c>
+      <c r="BS2">
+        <v>0.98</v>
+      </c>
+      <c r="BT2">
+        <v>0.09</v>
+      </c>
+      <c r="BU2">
+        <v>1.1527</v>
+      </c>
+      <c r="BV2">
+        <v>59.8</v>
+      </c>
+      <c r="BW2">
+        <v>58</v>
+      </c>
+      <c r="BX2">
+        <v>51.5</v>
+      </c>
+      <c r="BY2">
+        <v>-8.6</v>
+      </c>
+      <c r="BZ2">
+        <v>-0.5</v>
+      </c>
+      <c r="CA2">
+        <v>0</v>
+      </c>
+      <c r="CB2">
+        <v>0</v>
+      </c>
+      <c r="CC2">
+        <v>79.8</v>
+      </c>
+      <c r="CD2">
+        <v>89.40000000000001</v>
+      </c>
+      <c r="CE2">
+        <v>68.7</v>
+      </c>
+      <c r="CF2">
+        <v>52.1</v>
+      </c>
+      <c r="CG2">
+        <v>1012.6</v>
+      </c>
+      <c r="CH2">
+        <v>0</v>
+      </c>
+      <c r="CI2">
+        <v>0</v>
+      </c>
+      <c r="CJ2">
+        <v>9</v>
+      </c>
+      <c r="CK2">
+        <v>19.4</v>
+      </c>
+      <c r="CL2" t="s">
+        <v>198</v>
+      </c>
+      <c r="CM2">
+        <v>7.2</v>
+      </c>
+      <c r="CN2">
+        <v>2.8</v>
+      </c>
+      <c r="CO2">
         <v>8.4</v>
       </c>
-      <c r="BN2">
-        <v>5.8</v>
-      </c>
-      <c r="BO2">
-        <v>1.1527</v>
-      </c>
-      <c r="BP2">
-        <v>59.6</v>
-      </c>
-      <c r="BQ2">
-        <v>59</v>
-      </c>
-      <c r="BR2">
-        <v>52</v>
-      </c>
-      <c r="BS2">
-        <v>-8.699999999999999</v>
-      </c>
-      <c r="BT2">
-        <v>-0.1</v>
-      </c>
-      <c r="BU2">
-        <v>89.40000000000001</v>
-      </c>
-      <c r="BV2">
-        <v>68.5</v>
-      </c>
-      <c r="BW2">
-        <v>51.8</v>
-      </c>
-      <c r="BX2">
-        <v>1012.2</v>
-      </c>
-      <c r="BY2">
+      <c r="CP2">
+        <v>1.146</v>
+      </c>
+      <c r="CQ2">
+        <v>2032</v>
+      </c>
+      <c r="CR2">
+        <v>85.09999999999999</v>
+      </c>
+      <c r="CS2">
+        <v>1.084</v>
+      </c>
+      <c r="CT2">
+        <v>86.8</v>
+      </c>
+      <c r="CU2">
+        <v>81.7</v>
+      </c>
+      <c r="CV2">
+        <v>82</v>
+      </c>
+      <c r="CW2">
+        <v>91.3</v>
+      </c>
+      <c r="CX2">
+        <v>5.9</v>
+      </c>
+      <c r="CY2">
+        <v>10.9</v>
+      </c>
+      <c r="CZ2" t="s">
+        <v>190</v>
+      </c>
+      <c r="DA2">
+        <v>85.7</v>
+      </c>
+      <c r="DB2">
+        <v>68.3</v>
+      </c>
+      <c r="DC2">
+        <v>57.7</v>
+      </c>
+      <c r="DD2">
+        <v>1012.3</v>
+      </c>
+      <c r="DE2">
         <v>0</v>
       </c>
-      <c r="BZ2">
+      <c r="DF2">
         <v>0</v>
       </c>
-      <c r="CA2">
+      <c r="DG2">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="DH2">
+        <v>17.7</v>
+      </c>
+      <c r="DI2" t="s">
+        <v>198</v>
+      </c>
+      <c r="DJ2">
+        <v>7.1</v>
+      </c>
+      <c r="DK2">
+        <v>2.7</v>
+      </c>
+      <c r="DL2">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="DM2">
+        <v>1.1537</v>
+      </c>
+      <c r="DN2">
+        <v>1794</v>
+      </c>
+      <c r="DO2">
+        <v>82.2</v>
+      </c>
+      <c r="DP2">
+        <v>1.077</v>
+      </c>
+      <c r="DQ2">
+        <v>83.90000000000001</v>
+      </c>
+      <c r="DR2">
+        <v>79</v>
+      </c>
+      <c r="DS2">
+        <v>79.5</v>
+      </c>
+      <c r="DT2">
+        <v>91.5</v>
+      </c>
+      <c r="DU2">
+        <v>5.7</v>
+      </c>
+      <c r="DV2">
+        <v>8.6</v>
+      </c>
+      <c r="DW2" t="s">
+        <v>190</v>
+      </c>
+      <c r="DX2">
+        <v>83.3</v>
+      </c>
+      <c r="DY2">
+        <v>68.09999999999999</v>
+      </c>
+      <c r="DZ2">
+        <v>62</v>
+      </c>
+      <c r="EA2">
+        <v>1012.3</v>
+      </c>
+      <c r="EB2">
+        <v>0</v>
+      </c>
+      <c r="EC2">
+        <v>0</v>
+      </c>
+      <c r="ED2">
         <v>9</v>
       </c>
-      <c r="CB2">
-        <v>19.4</v>
-      </c>
-      <c r="CC2" t="s">
-        <v>188</v>
-      </c>
-      <c r="CD2">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="CE2">
-        <v>8.5</v>
-      </c>
-      <c r="CF2">
-        <v>5.8</v>
-      </c>
-      <c r="CG2">
-        <v>1.1457</v>
-      </c>
-      <c r="CH2">
-        <v>2042</v>
-      </c>
-      <c r="CI2">
-        <v>90.2</v>
-      </c>
-      <c r="CJ2">
-        <v>1.096</v>
-      </c>
-      <c r="CK2">
-        <v>87.59999999999999</v>
-      </c>
-      <c r="CL2">
-        <v>90</v>
-      </c>
-      <c r="CM2">
-        <v>86.7</v>
-      </c>
-      <c r="CN2">
-        <v>91.3</v>
-      </c>
-      <c r="CO2">
-        <v>5.9</v>
-      </c>
-      <c r="CP2">
-        <v>11.2</v>
-      </c>
-      <c r="CQ2" t="s">
-        <v>180</v>
-      </c>
-      <c r="CR2">
-        <v>85.7</v>
-      </c>
-      <c r="CS2">
-        <v>67.3</v>
-      </c>
-      <c r="CT2">
-        <v>56.1</v>
-      </c>
-      <c r="CU2">
-        <v>1012.1</v>
-      </c>
-      <c r="CV2">
-        <v>0</v>
-      </c>
-      <c r="CW2">
-        <v>0</v>
-      </c>
-      <c r="CX2">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="CY2">
-        <v>17.7</v>
-      </c>
-      <c r="CZ2" t="s">
-        <v>188</v>
-      </c>
-      <c r="DA2">
-        <v>8.5</v>
-      </c>
-      <c r="DB2">
+      <c r="EE2">
+        <v>17.8</v>
+      </c>
+      <c r="EF2" t="s">
+        <v>198</v>
+      </c>
+      <c r="EG2">
+        <v>7.2</v>
+      </c>
+      <c r="EH2">
+        <v>2.7</v>
+      </c>
+      <c r="EI2">
         <v>8.300000000000001</v>
       </c>
-      <c r="DC2">
-        <v>5.7</v>
-      </c>
-      <c r="DD2">
-        <v>1.1538</v>
-      </c>
-      <c r="DE2">
-        <v>1801</v>
-      </c>
-      <c r="DF2">
-        <v>87.2</v>
-      </c>
-      <c r="DG2">
-        <v>1.089</v>
-      </c>
-      <c r="DH2">
-        <v>84.59999999999999</v>
-      </c>
-      <c r="DI2">
-        <v>87</v>
-      </c>
-      <c r="DJ2">
-        <v>84</v>
-      </c>
-      <c r="DK2">
-        <v>91.40000000000001</v>
-      </c>
-      <c r="DL2">
-        <v>5.8</v>
-      </c>
-      <c r="DM2">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="DN2" t="s">
-        <v>180</v>
-      </c>
-      <c r="DO2">
-        <v>83.3</v>
-      </c>
-      <c r="DP2">
-        <v>67.40000000000001</v>
-      </c>
-      <c r="DQ2">
-        <v>60.7</v>
-      </c>
-      <c r="DR2">
-        <v>1012.2</v>
-      </c>
-      <c r="DS2">
-        <v>0</v>
-      </c>
-      <c r="DT2">
-        <v>0</v>
-      </c>
-      <c r="DU2">
-        <v>8.9</v>
-      </c>
-      <c r="DV2">
-        <v>17.8</v>
-      </c>
-      <c r="DW2" t="s">
-        <v>188</v>
-      </c>
-      <c r="DX2">
-        <v>8.6</v>
-      </c>
-      <c r="DY2">
-        <v>8.4</v>
-      </c>
-      <c r="DZ2">
-        <v>5.8</v>
-      </c>
-      <c r="EA2">
-        <v>1.1591</v>
-      </c>
-      <c r="EB2">
-        <v>1637</v>
-      </c>
-      <c r="EC2">
-        <v>86.09999999999999</v>
-      </c>
-      <c r="ED2">
-        <v>1.087</v>
-      </c>
-      <c r="EE2">
-        <v>83.5</v>
-      </c>
-      <c r="EF2">
-        <v>85.90000000000001</v>
-      </c>
-      <c r="EG2">
-        <v>82.2</v>
-      </c>
-      <c r="EH2">
-        <v>89.40000000000001</v>
-      </c>
-      <c r="EI2">
-        <v>9</v>
-      </c>
       <c r="EJ2">
-        <v>7.8</v>
-      </c>
-      <c r="EK2" t="s">
-        <v>180</v>
+        <v>1.1589</v>
+      </c>
+      <c r="EK2">
+        <v>1636</v>
       </c>
       <c r="EL2">
-        <v>80.7</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="EM2">
-        <v>67</v>
+        <v>1.075</v>
       </c>
       <c r="EN2">
-        <v>64.40000000000001</v>
+        <v>82.8</v>
       </c>
       <c r="EO2">
-        <v>1012.1</v>
+        <v>77.7</v>
       </c>
       <c r="EP2">
-        <v>0</v>
+        <v>77.8</v>
       </c>
       <c r="EQ2">
-        <v>0</v>
+        <v>89.5</v>
       </c>
       <c r="ER2">
         <v>8.800000000000001</v>
       </c>
       <c r="ES2">
+        <v>7.3</v>
+      </c>
+      <c r="ET2" t="s">
+        <v>190</v>
+      </c>
+      <c r="EU2">
+        <v>80.8</v>
+      </c>
+      <c r="EV2">
+        <v>67.90000000000001</v>
+      </c>
+      <c r="EW2">
+        <v>66.3</v>
+      </c>
+      <c r="EX2">
+        <v>1012.1</v>
+      </c>
+      <c r="EY2">
+        <v>0</v>
+      </c>
+      <c r="EZ2">
+        <v>0</v>
+      </c>
+      <c r="FA2">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="FB2">
         <v>17</v>
       </c>
-      <c r="ET2" t="s">
-        <v>188</v>
-      </c>
-      <c r="EU2">
-        <v>8.5</v>
-      </c>
-      <c r="EV2">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="EW2">
-        <v>5.7</v>
-      </c>
-      <c r="EX2">
-        <v>1.1645</v>
-      </c>
-      <c r="EY2">
-        <v>1474</v>
-      </c>
-      <c r="EZ2">
-        <v>84.2</v>
-      </c>
-      <c r="FA2">
-        <v>1.082</v>
-      </c>
-      <c r="FB2">
-        <v>81.59999999999999</v>
-      </c>
-      <c r="FC2">
-        <v>84</v>
+      <c r="FC2" t="s">
+        <v>198</v>
       </c>
       <c r="FD2">
-        <v>80.2</v>
+        <v>7.1</v>
       </c>
       <c r="FE2">
-        <v>88.5</v>
+        <v>2.7</v>
       </c>
       <c r="FF2">
-        <v>12.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="FG2">
+        <v>1.1641</v>
+      </c>
+      <c r="FH2">
+        <v>1476</v>
+      </c>
+      <c r="FI2">
+        <v>79.3</v>
+      </c>
+      <c r="FJ2">
+        <v>1.07</v>
+      </c>
+      <c r="FK2">
+        <v>80.90000000000001</v>
+      </c>
+      <c r="FL2">
+        <v>76</v>
+      </c>
+      <c r="FM2">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="FN2">
+        <v>88.59999999999999</v>
+      </c>
+      <c r="FO2">
+        <v>12</v>
+      </c>
+      <c r="FP2">
         <v>6</v>
       </c>
-      <c r="FH2" t="s">
-        <v>180</v>
-      </c>
-      <c r="FI2" t="s">
-        <v>189</v>
-      </c>
-      <c r="FJ2">
+      <c r="FQ2" t="s">
+        <v>190</v>
+      </c>
+      <c r="FR2" t="s">
+        <v>199</v>
+      </c>
+      <c r="FS2">
         <v>0</v>
       </c>
-      <c r="FK2">
+      <c r="FT2">
         <v>100</v>
+      </c>
+      <c r="FU2">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:FK2"/>
+  <autoFilter ref="A1:FU2"/>
   <conditionalFormatting sqref="C2">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>OR(ISNUMBER(SEARCH("Elite",$I2)),ISNUMBER(SEARCH("Excellent",$I2)),ISNUMBER(SEARCH("Very Good",$I2)),ISNUMBER(SEARCH("Good",$I2)))</formula>
@@ -2449,7 +2562,7 @@
   <sheetPr>
     <tabColor rgb="FF5B9BD5"/>
   </sheetPr>
-  <dimension ref="A1:BU5"/>
+  <dimension ref="A1:CD5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
@@ -2496,28 +2609,32 @@
     <col min="47" max="47" width="15.7109375" customWidth="1"/>
     <col min="48" max="48" width="11.7109375" customWidth="1"/>
     <col min="49" max="49" width="19.7109375" customWidth="1"/>
-    <col min="50" max="52" width="20.7109375" customWidth="1"/>
-    <col min="53" max="53" width="15.7109375" customWidth="1"/>
-    <col min="54" max="55" width="19.7109375" customWidth="1"/>
-    <col min="56" max="56" width="21.7109375" customWidth="1"/>
-    <col min="57" max="57" width="13.7109375" customWidth="1"/>
-    <col min="58" max="58" width="15.7109375" customWidth="1"/>
-    <col min="59" max="59" width="16.7109375" customWidth="1"/>
-    <col min="60" max="60" width="18.7109375" customWidth="1"/>
-    <col min="61" max="62" width="17.7109375" customWidth="1"/>
-    <col min="63" max="63" width="11.7109375" customWidth="1"/>
-    <col min="64" max="64" width="23.7109375" customWidth="1"/>
-    <col min="65" max="65" width="24.7109375" customWidth="1"/>
-    <col min="66" max="66" width="18.7109375" customWidth="1"/>
-    <col min="67" max="67" width="12.7109375" customWidth="1"/>
-    <col min="68" max="68" width="28.7109375" customWidth="1"/>
-    <col min="69" max="69" width="22.7109375" customWidth="1"/>
-    <col min="70" max="70" width="12.7109375" customWidth="1"/>
-    <col min="71" max="72" width="14.7109375" customWidth="1"/>
-    <col min="73" max="73" width="16.7109375" customWidth="1"/>
+    <col min="50" max="52" width="24.7109375" customWidth="1"/>
+    <col min="53" max="55" width="20.7109375" customWidth="1"/>
+    <col min="56" max="56" width="15.7109375" customWidth="1"/>
+    <col min="57" max="57" width="27.7109375" customWidth="1"/>
+    <col min="58" max="58" width="28.7109375" customWidth="1"/>
+    <col min="59" max="61" width="22.7109375" customWidth="1"/>
+    <col min="62" max="64" width="19.7109375" customWidth="1"/>
+    <col min="65" max="65" width="21.7109375" customWidth="1"/>
+    <col min="66" max="66" width="13.7109375" customWidth="1"/>
+    <col min="67" max="67" width="15.7109375" customWidth="1"/>
+    <col min="68" max="68" width="16.7109375" customWidth="1"/>
+    <col min="69" max="69" width="18.7109375" customWidth="1"/>
+    <col min="70" max="71" width="17.7109375" customWidth="1"/>
+    <col min="72" max="72" width="11.7109375" customWidth="1"/>
+    <col min="73" max="73" width="23.7109375" customWidth="1"/>
+    <col min="74" max="74" width="24.7109375" customWidth="1"/>
+    <col min="75" max="75" width="18.7109375" customWidth="1"/>
+    <col min="76" max="76" width="12.7109375" customWidth="1"/>
+    <col min="77" max="77" width="28.7109375" customWidth="1"/>
+    <col min="78" max="78" width="22.7109375" customWidth="1"/>
+    <col min="79" max="79" width="12.7109375" customWidth="1"/>
+    <col min="80" max="81" width="14.7109375" customWidth="1"/>
+    <col min="82" max="82" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:73" ht="34" customHeight="1">
+    <row r="1" spans="1:82" ht="34" customHeight="1">
       <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
@@ -2531,10 +2648,10 @@
         <v>6</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>53</v>
@@ -2549,61 +2666,61 @@
         <v>33</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="L1" s="3" t="s">
         <v>34</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>196</v>
+        <v>206</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>197</v>
+        <v>207</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>198</v>
+        <v>208</v>
       </c>
       <c r="S1" s="3" t="s">
-        <v>199</v>
+        <v>209</v>
       </c>
       <c r="T1" s="3" t="s">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="U1" s="3" t="s">
-        <v>201</v>
+        <v>211</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>202</v>
+        <v>212</v>
       </c>
       <c r="W1" s="3" t="s">
-        <v>203</v>
+        <v>213</v>
       </c>
       <c r="X1" s="3" t="s">
-        <v>204</v>
+        <v>214</v>
       </c>
       <c r="Y1" s="3" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="Z1" s="3" t="s">
-        <v>206</v>
+        <v>216</v>
       </c>
       <c r="AA1" s="3" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="AB1" s="3" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
       <c r="AC1" s="3" t="s">
-        <v>209</v>
+        <v>219</v>
       </c>
       <c r="AD1" s="3" t="s">
         <v>55</v>
@@ -2615,171 +2732,198 @@
         <v>57</v>
       </c>
       <c r="AG1" s="3" t="s">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="AH1" s="3" t="s">
-        <v>211</v>
+        <v>221</v>
       </c>
       <c r="AI1" s="3" t="s">
-        <v>212</v>
+        <v>222</v>
       </c>
       <c r="AJ1" s="3" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="AK1" s="3" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="AL1" s="3" t="s">
-        <v>215</v>
+        <v>225</v>
       </c>
       <c r="AM1" s="3" t="s">
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="AN1" s="3" t="s">
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="AO1" s="3" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="AP1" s="3" t="s">
-        <v>219</v>
+        <v>229</v>
       </c>
       <c r="AQ1" s="3" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="AR1" s="3" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="AS1" s="3" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="AT1" s="3" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="AU1" s="3" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="AV1" s="3" t="s">
-        <v>225</v>
+        <v>235</v>
       </c>
       <c r="AW1" s="3" t="s">
-        <v>226</v>
+        <v>236</v>
       </c>
       <c r="AX1" s="3" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="AY1" s="3" t="s">
-        <v>228</v>
+        <v>238</v>
       </c>
       <c r="AZ1" s="3" t="s">
-        <v>229</v>
+        <v>239</v>
       </c>
       <c r="BA1" s="3" t="s">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="BB1" s="3" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
       <c r="BC1" s="3" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="BD1" s="3" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="BE1" s="3" t="s">
-        <v>234</v>
+        <v>244</v>
       </c>
       <c r="BF1" s="3" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="BG1" s="3" t="s">
-        <v>236</v>
+        <v>68</v>
       </c>
       <c r="BH1" s="3" t="s">
-        <v>237</v>
+        <v>69</v>
       </c>
       <c r="BI1" s="3" t="s">
-        <v>238</v>
+        <v>70</v>
       </c>
       <c r="BJ1" s="3" t="s">
-        <v>239</v>
+        <v>71</v>
       </c>
       <c r="BK1" s="3" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="BL1" s="3" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="BM1" s="3" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="BN1" s="3" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="BO1" s="3" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="BP1" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="BQ1" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="BR1" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="BS1" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="BT1" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="BU1" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="BV1" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="BW1" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="BX1" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="BY1" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="BQ1" s="3" t="s">
+      <c r="BZ1" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="BR1" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="BS1" s="3" t="s">
-        <v>246</v>
-      </c>
-      <c r="BT1" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="BU1" s="3" t="s">
-        <v>248</v>
+      <c r="CA1" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="CB1" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="CC1" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="CD1" s="3" t="s">
+        <v>263</v>
       </c>
     </row>
-    <row r="2" spans="1:73">
+    <row r="2" spans="1:82">
       <c r="A2" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="B2" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="C2" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="D2" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="E2" t="s">
-        <v>249</v>
+        <v>264</v>
       </c>
       <c r="F2" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="G2" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="H2" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="I2" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
       <c r="J2">
-        <v>81.40000000000001</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="K2">
-        <v>4</v>
+        <v>3.7</v>
       </c>
       <c r="L2">
         <v>5</v>
       </c>
       <c r="M2">
-        <v>0.97</v>
+        <v>0.99</v>
       </c>
       <c r="N2">
-        <v>0.67</v>
+        <v>0.65</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -2788,7 +2932,7 @@
         <v>2.2</v>
       </c>
       <c r="Q2">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="R2">
         <v>100</v>
@@ -2797,25 +2941,25 @@
         <v>0</v>
       </c>
       <c r="T2" t="s">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="U2" t="s">
-        <v>257</v>
+        <v>272</v>
       </c>
       <c r="V2" t="s">
-        <v>258</v>
+        <v>273</v>
       </c>
       <c r="W2">
         <v>1</v>
       </c>
       <c r="X2">
-        <v>0.5169</v>
+        <v>0.5362</v>
       </c>
       <c r="Y2">
-        <v>-0</v>
+        <v>0.15</v>
       </c>
       <c r="Z2">
-        <v>-0.03</v>
+        <v>0.1</v>
       </c>
       <c r="AA2">
         <v>5.9</v>
@@ -2824,7 +2968,7 @@
         <v>91.3</v>
       </c>
       <c r="AC2">
-        <v>86.7</v>
+        <v>82</v>
       </c>
       <c r="AD2">
         <v>0.98</v>
@@ -2839,25 +2983,25 @@
         <v>1.6</v>
       </c>
       <c r="AH2" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
       <c r="AI2">
         <v>89.40000000000001</v>
       </c>
       <c r="AJ2">
-        <v>91</v>
+        <v>91.3</v>
       </c>
       <c r="AK2">
-        <v>68.5</v>
+        <v>68.7</v>
       </c>
       <c r="AL2">
-        <v>51.8</v>
+        <v>52.1</v>
       </c>
       <c r="AM2">
-        <v>1012.2</v>
+        <v>1012.6</v>
       </c>
       <c r="AN2">
-        <v>1014.5</v>
+        <v>1014.8</v>
       </c>
       <c r="AO2">
         <v>0</v>
@@ -2872,7 +3016,7 @@
         <v>71.40000000000001</v>
       </c>
       <c r="AS2">
-        <v>1120</v>
+        <v>1086</v>
       </c>
       <c r="AT2">
         <v>9</v>
@@ -2881,126 +3025,153 @@
         <v>19.4</v>
       </c>
       <c r="AV2" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="AW2">
         <v>225</v>
       </c>
       <c r="AX2">
-        <v>8.699999999999999</v>
+        <v>7.4</v>
       </c>
       <c r="AY2">
-        <v>8.5</v>
+        <v>3.1</v>
       </c>
       <c r="AZ2">
-        <v>5.8</v>
+        <v>9</v>
       </c>
       <c r="BA2">
-        <v>-2.3</v>
+        <v>7.2</v>
       </c>
       <c r="BB2">
-        <v>1.1457</v>
-      </c>
-      <c r="BC2" t="s">
-        <v>262</v>
+        <v>2.8</v>
+      </c>
+      <c r="BC2">
+        <v>8.4</v>
       </c>
       <c r="BD2">
-        <v>2042</v>
-      </c>
-      <c r="BE2" t="s">
-        <v>181</v>
-      </c>
-      <c r="BF2" t="s">
-        <v>182</v>
+        <v>5.1</v>
+      </c>
+      <c r="BE2">
+        <v>6.5</v>
+      </c>
+      <c r="BF2">
+        <v>0.8</v>
       </c>
       <c r="BG2">
-        <v>90.2</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="BH2">
-        <v>1.096</v>
+        <v>1.03</v>
       </c>
       <c r="BI2">
-        <v>87.59999999999999</v>
+        <v>0.98</v>
       </c>
       <c r="BJ2">
-        <v>90</v>
+        <v>0.09</v>
       </c>
       <c r="BK2">
-        <v>60.3</v>
-      </c>
-      <c r="BL2">
-        <v>59.8</v>
+        <v>1.146</v>
+      </c>
+      <c r="BL2" t="s">
+        <v>277</v>
       </c>
       <c r="BM2">
-        <v>46.9</v>
-      </c>
-      <c r="BN2">
-        <v>11.2</v>
+        <v>2032</v>
+      </c>
+      <c r="BN2" t="s">
+        <v>191</v>
       </c>
       <c r="BO2" t="s">
+        <v>192</v>
+      </c>
+      <c r="BP2">
+        <v>85.09999999999999</v>
+      </c>
+      <c r="BQ2">
+        <v>1.084</v>
+      </c>
+      <c r="BR2">
+        <v>86.8</v>
+      </c>
+      <c r="BS2">
+        <v>81.7</v>
+      </c>
+      <c r="BT2">
+        <v>60.5</v>
+      </c>
+      <c r="BU2">
+        <v>58.7</v>
+      </c>
+      <c r="BV2">
+        <v>46.7</v>
+      </c>
+      <c r="BW2">
+        <v>10.9</v>
+      </c>
+      <c r="BX2" t="s">
+        <v>190</v>
+      </c>
+      <c r="BY2">
+        <v>11</v>
+      </c>
+      <c r="BZ2" t="s">
+        <v>190</v>
+      </c>
+      <c r="CA2">
+        <v>91</v>
+      </c>
+      <c r="CB2">
+        <v>87.09999999999999</v>
+      </c>
+      <c r="CC2">
+        <v>10</v>
+      </c>
+      <c r="CD2">
+        <v>8.6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:82">
+      <c r="A3" t="s">
+        <v>178</v>
+      </c>
+      <c r="B3" t="s">
+        <v>179</v>
+      </c>
+      <c r="C3" t="s">
         <v>180</v>
       </c>
-      <c r="BP2">
-        <v>11.1</v>
-      </c>
-      <c r="BQ2" t="s">
-        <v>180</v>
-      </c>
-      <c r="BR2">
-        <v>91</v>
-      </c>
-      <c r="BS2">
-        <v>87.09999999999999</v>
-      </c>
-      <c r="BT2">
-        <v>10</v>
-      </c>
-      <c r="BU2">
-        <v>8.6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:73">
-      <c r="A3" t="s">
-        <v>168</v>
-      </c>
-      <c r="B3" t="s">
-        <v>169</v>
-      </c>
-      <c r="C3" t="s">
-        <v>170</v>
-      </c>
       <c r="D3" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="E3" t="s">
-        <v>250</v>
+        <v>265</v>
       </c>
       <c r="F3" t="s">
-        <v>253</v>
+        <v>268</v>
       </c>
       <c r="G3" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="H3" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="I3" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
       <c r="J3">
-        <v>81.40000000000001</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="K3">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="L3">
         <v>5</v>
       </c>
       <c r="M3">
-        <v>0.61</v>
+        <v>0.59</v>
       </c>
       <c r="N3">
-        <v>1.12</v>
+        <v>1.11</v>
       </c>
       <c r="O3">
         <v>0</v>
@@ -3009,7 +3180,7 @@
         <v>4.2</v>
       </c>
       <c r="Q3">
-        <v>1.2</v>
+        <v>0.5</v>
       </c>
       <c r="R3">
         <v>100</v>
@@ -3018,34 +3189,34 @@
         <v>0</v>
       </c>
       <c r="T3" t="s">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="U3" t="s">
-        <v>258</v>
+        <v>273</v>
       </c>
       <c r="V3" t="s">
-        <v>259</v>
+        <v>274</v>
       </c>
       <c r="W3">
         <v>1</v>
       </c>
       <c r="X3">
-        <v>0.4376</v>
+        <v>0.4539</v>
       </c>
       <c r="Y3">
-        <v>-0</v>
+        <v>0.12</v>
       </c>
       <c r="Z3">
-        <v>-0.02</v>
+        <v>0.08</v>
       </c>
       <c r="AA3">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="AB3">
-        <v>91.40000000000001</v>
+        <v>91.5</v>
       </c>
       <c r="AC3">
-        <v>84</v>
+        <v>79.5</v>
       </c>
       <c r="AD3">
         <v>0.98</v>
@@ -3060,25 +3231,25 @@
         <v>1.6</v>
       </c>
       <c r="AH3" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
       <c r="AI3">
         <v>85.7</v>
       </c>
       <c r="AJ3">
-        <v>85.5</v>
+        <v>86.7</v>
       </c>
       <c r="AK3">
-        <v>67.3</v>
+        <v>68.3</v>
       </c>
       <c r="AL3">
-        <v>56.1</v>
+        <v>57.7</v>
       </c>
       <c r="AM3">
-        <v>1012.1</v>
+        <v>1012.3</v>
       </c>
       <c r="AN3">
-        <v>1014.4</v>
+        <v>1014.6</v>
       </c>
       <c r="AO3">
         <v>0</v>
@@ -3093,7 +3264,7 @@
         <v>60.8</v>
       </c>
       <c r="AS3">
-        <v>825</v>
+        <v>859</v>
       </c>
       <c r="AT3">
         <v>8.800000000000001</v>
@@ -3102,126 +3273,153 @@
         <v>17.7</v>
       </c>
       <c r="AV3" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="AW3">
         <v>225</v>
       </c>
       <c r="AX3">
-        <v>8.5</v>
+        <v>7.2</v>
       </c>
       <c r="AY3">
-        <v>8.300000000000001</v>
+        <v>3</v>
       </c>
       <c r="AZ3">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="BA3">
+        <v>7.1</v>
+      </c>
+      <c r="BB3">
+        <v>2.7</v>
+      </c>
+      <c r="BC3">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="BD3">
+        <v>4.9</v>
+      </c>
+      <c r="BE3">
+        <v>6.4</v>
+      </c>
+      <c r="BF3">
+        <v>0.8</v>
+      </c>
+      <c r="BG3">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="BH3">
+        <v>1.03</v>
+      </c>
+      <c r="BI3">
+        <v>0.98</v>
+      </c>
+      <c r="BJ3">
+        <v>0.09</v>
+      </c>
+      <c r="BK3">
+        <v>1.1537</v>
+      </c>
+      <c r="BL3" t="s">
+        <v>277</v>
+      </c>
+      <c r="BM3">
+        <v>1794</v>
+      </c>
+      <c r="BN3" t="s">
+        <v>191</v>
+      </c>
+      <c r="BO3" t="s">
+        <v>192</v>
+      </c>
+      <c r="BP3">
+        <v>82.2</v>
+      </c>
+      <c r="BQ3">
+        <v>1.077</v>
+      </c>
+      <c r="BR3">
+        <v>83.90000000000001</v>
+      </c>
+      <c r="BS3">
+        <v>79</v>
+      </c>
+      <c r="BT3">
+        <v>59.6</v>
+      </c>
+      <c r="BU3">
+        <v>57.8</v>
+      </c>
+      <c r="BV3">
+        <v>52.7</v>
+      </c>
+      <c r="BW3">
+        <v>8.6</v>
+      </c>
+      <c r="BX3" t="s">
+        <v>190</v>
+      </c>
+      <c r="BY3">
+        <v>10.9</v>
+      </c>
+      <c r="BZ3" t="s">
+        <v>190</v>
+      </c>
+      <c r="CA3">
+        <v>87</v>
+      </c>
+      <c r="CB3">
+        <v>83.5</v>
+      </c>
+      <c r="CC3">
+        <v>10</v>
+      </c>
+      <c r="CD3">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:82">
+      <c r="A4" t="s">
+        <v>178</v>
+      </c>
+      <c r="B4" t="s">
+        <v>179</v>
+      </c>
+      <c r="C4" t="s">
+        <v>180</v>
+      </c>
+      <c r="D4" t="s">
+        <v>183</v>
+      </c>
+      <c r="E4" t="s">
+        <v>266</v>
+      </c>
+      <c r="F4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G4" t="s">
+        <v>196</v>
+      </c>
+      <c r="H4" t="s">
+        <v>189</v>
+      </c>
+      <c r="I4" t="s">
+        <v>197</v>
+      </c>
+      <c r="J4">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="K4">
         <v>5.7</v>
-      </c>
-      <c r="BA3">
-        <v>-2.3</v>
-      </c>
-      <c r="BB3">
-        <v>1.1538</v>
-      </c>
-      <c r="BC3" t="s">
-        <v>262</v>
-      </c>
-      <c r="BD3">
-        <v>1801</v>
-      </c>
-      <c r="BE3" t="s">
-        <v>181</v>
-      </c>
-      <c r="BF3" t="s">
-        <v>182</v>
-      </c>
-      <c r="BG3">
-        <v>87.2</v>
-      </c>
-      <c r="BH3">
-        <v>1.089</v>
-      </c>
-      <c r="BI3">
-        <v>84.59999999999999</v>
-      </c>
-      <c r="BJ3">
-        <v>87</v>
-      </c>
-      <c r="BK3">
-        <v>59.4</v>
-      </c>
-      <c r="BL3">
-        <v>58.7</v>
-      </c>
-      <c r="BM3">
-        <v>53.6</v>
-      </c>
-      <c r="BN3">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="BO3" t="s">
-        <v>180</v>
-      </c>
-      <c r="BP3">
-        <v>11</v>
-      </c>
-      <c r="BQ3" t="s">
-        <v>180</v>
-      </c>
-      <c r="BR3">
-        <v>87</v>
-      </c>
-      <c r="BS3">
-        <v>83.5</v>
-      </c>
-      <c r="BT3">
-        <v>10</v>
-      </c>
-      <c r="BU3">
-        <v>8.199999999999999</v>
-      </c>
-    </row>
-    <row r="4" spans="1:73">
-      <c r="A4" t="s">
-        <v>168</v>
-      </c>
-      <c r="B4" t="s">
-        <v>169</v>
-      </c>
-      <c r="C4" t="s">
-        <v>170</v>
-      </c>
-      <c r="D4" t="s">
-        <v>173</v>
-      </c>
-      <c r="E4" t="s">
-        <v>251</v>
-      </c>
-      <c r="F4" t="s">
-        <v>254</v>
-      </c>
-      <c r="G4" t="s">
-        <v>186</v>
-      </c>
-      <c r="H4" t="s">
-        <v>179</v>
-      </c>
-      <c r="I4" t="s">
-        <v>187</v>
-      </c>
-      <c r="J4">
-        <v>81.40000000000001</v>
-      </c>
-      <c r="K4">
-        <v>6</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>1.28</v>
+        <v>1.25</v>
       </c>
       <c r="N4">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="O4">
         <v>0</v>
@@ -3230,7 +3428,7 @@
         <v>6.1</v>
       </c>
       <c r="Q4">
-        <v>1.4</v>
+        <v>0.4</v>
       </c>
       <c r="R4">
         <v>100</v>
@@ -3239,34 +3437,34 @@
         <v>0</v>
       </c>
       <c r="T4" t="s">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="U4" t="s">
-        <v>259</v>
+        <v>274</v>
       </c>
       <c r="V4" t="s">
-        <v>260</v>
+        <v>275</v>
       </c>
       <c r="W4">
         <v>1</v>
       </c>
       <c r="X4">
-        <v>0.3704</v>
+        <v>0.3842</v>
       </c>
       <c r="Y4">
-        <v>-0</v>
+        <v>0.11</v>
       </c>
       <c r="Z4">
-        <v>-0.02</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="AA4">
-        <v>9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="AB4">
-        <v>89.40000000000001</v>
+        <v>89.5</v>
       </c>
       <c r="AC4">
-        <v>82.2</v>
+        <v>77.8</v>
       </c>
       <c r="AD4">
         <v>0.98</v>
@@ -3281,25 +3479,25 @@
         <v>1.6</v>
       </c>
       <c r="AH4" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
       <c r="AI4">
         <v>83.3</v>
       </c>
       <c r="AJ4">
-        <v>82.59999999999999</v>
+        <v>83.5</v>
       </c>
       <c r="AK4">
-        <v>67.40000000000001</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="AL4">
-        <v>60.7</v>
+        <v>62</v>
       </c>
       <c r="AM4">
-        <v>1012.2</v>
+        <v>1012.3</v>
       </c>
       <c r="AN4">
-        <v>1014.5</v>
+        <v>1014.6</v>
       </c>
       <c r="AO4">
         <v>0</v>
@@ -3314,135 +3512,162 @@
         <v>50.6</v>
       </c>
       <c r="AS4">
-        <v>779</v>
+        <v>734</v>
       </c>
       <c r="AT4">
-        <v>8.9</v>
+        <v>9</v>
       </c>
       <c r="AU4">
         <v>17.8</v>
       </c>
       <c r="AV4" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="AW4">
         <v>225</v>
       </c>
       <c r="AX4">
-        <v>8.6</v>
+        <v>7.3</v>
       </c>
       <c r="AY4">
+        <v>3.1</v>
+      </c>
+      <c r="AZ4">
+        <v>9</v>
+      </c>
+      <c r="BA4">
+        <v>7.2</v>
+      </c>
+      <c r="BB4">
+        <v>2.7</v>
+      </c>
+      <c r="BC4">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="BD4">
+        <v>5</v>
+      </c>
+      <c r="BE4">
+        <v>6.4</v>
+      </c>
+      <c r="BF4">
+        <v>0.8</v>
+      </c>
+      <c r="BG4">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="BH4">
+        <v>1.03</v>
+      </c>
+      <c r="BI4">
+        <v>0.98</v>
+      </c>
+      <c r="BJ4">
+        <v>0.09</v>
+      </c>
+      <c r="BK4">
+        <v>1.1589</v>
+      </c>
+      <c r="BL4" t="s">
+        <v>277</v>
+      </c>
+      <c r="BM4">
+        <v>1636</v>
+      </c>
+      <c r="BN4" t="s">
+        <v>191</v>
+      </c>
+      <c r="BO4" t="s">
+        <v>192</v>
+      </c>
+      <c r="BP4">
+        <v>81.09999999999999</v>
+      </c>
+      <c r="BQ4">
+        <v>1.075</v>
+      </c>
+      <c r="BR4">
+        <v>82.8</v>
+      </c>
+      <c r="BS4">
+        <v>77.7</v>
+      </c>
+      <c r="BT4">
+        <v>59.2</v>
+      </c>
+      <c r="BU4">
+        <v>57.3</v>
+      </c>
+      <c r="BV4">
+        <v>55.4</v>
+      </c>
+      <c r="BW4">
+        <v>7.3</v>
+      </c>
+      <c r="BX4" t="s">
+        <v>190</v>
+      </c>
+      <c r="BY4">
+        <v>12</v>
+      </c>
+      <c r="BZ4" t="s">
+        <v>190</v>
+      </c>
+      <c r="CA4">
+        <v>85</v>
+      </c>
+      <c r="CB4">
+        <v>80.8</v>
+      </c>
+      <c r="CC4">
+        <v>10</v>
+      </c>
+      <c r="CD4">
         <v>8.4</v>
       </c>
-      <c r="AZ4">
-        <v>5.8</v>
-      </c>
-      <c r="BA4">
-        <v>-2.3</v>
-      </c>
-      <c r="BB4">
-        <v>1.1591</v>
-      </c>
-      <c r="BC4" t="s">
-        <v>262</v>
-      </c>
-      <c r="BD4">
-        <v>1637</v>
-      </c>
-      <c r="BE4" t="s">
-        <v>181</v>
-      </c>
-      <c r="BF4" t="s">
-        <v>182</v>
-      </c>
-      <c r="BG4">
-        <v>86.09999999999999</v>
-      </c>
-      <c r="BH4">
-        <v>1.087</v>
-      </c>
-      <c r="BI4">
-        <v>83.5</v>
-      </c>
-      <c r="BJ4">
-        <v>85.90000000000001</v>
-      </c>
-      <c r="BK4">
-        <v>59.1</v>
-      </c>
-      <c r="BL4">
-        <v>58.3</v>
-      </c>
-      <c r="BM4">
-        <v>56.1</v>
-      </c>
-      <c r="BN4">
-        <v>7.8</v>
-      </c>
-      <c r="BO4" t="s">
+    </row>
+    <row r="5" spans="1:82">
+      <c r="A5" t="s">
+        <v>178</v>
+      </c>
+      <c r="B5" t="s">
+        <v>179</v>
+      </c>
+      <c r="C5" t="s">
         <v>180</v>
       </c>
-      <c r="BP4">
-        <v>12</v>
-      </c>
-      <c r="BQ4" t="s">
-        <v>180</v>
-      </c>
-      <c r="BR4">
-        <v>85</v>
-      </c>
-      <c r="BS4">
-        <v>80.8</v>
-      </c>
-      <c r="BT4">
-        <v>10</v>
-      </c>
-      <c r="BU4">
-        <v>8.4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:73">
-      <c r="A5" t="s">
-        <v>168</v>
-      </c>
-      <c r="B5" t="s">
-        <v>169</v>
-      </c>
-      <c r="C5" t="s">
-        <v>170</v>
-      </c>
       <c r="D5" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="E5" t="s">
-        <v>252</v>
+        <v>267</v>
       </c>
       <c r="F5" t="s">
-        <v>255</v>
+        <v>270</v>
       </c>
       <c r="G5" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="H5" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="I5" t="s">
-        <v>187</v>
+        <v>197</v>
       </c>
       <c r="J5">
-        <v>81.40000000000001</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="K5">
-        <v>7</v>
+        <v>6.7</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>1.98</v>
+        <v>1.96</v>
       </c>
       <c r="N5">
-        <v>1.4</v>
+        <v>1.39</v>
       </c>
       <c r="O5">
         <v>0</v>
@@ -3451,7 +3676,7 @@
         <v>7.9</v>
       </c>
       <c r="Q5">
-        <v>1.5</v>
+        <v>0.3</v>
       </c>
       <c r="R5">
         <v>100</v>
@@ -3460,34 +3685,34 @@
         <v>0</v>
       </c>
       <c r="T5" t="s">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="U5" t="s">
-        <v>260</v>
+        <v>275</v>
       </c>
       <c r="V5" t="s">
-        <v>261</v>
+        <v>276</v>
       </c>
       <c r="W5">
         <v>1</v>
       </c>
       <c r="X5">
-        <v>0.3135</v>
+        <v>0.3252</v>
       </c>
       <c r="Y5">
-        <v>-0</v>
+        <v>0.09</v>
       </c>
       <c r="Z5">
-        <v>-0.02</v>
+        <v>0.06</v>
       </c>
       <c r="AA5">
-        <v>12.1</v>
+        <v>12</v>
       </c>
       <c r="AB5">
-        <v>88.5</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="AC5">
-        <v>80.2</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="AD5">
         <v>0.98</v>
@@ -3502,25 +3727,25 @@
         <v>1.6</v>
       </c>
       <c r="AH5" t="s">
-        <v>185</v>
+        <v>195</v>
       </c>
       <c r="AI5">
-        <v>80.7</v>
+        <v>80.8</v>
       </c>
       <c r="AJ5">
-        <v>79.7</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="AK5">
-        <v>67</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="AL5">
-        <v>64.40000000000001</v>
+        <v>66.3</v>
       </c>
       <c r="AM5">
         <v>1012.1</v>
       </c>
       <c r="AN5">
-        <v>1014.4</v>
+        <v>1014.3</v>
       </c>
       <c r="AO5">
         <v>0</v>
@@ -3544,86 +3769,113 @@
         <v>17</v>
       </c>
       <c r="AV5" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="AW5">
         <v>225</v>
       </c>
       <c r="AX5">
-        <v>8.5</v>
+        <v>7.2</v>
       </c>
       <c r="AY5">
-        <v>8.300000000000001</v>
+        <v>3</v>
       </c>
       <c r="AZ5">
-        <v>5.7</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="BA5">
-        <v>-2.3</v>
+        <v>7.1</v>
       </c>
       <c r="BB5">
-        <v>1.1645</v>
-      </c>
-      <c r="BC5" t="s">
-        <v>263</v>
+        <v>2.7</v>
+      </c>
+      <c r="BC5">
+        <v>8.199999999999999</v>
       </c>
       <c r="BD5">
-        <v>1474</v>
-      </c>
-      <c r="BE5" t="s">
-        <v>181</v>
-      </c>
-      <c r="BF5" t="s">
-        <v>182</v>
+        <v>4.9</v>
+      </c>
+      <c r="BE5">
+        <v>6.4</v>
+      </c>
+      <c r="BF5">
+        <v>0.8</v>
       </c>
       <c r="BG5">
-        <v>84.2</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="BH5">
-        <v>1.082</v>
+        <v>1.03</v>
       </c>
       <c r="BI5">
-        <v>81.59999999999999</v>
+        <v>0.98</v>
       </c>
       <c r="BJ5">
-        <v>84</v>
+        <v>0.09</v>
       </c>
       <c r="BK5">
-        <v>58.5</v>
-      </c>
-      <c r="BL5">
-        <v>57.6</v>
+        <v>1.1641</v>
+      </c>
+      <c r="BL5" t="s">
+        <v>278</v>
       </c>
       <c r="BM5">
-        <v>59.8</v>
-      </c>
-      <c r="BN5">
+        <v>1476</v>
+      </c>
+      <c r="BN5" t="s">
+        <v>191</v>
+      </c>
+      <c r="BO5" t="s">
+        <v>192</v>
+      </c>
+      <c r="BP5">
+        <v>79.3</v>
+      </c>
+      <c r="BQ5">
+        <v>1.07</v>
+      </c>
+      <c r="BR5">
+        <v>80.90000000000001</v>
+      </c>
+      <c r="BS5">
+        <v>76</v>
+      </c>
+      <c r="BT5">
+        <v>58.6</v>
+      </c>
+      <c r="BU5">
+        <v>56.7</v>
+      </c>
+      <c r="BV5">
+        <v>58.9</v>
+      </c>
+      <c r="BW5">
         <v>6</v>
       </c>
-      <c r="BO5" t="s">
-        <v>180</v>
-      </c>
-      <c r="BP5">
+      <c r="BX5" t="s">
+        <v>190</v>
+      </c>
+      <c r="BY5">
         <v>10.9</v>
       </c>
-      <c r="BQ5" t="s">
-        <v>180</v>
-      </c>
-      <c r="BR5">
+      <c r="BZ5" t="s">
+        <v>190</v>
+      </c>
+      <c r="CA5">
         <v>82</v>
       </c>
-      <c r="BS5">
+      <c r="CB5">
         <v>78.59999999999999</v>
       </c>
-      <c r="BT5">
+      <c r="CC5">
         <v>10</v>
       </c>
-      <c r="BU5">
+      <c r="CD5">
         <v>8.199999999999999</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BU5"/>
+  <autoFilter ref="A1:CD5"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3633,7 +3885,7 @@
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:S2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="25.7109375" customWidth="1"/>
@@ -3644,17 +3896,18 @@
     <col min="7" max="7" width="18.7109375" customWidth="1"/>
     <col min="8" max="8" width="13.7109375" customWidth="1"/>
     <col min="9" max="9" width="18.7109375" style="4" customWidth="1"/>
-    <col min="10" max="10" width="18.7109375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="19.7109375" customWidth="1"/>
-    <col min="12" max="13" width="25.7109375" customWidth="1"/>
-    <col min="14" max="14" width="17.7109375" customWidth="1"/>
-    <col min="15" max="15" width="25.7109375" customWidth="1"/>
-    <col min="16" max="16" width="23.7109375" customWidth="1"/>
-    <col min="17" max="17" width="16.7109375" customWidth="1"/>
-    <col min="18" max="18" width="18.7109375" customWidth="1"/>
+    <col min="10" max="10" width="25.7109375" customWidth="1"/>
+    <col min="11" max="11" width="18.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="19.7109375" customWidth="1"/>
+    <col min="13" max="14" width="25.7109375" customWidth="1"/>
+    <col min="15" max="15" width="17.7109375" customWidth="1"/>
+    <col min="16" max="16" width="25.7109375" customWidth="1"/>
+    <col min="17" max="17" width="23.7109375" customWidth="1"/>
+    <col min="18" max="18" width="16.7109375" customWidth="1"/>
+    <col min="19" max="19" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="38" customHeight="1">
+    <row r="1" spans="1:19" ht="38" customHeight="1">
       <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
@@ -3683,111 +3936,117 @@
         <v>14</v>
       </c>
       <c r="J1" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="K1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:18">
+    <row r="2" spans="1:19">
       <c r="A2" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="B2" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="C2" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="D2" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="E2">
-        <v>87.90000000000001</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="F2">
-        <v>84.3</v>
+        <v>79.8</v>
       </c>
       <c r="G2" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="H2" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="I2" s="4">
-        <v>19</v>
-      </c>
-      <c r="J2" s="5">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="K2" t="s">
-        <v>174</v>
-      </c>
-      <c r="L2">
+        <v>16</v>
+      </c>
+      <c r="J2">
+        <v>5</v>
+      </c>
+      <c r="K2" s="5">
+        <v>7.2</v>
+      </c>
+      <c r="L2" t="s">
+        <v>184</v>
+      </c>
+      <c r="M2">
         <v>90.7</v>
       </c>
-      <c r="M2">
-        <v>8.6</v>
-      </c>
       <c r="N2">
+        <v>7.2</v>
+      </c>
+      <c r="O2">
         <v>86.2</v>
       </c>
-      <c r="O2">
-        <v>1832</v>
-      </c>
-      <c r="P2" t="s">
-        <v>181</v>
+      <c r="P2">
+        <v>1826</v>
       </c>
       <c r="Q2" t="s">
-        <v>180</v>
-      </c>
-      <c r="R2">
+        <v>191</v>
+      </c>
+      <c r="R2" t="s">
+        <v>190</v>
+      </c>
+      <c r="S2">
         <v>5</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R2"/>
+  <autoFilter ref="A1:S2"/>
   <conditionalFormatting sqref="A2">
     <cfRule type="expression" dxfId="0" priority="1">
-      <formula>OR(ISNUMBER(SEARCH("Elite",$K2)),ISNUMBER(SEARCH("Excellent",$K2)),ISNUMBER(SEARCH("Very Good",$K2)),ISNUMBER(SEARCH("Good",$K2)))</formula>
+      <formula>OR(ISNUMBER(SEARCH("Elite",$L2)),ISNUMBER(SEARCH("Excellent",$L2)),ISNUMBER(SEARCH("Very Good",$L2)),ISNUMBER(SEARCH("Good",$L2)))</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="2">
-      <formula>ISNUMBER(SEARCH("Neutral",$K2))</formula>
+      <formula>ISNUMBER(SEARCH("Neutral",$L2))</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="3">
-      <formula>OR(ISNUMBER(SEARCH("Below Average",$K2)),ISNUMBER(SEARCH("Poor",$K2)))</formula>
+      <formula>OR(ISNUMBER(SEARCH("Below Average",$L2)),ISNUMBER(SEARCH("Poor",$L2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2">
     <cfRule type="expression" dxfId="0" priority="4">
-      <formula>OR(ISNUMBER(SEARCH("Elite",$K2)),ISNUMBER(SEARCH("Excellent",$K2)),ISNUMBER(SEARCH("Very Good",$K2)),ISNUMBER(SEARCH("Good",$K2)))</formula>
+      <formula>OR(ISNUMBER(SEARCH("Elite",$L2)),ISNUMBER(SEARCH("Excellent",$L2)),ISNUMBER(SEARCH("Very Good",$L2)),ISNUMBER(SEARCH("Good",$L2)))</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="5">
-      <formula>ISNUMBER(SEARCH("Neutral",$K2))</formula>
+      <formula>ISNUMBER(SEARCH("Neutral",$L2))</formula>
     </cfRule>
     <cfRule type="expression" dxfId="2" priority="6">
-      <formula>OR(ISNUMBER(SEARCH("Below Average",$K2)),ISNUMBER(SEARCH("Poor",$K2)))</formula>
+      <formula>OR(ISNUMBER(SEARCH("Below Average",$L2)),ISNUMBER(SEARCH("Poor",$L2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 01:19 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_2026_07_14.xlsx
+++ b/mlb_weather_professional_2026_07_14.xlsx
@@ -551,7 +551,7 @@
     <t>Carry Percentile Value</t>
   </si>
   <si>
-    <t>Estimated FT Change by Wind</t>
+    <t>Estimated FT Change by Wind2</t>
   </si>
   <si>
     <t>2026-07-14</t>
@@ -587,10 +587,10 @@
     <t>A-</t>
   </si>
   <si>
-    <t>WORSENING RAPIDLY</t>
-  </si>
-  <si>
-    <t>2026-07-14 01:15:39 PM PDT</t>
+    <t>STEADY</t>
+  </si>
+  <si>
+    <t>2026-07-14 01:19:22 PM PDT</t>
   </si>
   <si>
     <t>LOW</t>
@@ -611,16 +611,16 @@
     <t>Clear</t>
   </si>
   <si>
+    <t>2026-07-14 20:19:22 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14T18:41:01+00:00</t>
+  </si>
+  <si>
+    <t>SW</t>
+  </si>
+  <si>
     <t>2026-07-14 20:15:39 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14T18:41:01+00:00</t>
-  </si>
-  <si>
-    <t>SW</t>
-  </si>
-  <si>
-    <t>2026-07-14 20:02:26 UTC</t>
   </si>
   <si>
     <t>Period</t>
@@ -1336,7 +1336,7 @@
     <col min="19" max="19" width="27.7109375" customWidth="1"/>
     <col min="20" max="20" width="34.7109375" customWidth="1"/>
     <col min="21" max="21" width="20.7109375" style="2" customWidth="1"/>
-    <col min="22" max="22" width="19.7109375" customWidth="1"/>
+    <col min="22" max="22" width="16.7109375" customWidth="1"/>
     <col min="23" max="23" width="34.7109375" customWidth="1"/>
     <col min="24" max="24" width="30.7109375" customWidth="1"/>
     <col min="25" max="29" width="34.7109375" customWidth="1"/>
@@ -1460,7 +1460,7 @@
     <col min="174" max="174" width="27.7109375" customWidth="1"/>
     <col min="175" max="175" width="34.7109375" customWidth="1"/>
     <col min="176" max="176" width="24.7109375" customWidth="1"/>
-    <col min="177" max="177" width="29.7109375" customWidth="1"/>
+    <col min="177" max="177" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:177" ht="34" customHeight="1">
@@ -2064,13 +2064,13 @@
         <v>188</v>
       </c>
       <c r="W2">
-        <v>-4.5</v>
+        <v>0</v>
       </c>
       <c r="X2">
         <v>0</v>
       </c>
       <c r="Y2">
-        <v>-1.4</v>
+        <v>0</v>
       </c>
       <c r="Z2">
         <v>0</v>
@@ -2091,13 +2091,13 @@
         <v>0.15</v>
       </c>
       <c r="AF2">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="AG2" t="s">
         <v>189</v>
       </c>
       <c r="AH2">
-        <v>94.59999999999999</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="AI2">
         <v>5</v>
@@ -2400,7 +2400,7 @@
         <v>9</v>
       </c>
       <c r="EE2">
-        <v>17.8</v>
+        <v>17.7</v>
       </c>
       <c r="EF2" t="s">
         <v>198</v>
@@ -2436,7 +2436,7 @@
         <v>77.8</v>
       </c>
       <c r="EQ2">
-        <v>89.5</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="ER2">
         <v>8.800000000000001</v>
@@ -2911,7 +2911,7 @@
         <v>197</v>
       </c>
       <c r="J2">
-        <v>94.59999999999999</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="K2">
         <v>3.7</v>
@@ -2923,7 +2923,7 @@
         <v>0.99</v>
       </c>
       <c r="N2">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="O2">
         <v>0</v>
@@ -2953,13 +2953,13 @@
         <v>1</v>
       </c>
       <c r="X2">
-        <v>0.5362</v>
+        <v>0.5417999999999999</v>
       </c>
       <c r="Y2">
         <v>0.15</v>
       </c>
       <c r="Z2">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="AA2">
         <v>5.9</v>
@@ -3159,7 +3159,7 @@
         <v>197</v>
       </c>
       <c r="J3">
-        <v>94.59999999999999</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="K3">
         <v>4.7</v>
@@ -3201,13 +3201,13 @@
         <v>1</v>
       </c>
       <c r="X3">
-        <v>0.4539</v>
+        <v>0.4586</v>
       </c>
       <c r="Y3">
         <v>0.12</v>
       </c>
       <c r="Z3">
-        <v>0.08</v>
+        <v>0.05</v>
       </c>
       <c r="AA3">
         <v>5.7</v>
@@ -3407,7 +3407,7 @@
         <v>197</v>
       </c>
       <c r="J4">
-        <v>94.59999999999999</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="K4">
         <v>5.7</v>
@@ -3419,7 +3419,7 @@
         <v>1.25</v>
       </c>
       <c r="N4">
-        <v>1.27</v>
+        <v>1.28</v>
       </c>
       <c r="O4">
         <v>0</v>
@@ -3449,19 +3449,19 @@
         <v>1</v>
       </c>
       <c r="X4">
-        <v>0.3842</v>
+        <v>0.3882</v>
       </c>
       <c r="Y4">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="Z4">
-        <v>0.07000000000000001</v>
+        <v>0.04</v>
       </c>
       <c r="AA4">
         <v>8.800000000000001</v>
       </c>
       <c r="AB4">
-        <v>89.5</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="AC4">
         <v>77.8</v>
@@ -3518,7 +3518,7 @@
         <v>9</v>
       </c>
       <c r="AU4">
-        <v>17.8</v>
+        <v>17.7</v>
       </c>
       <c r="AV4" t="s">
         <v>198</v>
@@ -3655,7 +3655,7 @@
         <v>197</v>
       </c>
       <c r="J5">
-        <v>94.59999999999999</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="K5">
         <v>6.7</v>
@@ -3667,7 +3667,7 @@
         <v>1.96</v>
       </c>
       <c r="N5">
-        <v>1.39</v>
+        <v>1.4</v>
       </c>
       <c r="O5">
         <v>0</v>
@@ -3697,13 +3697,13 @@
         <v>1</v>
       </c>
       <c r="X5">
-        <v>0.3252</v>
+        <v>0.3286</v>
       </c>
       <c r="Y5">
         <v>0.09</v>
       </c>
       <c r="Z5">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="AA5">
         <v>12</v>

</xml_diff>

<commit_message>
Update MLB weather 2026-07-14 02:16 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_2026_07_14.xlsx
+++ b/mlb_weather_professional_2026_07_14.xlsx
@@ -575,22 +575,22 @@
     <t>Citizens Bank Park</t>
   </si>
   <si>
-    <t>🟢 Very Good</t>
-  </si>
-  <si>
-    <t>adjusted carry 79.8; +16 ft carry; +7.2% HR env.</t>
+    <t>🔥 Excellent</t>
+  </si>
+  <si>
+    <t>adjusted carry 80.5; +17 ft carry; +7.3% HR env.</t>
   </si>
   <si>
     <t>100th</t>
   </si>
   <si>
-    <t>A-</t>
-  </si>
-  <si>
-    <t>STEADY</t>
-  </si>
-  <si>
-    <t>2026-07-14 01:19:22 PM PDT</t>
+    <t>A</t>
+  </si>
+  <si>
+    <t>IMPROVING RAPIDLY</t>
+  </si>
+  <si>
+    <t>2026-07-14 02:16:07 PM PDT</t>
   </si>
   <si>
     <t>LOW</t>
@@ -611,16 +611,16 @@
     <t>Clear</t>
   </si>
   <si>
-    <t>2026-07-14 20:19:22 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-14T18:41:01+00:00</t>
+    <t>2026-07-14 21:16:07 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-14T20:08:45+00:00</t>
   </si>
   <si>
     <t>SW</t>
   </si>
   <si>
-    <t>2026-07-14 20:15:39 UTC</t>
+    <t>2026-07-14 21:15:59 UTC</t>
   </si>
   <si>
     <t>Period</t>
@@ -1336,7 +1336,7 @@
     <col min="19" max="19" width="27.7109375" customWidth="1"/>
     <col min="20" max="20" width="34.7109375" customWidth="1"/>
     <col min="21" max="21" width="20.7109375" style="2" customWidth="1"/>
-    <col min="22" max="22" width="16.7109375" customWidth="1"/>
+    <col min="22" max="22" width="19.7109375" customWidth="1"/>
     <col min="23" max="23" width="34.7109375" customWidth="1"/>
     <col min="24" max="24" width="30.7109375" customWidth="1"/>
     <col min="25" max="29" width="34.7109375" customWidth="1"/>
@@ -2028,10 +2028,10 @@
         <v>185</v>
       </c>
       <c r="K2">
-        <v>82.90000000000001</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="L2">
-        <v>79.8</v>
+        <v>80.5</v>
       </c>
       <c r="M2" t="s">
         <v>186</v>
@@ -2040,31 +2040,31 @@
         <v>187</v>
       </c>
       <c r="O2">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P2">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="Q2" s="1">
-        <v>82.90000000000001</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="R2">
-        <v>79.8</v>
+        <v>80.5</v>
       </c>
       <c r="S2">
-        <v>90.7</v>
+        <v>91.2</v>
       </c>
       <c r="T2">
-        <v>7</v>
+        <v>6.8</v>
       </c>
       <c r="U2" s="2">
-        <v>1.072</v>
+        <v>1.073</v>
       </c>
       <c r="V2" t="s">
         <v>188</v>
       </c>
       <c r="W2">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="X2">
         <v>0</v>
@@ -2082,49 +2082,49 @@
         <v>0</v>
       </c>
       <c r="AC2">
-        <v>4.2</v>
+        <v>3.6</v>
       </c>
       <c r="AD2">
         <v>0.4</v>
       </c>
       <c r="AE2">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="AF2">
-        <v>0.06</v>
+        <v>0.21</v>
       </c>
       <c r="AG2" t="s">
         <v>189</v>
       </c>
       <c r="AH2">
-        <v>98.40000000000001</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="AI2">
         <v>5</v>
       </c>
       <c r="AJ2" s="1">
-        <v>84.5</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="AK2" s="1">
-        <v>79.5</v>
+        <v>80</v>
       </c>
       <c r="AL2">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="AM2">
-        <v>1826</v>
+        <v>1822</v>
       </c>
       <c r="AN2" t="s">
         <v>190</v>
       </c>
       <c r="AO2">
-        <v>10.9</v>
+        <v>10.5</v>
       </c>
       <c r="AP2" t="s">
         <v>190</v>
       </c>
       <c r="AQ2">
-        <v>12</v>
+        <v>11.3</v>
       </c>
       <c r="AR2" t="s">
         <v>191</v>
@@ -2172,31 +2172,31 @@
         <v>1.6</v>
       </c>
       <c r="BG2">
-        <v>86.2</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="BH2">
-        <v>68.40000000000001</v>
+        <v>68.5</v>
       </c>
       <c r="BI2">
-        <v>57.2</v>
+        <v>57.6</v>
       </c>
       <c r="BJ2">
-        <v>1012.4</v>
+        <v>1012.3</v>
       </c>
       <c r="BK2">
-        <v>8.9</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="BL2">
-        <v>19.4</v>
+        <v>20.8</v>
       </c>
       <c r="BM2">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="BN2">
-        <v>8.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="BO2">
-        <v>6.4</v>
+        <v>6.6</v>
       </c>
       <c r="BP2">
         <v>0.8</v>
@@ -2214,22 +2214,22 @@
         <v>0.09</v>
       </c>
       <c r="BU2">
-        <v>1.1527</v>
+        <v>1.1528</v>
       </c>
       <c r="BV2">
-        <v>59.8</v>
+        <v>59.9</v>
       </c>
       <c r="BW2">
-        <v>58</v>
+        <v>58.1</v>
       </c>
       <c r="BX2">
-        <v>51.5</v>
+        <v>51</v>
       </c>
       <c r="BY2">
-        <v>-8.6</v>
+        <v>-8.4</v>
       </c>
       <c r="BZ2">
-        <v>-0.5</v>
+        <v>-0.4</v>
       </c>
       <c r="CA2">
         <v>0</v>
@@ -2238,19 +2238,19 @@
         <v>0</v>
       </c>
       <c r="CC2">
-        <v>79.8</v>
+        <v>80.5</v>
       </c>
       <c r="CD2">
-        <v>89.40000000000001</v>
+        <v>89.3</v>
       </c>
       <c r="CE2">
-        <v>68.7</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="CF2">
         <v>52.1</v>
       </c>
       <c r="CG2">
-        <v>1012.6</v>
+        <v>1012.4</v>
       </c>
       <c r="CH2">
         <v>0</v>
@@ -2259,64 +2259,64 @@
         <v>0</v>
       </c>
       <c r="CJ2">
-        <v>9</v>
+        <v>9.4</v>
       </c>
       <c r="CK2">
-        <v>19.4</v>
+        <v>20.8</v>
       </c>
       <c r="CL2" t="s">
         <v>198</v>
       </c>
       <c r="CM2">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="CN2">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="CO2">
-        <v>8.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="CP2">
-        <v>1.146</v>
+        <v>1.1462</v>
       </c>
       <c r="CQ2">
-        <v>2032</v>
+        <v>2027</v>
       </c>
       <c r="CR2">
-        <v>85.09999999999999</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="CS2">
-        <v>1.084</v>
+        <v>1.086</v>
       </c>
       <c r="CT2">
-        <v>86.8</v>
+        <v>87.7</v>
       </c>
       <c r="CU2">
-        <v>81.7</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="CV2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="CW2">
-        <v>91.3</v>
+        <v>92</v>
       </c>
       <c r="CX2">
-        <v>5.9</v>
+        <v>5.5</v>
       </c>
       <c r="CY2">
-        <v>10.9</v>
+        <v>10.5</v>
       </c>
       <c r="CZ2" t="s">
         <v>190</v>
       </c>
       <c r="DA2">
-        <v>85.7</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="DB2">
-        <v>68.3</v>
+        <v>68.5</v>
       </c>
       <c r="DC2">
-        <v>57.7</v>
+        <v>58.3</v>
       </c>
       <c r="DD2">
         <v>1012.3</v>
@@ -2328,64 +2328,64 @@
         <v>0</v>
       </c>
       <c r="DG2">
-        <v>8.800000000000001</v>
+        <v>9</v>
       </c>
       <c r="DH2">
-        <v>17.7</v>
+        <v>17.6</v>
       </c>
       <c r="DI2" t="s">
         <v>198</v>
       </c>
       <c r="DJ2">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="DK2">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="DL2">
-        <v>8.199999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="DM2">
-        <v>1.1537</v>
+        <v>1.1538</v>
       </c>
       <c r="DN2">
-        <v>1794</v>
+        <v>1789</v>
       </c>
       <c r="DO2">
-        <v>82.2</v>
+        <v>82.5</v>
       </c>
       <c r="DP2">
-        <v>1.077</v>
+        <v>1.078</v>
       </c>
       <c r="DQ2">
-        <v>83.90000000000001</v>
+        <v>84.2</v>
       </c>
       <c r="DR2">
-        <v>79</v>
+        <v>79.2</v>
       </c>
       <c r="DS2">
-        <v>79.5</v>
+        <v>79.8</v>
       </c>
       <c r="DT2">
-        <v>91.5</v>
+        <v>91.7</v>
       </c>
       <c r="DU2">
-        <v>5.7</v>
+        <v>5.9</v>
       </c>
       <c r="DV2">
-        <v>8.6</v>
+        <v>9.4</v>
       </c>
       <c r="DW2" t="s">
         <v>190</v>
       </c>
       <c r="DX2">
-        <v>83.3</v>
+        <v>83.2</v>
       </c>
       <c r="DY2">
-        <v>68.09999999999999</v>
+        <v>68.5</v>
       </c>
       <c r="DZ2">
-        <v>62</v>
+        <v>62.9</v>
       </c>
       <c r="EA2">
         <v>1012.3</v>
@@ -2397,67 +2397,67 @@
         <v>0</v>
       </c>
       <c r="ED2">
-        <v>9</v>
+        <v>9.1</v>
       </c>
       <c r="EE2">
-        <v>17.7</v>
+        <v>18</v>
       </c>
       <c r="EF2" t="s">
         <v>198</v>
       </c>
       <c r="EG2">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="EH2">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="EI2">
-        <v>8.300000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="EJ2">
-        <v>1.1589</v>
+        <v>1.1588</v>
       </c>
       <c r="EK2">
-        <v>1636</v>
+        <v>1632</v>
       </c>
       <c r="EL2">
-        <v>81.09999999999999</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="EM2">
         <v>1.075</v>
       </c>
       <c r="EN2">
-        <v>82.8</v>
+        <v>83.2</v>
       </c>
       <c r="EO2">
-        <v>77.7</v>
+        <v>78</v>
       </c>
       <c r="EP2">
-        <v>77.8</v>
+        <v>78.3</v>
       </c>
       <c r="EQ2">
-        <v>89.40000000000001</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="ER2">
-        <v>8.800000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="ES2">
-        <v>7.3</v>
+        <v>8.9</v>
       </c>
       <c r="ET2" t="s">
         <v>190</v>
       </c>
       <c r="EU2">
-        <v>80.8</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="EV2">
-        <v>67.90000000000001</v>
+        <v>68.3</v>
       </c>
       <c r="EW2">
-        <v>66.3</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="EX2">
-        <v>1012.1</v>
+        <v>1012</v>
       </c>
       <c r="EY2">
         <v>0</v>
@@ -2466,52 +2466,52 @@
         <v>0</v>
       </c>
       <c r="FA2">
-        <v>8.800000000000001</v>
+        <v>8.9</v>
       </c>
       <c r="FB2">
-        <v>17</v>
+        <v>17.2</v>
       </c>
       <c r="FC2" t="s">
         <v>198</v>
       </c>
       <c r="FD2">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="FE2">
         <v>2.7</v>
       </c>
       <c r="FF2">
-        <v>8.199999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="FG2">
-        <v>1.1641</v>
+        <v>1.1637</v>
       </c>
       <c r="FH2">
-        <v>1476</v>
+        <v>1485</v>
       </c>
       <c r="FI2">
-        <v>79.3</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="FJ2">
-        <v>1.07</v>
+        <v>1.071</v>
       </c>
       <c r="FK2">
-        <v>80.90000000000001</v>
+        <v>81.3</v>
       </c>
       <c r="FL2">
-        <v>76</v>
+        <v>76.3</v>
       </c>
       <c r="FM2">
-        <v>75.90000000000001</v>
+        <v>76.5</v>
       </c>
       <c r="FN2">
-        <v>88.59999999999999</v>
+        <v>89.5</v>
       </c>
       <c r="FO2">
-        <v>12</v>
+        <v>11.1</v>
       </c>
       <c r="FP2">
-        <v>6</v>
+        <v>7.9</v>
       </c>
       <c r="FQ2" t="s">
         <v>190</v>
@@ -2911,28 +2911,28 @@
         <v>197</v>
       </c>
       <c r="J2">
-        <v>98.40000000000001</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="K2">
-        <v>3.7</v>
+        <v>2.7</v>
       </c>
       <c r="L2">
         <v>5</v>
       </c>
       <c r="M2">
-        <v>0.99</v>
+        <v>0.89</v>
       </c>
       <c r="N2">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>2.2</v>
+        <v>0.8</v>
       </c>
       <c r="Q2">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="R2">
         <v>100</v>
@@ -2953,22 +2953,22 @@
         <v>1</v>
       </c>
       <c r="X2">
-        <v>0.5417999999999999</v>
+        <v>0.6343</v>
       </c>
       <c r="Y2">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="Z2">
-        <v>0.06</v>
+        <v>0.21</v>
       </c>
       <c r="AA2">
-        <v>5.9</v>
+        <v>5.5</v>
       </c>
       <c r="AB2">
-        <v>91.3</v>
+        <v>92</v>
       </c>
       <c r="AC2">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AD2">
         <v>0.98</v>
@@ -2986,22 +2986,22 @@
         <v>195</v>
       </c>
       <c r="AI2">
-        <v>89.40000000000001</v>
+        <v>89.3</v>
       </c>
       <c r="AJ2">
-        <v>91.3</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="AK2">
-        <v>68.7</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="AL2">
         <v>52.1</v>
       </c>
       <c r="AM2">
-        <v>1012.6</v>
+        <v>1012.4</v>
       </c>
       <c r="AN2">
-        <v>1014.8</v>
+        <v>1014.7</v>
       </c>
       <c r="AO2">
         <v>0</v>
@@ -3013,16 +3013,16 @@
         <v>0</v>
       </c>
       <c r="AR2">
-        <v>71.40000000000001</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="AS2">
-        <v>1086</v>
+        <v>1052</v>
       </c>
       <c r="AT2">
-        <v>9</v>
+        <v>9.4</v>
       </c>
       <c r="AU2">
-        <v>19.4</v>
+        <v>20.8</v>
       </c>
       <c r="AV2" t="s">
         <v>198</v>
@@ -3031,28 +3031,28 @@
         <v>225</v>
       </c>
       <c r="AX2">
-        <v>7.4</v>
+        <v>7.7</v>
       </c>
       <c r="AY2">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="AZ2">
-        <v>9</v>
+        <v>9.4</v>
       </c>
       <c r="BA2">
-        <v>7.2</v>
+        <v>7.5</v>
       </c>
       <c r="BB2">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="BC2">
-        <v>8.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="BD2">
-        <v>5.1</v>
+        <v>5.3</v>
       </c>
       <c r="BE2">
-        <v>6.5</v>
+        <v>6.8</v>
       </c>
       <c r="BF2">
         <v>0.8</v>
@@ -3070,13 +3070,13 @@
         <v>0.09</v>
       </c>
       <c r="BK2">
-        <v>1.146</v>
+        <v>1.1462</v>
       </c>
       <c r="BL2" t="s">
         <v>277</v>
       </c>
       <c r="BM2">
-        <v>2032</v>
+        <v>2027</v>
       </c>
       <c r="BN2" t="s">
         <v>191</v>
@@ -3085,34 +3085,34 @@
         <v>192</v>
       </c>
       <c r="BP2">
-        <v>85.09999999999999</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="BQ2">
-        <v>1.084</v>
+        <v>1.086</v>
       </c>
       <c r="BR2">
-        <v>86.8</v>
+        <v>87.7</v>
       </c>
       <c r="BS2">
-        <v>81.7</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="BT2">
-        <v>60.5</v>
+        <v>60.7</v>
       </c>
       <c r="BU2">
-        <v>58.7</v>
+        <v>58.8</v>
       </c>
       <c r="BV2">
-        <v>46.7</v>
+        <v>46</v>
       </c>
       <c r="BW2">
-        <v>10.9</v>
+        <v>10.5</v>
       </c>
       <c r="BX2" t="s">
         <v>190</v>
       </c>
       <c r="BY2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="BZ2" t="s">
         <v>190</v>
@@ -3121,13 +3121,13 @@
         <v>91</v>
       </c>
       <c r="CB2">
-        <v>87.09999999999999</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="CC2">
         <v>10</v>
       </c>
       <c r="CD2">
-        <v>8.6</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:82">
@@ -3159,25 +3159,25 @@
         <v>197</v>
       </c>
       <c r="J3">
-        <v>98.40000000000001</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="K3">
-        <v>4.7</v>
+        <v>3.7</v>
       </c>
       <c r="L3">
         <v>5</v>
       </c>
       <c r="M3">
-        <v>0.59</v>
+        <v>0.68</v>
       </c>
       <c r="N3">
-        <v>1.11</v>
+        <v>1.06</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>4.2</v>
+        <v>3.9</v>
       </c>
       <c r="Q3">
         <v>0.5</v>
@@ -3201,22 +3201,22 @@
         <v>1</v>
       </c>
       <c r="X3">
-        <v>0.4586</v>
+        <v>0.5369</v>
       </c>
       <c r="Y3">
-        <v>0.12</v>
+        <v>0.09</v>
       </c>
       <c r="Z3">
-        <v>0.05</v>
+        <v>0.18</v>
       </c>
       <c r="AA3">
-        <v>5.7</v>
+        <v>5.9</v>
       </c>
       <c r="AB3">
-        <v>91.5</v>
+        <v>91.7</v>
       </c>
       <c r="AC3">
-        <v>79.5</v>
+        <v>79.8</v>
       </c>
       <c r="AD3">
         <v>0.98</v>
@@ -3234,16 +3234,16 @@
         <v>195</v>
       </c>
       <c r="AI3">
-        <v>85.7</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="AJ3">
-        <v>86.7</v>
+        <v>86.5</v>
       </c>
       <c r="AK3">
-        <v>68.3</v>
+        <v>68.5</v>
       </c>
       <c r="AL3">
-        <v>57.7</v>
+        <v>58.3</v>
       </c>
       <c r="AM3">
         <v>1012.3</v>
@@ -3261,16 +3261,16 @@
         <v>0</v>
       </c>
       <c r="AR3">
-        <v>60.8</v>
+        <v>58.3</v>
       </c>
       <c r="AS3">
-        <v>859</v>
+        <v>943</v>
       </c>
       <c r="AT3">
-        <v>8.800000000000001</v>
+        <v>9</v>
       </c>
       <c r="AU3">
-        <v>17.7</v>
+        <v>17.6</v>
       </c>
       <c r="AV3" t="s">
         <v>198</v>
@@ -3279,28 +3279,28 @@
         <v>225</v>
       </c>
       <c r="AX3">
+        <v>7.4</v>
+      </c>
+      <c r="AY3">
+        <v>3.1</v>
+      </c>
+      <c r="AZ3">
+        <v>9</v>
+      </c>
+      <c r="BA3">
         <v>7.2</v>
       </c>
-      <c r="AY3">
-        <v>3</v>
-      </c>
-      <c r="AZ3">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="BA3">
-        <v>7.1</v>
-      </c>
       <c r="BB3">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="BC3">
-        <v>8.199999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="BD3">
-        <v>4.9</v>
+        <v>5.1</v>
       </c>
       <c r="BE3">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="BF3">
         <v>0.8</v>
@@ -3318,13 +3318,13 @@
         <v>0.09</v>
       </c>
       <c r="BK3">
-        <v>1.1537</v>
+        <v>1.1538</v>
       </c>
       <c r="BL3" t="s">
         <v>277</v>
       </c>
       <c r="BM3">
-        <v>1794</v>
+        <v>1789</v>
       </c>
       <c r="BN3" t="s">
         <v>191</v>
@@ -3333,34 +3333,34 @@
         <v>192</v>
       </c>
       <c r="BP3">
-        <v>82.2</v>
+        <v>82.5</v>
       </c>
       <c r="BQ3">
-        <v>1.077</v>
+        <v>1.078</v>
       </c>
       <c r="BR3">
-        <v>83.90000000000001</v>
+        <v>84.2</v>
       </c>
       <c r="BS3">
-        <v>79</v>
+        <v>79.2</v>
       </c>
       <c r="BT3">
-        <v>59.6</v>
+        <v>59.7</v>
       </c>
       <c r="BU3">
-        <v>57.8</v>
+        <v>57.9</v>
       </c>
       <c r="BV3">
-        <v>52.7</v>
+        <v>52.6</v>
       </c>
       <c r="BW3">
-        <v>8.6</v>
+        <v>9.4</v>
       </c>
       <c r="BX3" t="s">
         <v>190</v>
       </c>
       <c r="BY3">
-        <v>10.9</v>
+        <v>10.3</v>
       </c>
       <c r="BZ3" t="s">
         <v>190</v>
@@ -3369,13 +3369,13 @@
         <v>87</v>
       </c>
       <c r="CB3">
-        <v>83.5</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="CC3">
         <v>10</v>
       </c>
       <c r="CD3">
-        <v>8.199999999999999</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="4" spans="1:82">
@@ -3407,25 +3407,25 @@
         <v>197</v>
       </c>
       <c r="J4">
-        <v>98.40000000000001</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="K4">
-        <v>5.7</v>
+        <v>4.7</v>
       </c>
       <c r="L4">
         <v>5</v>
       </c>
       <c r="M4">
-        <v>1.25</v>
+        <v>1.31</v>
       </c>
       <c r="N4">
-        <v>1.28</v>
+        <v>1.16</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>6.1</v>
+        <v>6.4</v>
       </c>
       <c r="Q4">
         <v>0.4</v>
@@ -3449,22 +3449,22 @@
         <v>1</v>
       </c>
       <c r="X4">
-        <v>0.3882</v>
+        <v>0.4545</v>
       </c>
       <c r="Y4">
-        <v>0.1</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Z4">
-        <v>0.04</v>
+        <v>0.15</v>
       </c>
       <c r="AA4">
-        <v>8.800000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="AB4">
-        <v>89.40000000000001</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="AC4">
-        <v>77.8</v>
+        <v>78.3</v>
       </c>
       <c r="AD4">
         <v>0.98</v>
@@ -3482,16 +3482,16 @@
         <v>195</v>
       </c>
       <c r="AI4">
-        <v>83.3</v>
+        <v>83.2</v>
       </c>
       <c r="AJ4">
-        <v>83.5</v>
+        <v>83.7</v>
       </c>
       <c r="AK4">
-        <v>68.09999999999999</v>
+        <v>68.5</v>
       </c>
       <c r="AL4">
-        <v>62</v>
+        <v>62.9</v>
       </c>
       <c r="AM4">
         <v>1012.3</v>
@@ -3509,16 +3509,16 @@
         <v>0</v>
       </c>
       <c r="AR4">
-        <v>50.6</v>
+        <v>46.9</v>
       </c>
       <c r="AS4">
-        <v>734</v>
+        <v>886</v>
       </c>
       <c r="AT4">
-        <v>9</v>
+        <v>9.1</v>
       </c>
       <c r="AU4">
-        <v>17.7</v>
+        <v>18</v>
       </c>
       <c r="AV4" t="s">
         <v>198</v>
@@ -3527,28 +3527,28 @@
         <v>225</v>
       </c>
       <c r="AX4">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="AY4">
         <v>3.1</v>
       </c>
       <c r="AZ4">
-        <v>9</v>
+        <v>9.1</v>
       </c>
       <c r="BA4">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="BB4">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="BC4">
-        <v>8.300000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="BD4">
-        <v>5</v>
+        <v>5.1</v>
       </c>
       <c r="BE4">
-        <v>6.4</v>
+        <v>6.6</v>
       </c>
       <c r="BF4">
         <v>0.8</v>
@@ -3566,13 +3566,13 @@
         <v>0.09</v>
       </c>
       <c r="BK4">
-        <v>1.1589</v>
+        <v>1.1588</v>
       </c>
       <c r="BL4" t="s">
         <v>277</v>
       </c>
       <c r="BM4">
-        <v>1636</v>
+        <v>1632</v>
       </c>
       <c r="BN4" t="s">
         <v>191</v>
@@ -3581,34 +3581,34 @@
         <v>192</v>
       </c>
       <c r="BP4">
-        <v>81.09999999999999</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="BQ4">
         <v>1.075</v>
       </c>
       <c r="BR4">
-        <v>82.8</v>
+        <v>83.2</v>
       </c>
       <c r="BS4">
-        <v>77.7</v>
+        <v>78</v>
       </c>
       <c r="BT4">
-        <v>59.2</v>
+        <v>59.3</v>
       </c>
       <c r="BU4">
-        <v>57.3</v>
+        <v>57.4</v>
       </c>
       <c r="BV4">
-        <v>55.4</v>
+        <v>54.8</v>
       </c>
       <c r="BW4">
-        <v>7.3</v>
+        <v>8.9</v>
       </c>
       <c r="BX4" t="s">
         <v>190</v>
       </c>
       <c r="BY4">
-        <v>12</v>
+        <v>11.3</v>
       </c>
       <c r="BZ4" t="s">
         <v>190</v>
@@ -3623,7 +3623,7 @@
         <v>10</v>
       </c>
       <c r="CD4">
-        <v>8.4</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:82">
@@ -3655,19 +3655,19 @@
         <v>197</v>
       </c>
       <c r="J5">
-        <v>98.40000000000001</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="K5">
-        <v>6.7</v>
+        <v>5.7</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>1.96</v>
+        <v>1.81</v>
       </c>
       <c r="N5">
-        <v>1.4</v>
+        <v>1.29</v>
       </c>
       <c r="O5">
         <v>0</v>
@@ -3697,22 +3697,22 @@
         <v>1</v>
       </c>
       <c r="X5">
-        <v>0.3286</v>
+        <v>0.3847</v>
       </c>
       <c r="Y5">
-        <v>0.09</v>
+        <v>0.06</v>
       </c>
       <c r="Z5">
-        <v>0.04</v>
+        <v>0.13</v>
       </c>
       <c r="AA5">
-        <v>12</v>
+        <v>11.1</v>
       </c>
       <c r="AB5">
-        <v>88.59999999999999</v>
+        <v>89.5</v>
       </c>
       <c r="AC5">
-        <v>75.90000000000001</v>
+        <v>76.5</v>
       </c>
       <c r="AD5">
         <v>0.98</v>
@@ -3730,19 +3730,19 @@
         <v>195</v>
       </c>
       <c r="AI5">
-        <v>80.8</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="AJ5">
-        <v>80.90000000000001</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="AK5">
-        <v>67.90000000000001</v>
+        <v>68.3</v>
       </c>
       <c r="AL5">
-        <v>66.3</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="AM5">
-        <v>1012.1</v>
+        <v>1012</v>
       </c>
       <c r="AN5">
         <v>1014.3</v>
@@ -3757,16 +3757,16 @@
         <v>0</v>
       </c>
       <c r="AR5">
-        <v>43.6</v>
+        <v>40.4</v>
       </c>
       <c r="AS5">
-        <v>602</v>
+        <v>793</v>
       </c>
       <c r="AT5">
-        <v>8.800000000000001</v>
+        <v>8.9</v>
       </c>
       <c r="AU5">
-        <v>17</v>
+        <v>17.2</v>
       </c>
       <c r="AV5" t="s">
         <v>198</v>
@@ -3775,25 +3775,25 @@
         <v>225</v>
       </c>
       <c r="AX5">
+        <v>7.3</v>
+      </c>
+      <c r="AY5">
+        <v>3.1</v>
+      </c>
+      <c r="AZ5">
+        <v>8.9</v>
+      </c>
+      <c r="BA5">
         <v>7.2</v>
-      </c>
-      <c r="AY5">
-        <v>3</v>
-      </c>
-      <c r="AZ5">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="BA5">
-        <v>7.1</v>
       </c>
       <c r="BB5">
         <v>2.7</v>
       </c>
       <c r="BC5">
-        <v>8.199999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="BD5">
-        <v>4.9</v>
+        <v>5</v>
       </c>
       <c r="BE5">
         <v>6.4</v>
@@ -3814,13 +3814,13 @@
         <v>0.09</v>
       </c>
       <c r="BK5">
-        <v>1.1641</v>
+        <v>1.1637</v>
       </c>
       <c r="BL5" t="s">
         <v>278</v>
       </c>
       <c r="BM5">
-        <v>1476</v>
+        <v>1485</v>
       </c>
       <c r="BN5" t="s">
         <v>191</v>
@@ -3829,34 +3829,34 @@
         <v>192</v>
       </c>
       <c r="BP5">
-        <v>79.3</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="BQ5">
-        <v>1.07</v>
+        <v>1.071</v>
       </c>
       <c r="BR5">
-        <v>80.90000000000001</v>
+        <v>81.3</v>
       </c>
       <c r="BS5">
-        <v>76</v>
+        <v>76.3</v>
       </c>
       <c r="BT5">
-        <v>58.6</v>
+        <v>58.7</v>
       </c>
       <c r="BU5">
-        <v>56.7</v>
+        <v>56.8</v>
       </c>
       <c r="BV5">
-        <v>58.9</v>
+        <v>58.3</v>
       </c>
       <c r="BW5">
-        <v>6</v>
+        <v>7.9</v>
       </c>
       <c r="BX5" t="s">
         <v>190</v>
       </c>
       <c r="BY5">
-        <v>10.9</v>
+        <v>10</v>
       </c>
       <c r="BZ5" t="s">
         <v>190</v>
@@ -3865,13 +3865,13 @@
         <v>82</v>
       </c>
       <c r="CB5">
-        <v>78.59999999999999</v>
+        <v>78.8</v>
       </c>
       <c r="CC5">
         <v>10</v>
       </c>
       <c r="CD5">
-        <v>8.199999999999999</v>
+        <v>8.4</v>
       </c>
     </row>
   </sheetData>
@@ -3980,10 +3980,10 @@
         <v>183</v>
       </c>
       <c r="E2">
-        <v>82.90000000000001</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="F2">
-        <v>79.8</v>
+        <v>80.5</v>
       </c>
       <c r="G2" t="s">
         <v>186</v>
@@ -3992,28 +3992,28 @@
         <v>187</v>
       </c>
       <c r="I2" s="4">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J2">
         <v>5</v>
       </c>
       <c r="K2" s="5">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="L2" t="s">
         <v>184</v>
       </c>
       <c r="M2">
-        <v>90.7</v>
+        <v>91.2</v>
       </c>
       <c r="N2">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="O2">
-        <v>86.2</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="P2">
-        <v>1826</v>
+        <v>1822</v>
       </c>
       <c r="Q2" t="s">
         <v>191</v>

</xml_diff>